<commit_message>
fix: View_8 금지 — 가공도 N 화살표 View_6 재배정 (AccessViolation 원인)
가공도 캡처 AccessViolation 격리: 템플릿 태그·잔여영역 정리 후에도
같은 지점(캡처)에서 사망. 새 제작도(최대 View_7)=정상 vs View_8
첫 도입된 가공도=사망, "메모리 손상" 예외 문구 → View_8 태그가
import 단계에서 SDK 내부 배열 범위를 넘겨 힙을 긁고 다음 네이티브
호출(캡처)에서 터지는 것으로 추정 (SDK View 번호 7까지 지원 추정,
벤더 확인 요청 후보).

- 템플릿(COM): CLIENT 예약 {View_6}(AW49, 코드 미사용) 태그 삭제,
  N 화살표 {View_8}(AT3) → {View_6}
- 코드: 북쪽 화살표 슬롯 View_8 → View_6, View_8 금지 주석
- 템플릿 규칙 확립: View 번호는 1~7만 사용
- docs: 가공도 시트.md, form1-mfg-drawing.md

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/가공도_도면_1.xlsx
+++ b/가공도_도면_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\duddl\Desktop\Project\a2z\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63D8859C-E3C6-4E7C-A1C0-616F0DF53E31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F61223F-06A7-4095-8945-B8EEA7011485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="1440" windowWidth="20256" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="696" yWindow="720" windowWidth="20256" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="237">
   <si>
     <t>A</t>
   </si>
@@ -674,9 +674,6 @@
   </si>
   <si>
     <t>{Input_1}</t>
-  </si>
-  <si>
-    <t>{View_6}</t>
   </si>
   <si>
     <t>{Input_2}</t>
@@ -720,26 +717,26 @@
     <t>{View_7}</t>
   </si>
   <si>
-    <t>{View_8}</t>
+    <t>{Input_200}</t>
+  </si>
+  <si>
+    <t>{Input_201}</t>
+  </si>
+  <si>
+    <t>{Input_202}</t>
+  </si>
+  <si>
+    <t>{Input_203}</t>
+  </si>
+  <si>
+    <t>{Input_204}</t>
+  </si>
+  <si>
+    <t>{View_5}</t>
+  </si>
+  <si>
+    <t>{View_6}</t>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{Input_200}</t>
-  </si>
-  <si>
-    <t>{Input_201}</t>
-  </si>
-  <si>
-    <t>{Input_202}</t>
-  </si>
-  <si>
-    <t>{Input_203}</t>
-  </si>
-  <si>
-    <t>{Input_204}</t>
-  </si>
-  <si>
-    <t>{View_5}</t>
   </si>
 </sst>
 </file>
@@ -967,7 +964,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -995,17 +992,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1016,7 +1011,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1031,10 +1041,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1046,20 +1056,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1524,189 +1520,189 @@
       <c r="BR2" s="2"/>
     </row>
     <row r="3" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="31" t="s">
+      <c r="C3" s="14" t="s">
+        <v>229</v>
+      </c>
+      <c r="D3" s="14"/>
+      <c r="Y3" s="3"/>
+      <c r="AT3" s="14" t="s">
+        <v>236</v>
+      </c>
+      <c r="AU3" s="14"/>
+      <c r="AV3" s="14"/>
+      <c r="AW3" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="AX3" s="22"/>
+      <c r="AY3" s="22"/>
+      <c r="AZ3" s="22"/>
+      <c r="BA3" s="22"/>
+      <c r="BB3" s="22"/>
+      <c r="BC3" s="22"/>
+      <c r="BD3" s="22"/>
+      <c r="BE3" s="22"/>
+      <c r="BF3" s="22"/>
+      <c r="BG3" s="22"/>
+      <c r="BH3" s="22"/>
+      <c r="BI3" s="22"/>
+      <c r="BJ3" s="22"/>
+      <c r="BK3" s="22"/>
+      <c r="BL3" s="22"/>
+      <c r="BM3" s="22"/>
+      <c r="BN3" s="22"/>
+      <c r="BO3" s="22"/>
+      <c r="BP3" s="22"/>
+      <c r="BQ3" s="23"/>
+      <c r="BR3" s="18" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B4" s="19"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="11"/>
+      <c r="AA4" s="11"/>
+      <c r="AT4" s="14"/>
+      <c r="AU4" s="14"/>
+      <c r="AV4" s="14"/>
+      <c r="AW4" s="24"/>
+      <c r="AX4" s="25"/>
+      <c r="AY4" s="25"/>
+      <c r="AZ4" s="25"/>
+      <c r="BA4" s="25"/>
+      <c r="BB4" s="25"/>
+      <c r="BC4" s="25"/>
+      <c r="BD4" s="25"/>
+      <c r="BE4" s="25"/>
+      <c r="BF4" s="25"/>
+      <c r="BG4" s="25"/>
+      <c r="BH4" s="25"/>
+      <c r="BI4" s="25"/>
+      <c r="BJ4" s="25"/>
+      <c r="BK4" s="25"/>
+      <c r="BL4" s="25"/>
+      <c r="BM4" s="25"/>
+      <c r="BN4" s="25"/>
+      <c r="BO4" s="25"/>
+      <c r="BP4" s="25"/>
+      <c r="BQ4" s="26"/>
+      <c r="BR4" s="19"/>
+    </row>
+    <row r="5" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="19"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="AT5" s="14"/>
+      <c r="AU5" s="14"/>
+      <c r="AV5" s="14"/>
+      <c r="AW5" s="21" t="s">
+        <v>224</v>
+      </c>
+      <c r="AX5" s="23"/>
+      <c r="AY5" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="AZ5" s="22"/>
+      <c r="BA5" s="22"/>
+      <c r="BB5" s="23"/>
+      <c r="BC5" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="BD5" s="22"/>
+      <c r="BE5" s="23"/>
+      <c r="BF5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="BG5" s="22"/>
+      <c r="BH5" s="22"/>
+      <c r="BI5" s="22"/>
+      <c r="BJ5" s="22"/>
+      <c r="BK5" s="23"/>
+      <c r="BL5" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="BM5" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="BN5" s="22"/>
+      <c r="BO5" s="23"/>
+      <c r="BP5" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="BQ5" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="BR5" s="19"/>
+    </row>
+    <row r="6" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B6" s="19"/>
+      <c r="AT6" s="14"/>
+      <c r="AU6" s="14"/>
+      <c r="AV6" s="14"/>
+      <c r="AW6" s="24"/>
+      <c r="AX6" s="26"/>
+      <c r="AY6" s="24"/>
+      <c r="AZ6" s="25"/>
+      <c r="BA6" s="25"/>
+      <c r="BB6" s="26"/>
+      <c r="BC6" s="24"/>
+      <c r="BD6" s="25"/>
+      <c r="BE6" s="26"/>
+      <c r="BF6" s="24"/>
+      <c r="BG6" s="25"/>
+      <c r="BH6" s="25"/>
+      <c r="BI6" s="25"/>
+      <c r="BJ6" s="25"/>
+      <c r="BK6" s="26"/>
+      <c r="BL6" s="20"/>
+      <c r="BM6" s="24"/>
+      <c r="BN6" s="25"/>
+      <c r="BO6" s="26"/>
+      <c r="BP6" s="20"/>
+      <c r="BQ6" s="20"/>
+      <c r="BR6" s="19"/>
+    </row>
+    <row r="7" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B7" s="19"/>
+      <c r="E7" s="12" t="s">
         <v>230</v>
       </c>
-      <c r="D3" s="31"/>
-      <c r="Y3" s="3"/>
-      <c r="AT3" s="31" t="s">
-        <v>231</v>
-      </c>
-      <c r="AU3" s="31"/>
-      <c r="AV3" s="31"/>
-      <c r="AW3" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="AX3" s="11"/>
-      <c r="AY3" s="11"/>
-      <c r="AZ3" s="11"/>
-      <c r="BA3" s="11"/>
-      <c r="BB3" s="11"/>
-      <c r="BC3" s="11"/>
-      <c r="BD3" s="11"/>
-      <c r="BE3" s="11"/>
-      <c r="BF3" s="11"/>
-      <c r="BG3" s="11"/>
-      <c r="BH3" s="11"/>
-      <c r="BI3" s="11"/>
-      <c r="BJ3" s="11"/>
-      <c r="BK3" s="11"/>
-      <c r="BL3" s="11"/>
-      <c r="BM3" s="11"/>
-      <c r="BN3" s="11"/>
-      <c r="BO3" s="11"/>
-      <c r="BP3" s="11"/>
-      <c r="BQ3" s="12"/>
-      <c r="BR3" s="23" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="28"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="32"/>
-      <c r="AA4" s="32"/>
-      <c r="AT4" s="31"/>
-      <c r="AU4" s="31"/>
-      <c r="AV4" s="31"/>
-      <c r="AW4" s="19"/>
-      <c r="AX4" s="20"/>
-      <c r="AY4" s="20"/>
-      <c r="AZ4" s="20"/>
-      <c r="BA4" s="20"/>
-      <c r="BB4" s="20"/>
-      <c r="BC4" s="20"/>
-      <c r="BD4" s="20"/>
-      <c r="BE4" s="20"/>
-      <c r="BF4" s="20"/>
-      <c r="BG4" s="20"/>
-      <c r="BH4" s="20"/>
-      <c r="BI4" s="20"/>
-      <c r="BJ4" s="20"/>
-      <c r="BK4" s="20"/>
-      <c r="BL4" s="20"/>
-      <c r="BM4" s="20"/>
-      <c r="BN4" s="20"/>
-      <c r="BO4" s="20"/>
-      <c r="BP4" s="20"/>
-      <c r="BQ4" s="21"/>
-      <c r="BR4" s="28"/>
-    </row>
-    <row r="5" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="28"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="AT5" s="31"/>
-      <c r="AU5" s="31"/>
-      <c r="AV5" s="31"/>
-      <c r="AW5" s="18" t="s">
-        <v>225</v>
-      </c>
-      <c r="AX5" s="12"/>
-      <c r="AY5" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="AZ5" s="11"/>
-      <c r="BA5" s="11"/>
-      <c r="BB5" s="12"/>
-      <c r="BC5" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="BD5" s="11"/>
-      <c r="BE5" s="12"/>
-      <c r="BF5" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="BG5" s="11"/>
-      <c r="BH5" s="11"/>
-      <c r="BI5" s="11"/>
-      <c r="BJ5" s="11"/>
-      <c r="BK5" s="12"/>
-      <c r="BL5" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="BM5" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="BN5" s="11"/>
-      <c r="BO5" s="12"/>
-      <c r="BP5" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="BQ5" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="BR5" s="28"/>
-    </row>
-    <row r="6" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="28"/>
-      <c r="AT6" s="31"/>
-      <c r="AU6" s="31"/>
-      <c r="AV6" s="31"/>
-      <c r="AW6" s="19"/>
-      <c r="AX6" s="21"/>
-      <c r="AY6" s="19"/>
-      <c r="AZ6" s="20"/>
-      <c r="BA6" s="20"/>
-      <c r="BB6" s="21"/>
-      <c r="BC6" s="19"/>
-      <c r="BD6" s="20"/>
-      <c r="BE6" s="21"/>
-      <c r="BF6" s="19"/>
-      <c r="BG6" s="20"/>
-      <c r="BH6" s="20"/>
-      <c r="BI6" s="20"/>
-      <c r="BJ6" s="20"/>
-      <c r="BK6" s="21"/>
-      <c r="BL6" s="24"/>
-      <c r="BM6" s="19"/>
-      <c r="BN6" s="20"/>
-      <c r="BO6" s="21"/>
-      <c r="BP6" s="24"/>
-      <c r="BQ6" s="24"/>
-      <c r="BR6" s="28"/>
-    </row>
-    <row r="7" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="28"/>
-      <c r="E7" s="29" t="s">
-        <v>232</v>
-      </c>
-      <c r="F7" s="30"/>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="30"/>
-      <c r="K7" s="30"/>
-      <c r="L7" s="30"/>
-      <c r="M7" s="30"/>
-      <c r="N7" s="30"/>
-      <c r="O7" s="30"/>
-      <c r="P7" s="30"/>
-      <c r="Q7" s="30"/>
-      <c r="R7" s="30"/>
-      <c r="T7" s="29" t="s">
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
+      <c r="P7" s="13"/>
+      <c r="Q7" s="13"/>
+      <c r="R7" s="13"/>
+      <c r="T7" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="U7" s="30"/>
-      <c r="V7" s="30"/>
-      <c r="W7" s="30"/>
-      <c r="X7" s="30"/>
-      <c r="Y7" s="30"/>
-      <c r="Z7" s="30"/>
-      <c r="AA7" s="30"/>
-      <c r="AB7" s="30"/>
-      <c r="AC7" s="30"/>
-      <c r="AD7" s="30"/>
-      <c r="AE7" s="30"/>
-      <c r="AF7" s="30"/>
-      <c r="AG7" s="30"/>
-      <c r="AT7" s="31"/>
-      <c r="AU7" s="31"/>
-      <c r="AV7" s="31"/>
+      <c r="U7" s="13"/>
+      <c r="V7" s="13"/>
+      <c r="W7" s="13"/>
+      <c r="X7" s="13"/>
+      <c r="Y7" s="13"/>
+      <c r="Z7" s="13"/>
+      <c r="AA7" s="13"/>
+      <c r="AB7" s="13"/>
+      <c r="AC7" s="13"/>
+      <c r="AD7" s="13"/>
+      <c r="AE7" s="13"/>
+      <c r="AF7" s="13"/>
+      <c r="AG7" s="13"/>
+      <c r="AT7" s="14"/>
+      <c r="AU7" s="14"/>
+      <c r="AV7" s="14"/>
       <c r="AW7" s="15" t="s">
         <v>11</v>
       </c>
@@ -1744,41 +1740,41 @@
       <c r="BQ7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="BR7" s="28"/>
+      <c r="BR7" s="19"/>
     </row>
     <row r="8" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B8" s="28"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30"/>
-      <c r="K8" s="30"/>
-      <c r="L8" s="30"/>
-      <c r="M8" s="30"/>
-      <c r="N8" s="30"/>
-      <c r="O8" s="30"/>
-      <c r="P8" s="30"/>
-      <c r="Q8" s="30"/>
-      <c r="R8" s="30"/>
-      <c r="T8" s="30"/>
-      <c r="U8" s="30"/>
-      <c r="V8" s="30"/>
-      <c r="W8" s="30"/>
-      <c r="X8" s="30"/>
-      <c r="Y8" s="30"/>
-      <c r="Z8" s="30"/>
-      <c r="AA8" s="30"/>
-      <c r="AB8" s="30"/>
-      <c r="AC8" s="30"/>
-      <c r="AD8" s="30"/>
-      <c r="AE8" s="30"/>
-      <c r="AF8" s="30"/>
-      <c r="AG8" s="30"/>
-      <c r="AT8" s="31"/>
-      <c r="AU8" s="31"/>
-      <c r="AV8" s="31"/>
+      <c r="B8" s="19"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13"/>
+      <c r="L8" s="13"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="13"/>
+      <c r="O8" s="13"/>
+      <c r="P8" s="13"/>
+      <c r="Q8" s="13"/>
+      <c r="R8" s="13"/>
+      <c r="T8" s="13"/>
+      <c r="U8" s="13"/>
+      <c r="V8" s="13"/>
+      <c r="W8" s="13"/>
+      <c r="X8" s="13"/>
+      <c r="Y8" s="13"/>
+      <c r="Z8" s="13"/>
+      <c r="AA8" s="13"/>
+      <c r="AB8" s="13"/>
+      <c r="AC8" s="13"/>
+      <c r="AD8" s="13"/>
+      <c r="AE8" s="13"/>
+      <c r="AF8" s="13"/>
+      <c r="AG8" s="13"/>
+      <c r="AT8" s="14"/>
+      <c r="AU8" s="14"/>
+      <c r="AV8" s="14"/>
       <c r="AW8" s="15" t="s">
         <v>19</v>
       </c>
@@ -1816,41 +1812,41 @@
       <c r="BQ8" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="BR8" s="28"/>
+      <c r="BR8" s="19"/>
     </row>
     <row r="9" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B9" s="28"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="30"/>
-      <c r="K9" s="30"/>
-      <c r="L9" s="30"/>
-      <c r="M9" s="30"/>
-      <c r="N9" s="30"/>
-      <c r="O9" s="30"/>
-      <c r="P9" s="30"/>
-      <c r="Q9" s="30"/>
-      <c r="R9" s="30"/>
-      <c r="T9" s="30"/>
-      <c r="U9" s="30"/>
-      <c r="V9" s="30"/>
-      <c r="W9" s="30"/>
-      <c r="X9" s="30"/>
-      <c r="Y9" s="30"/>
-      <c r="Z9" s="30"/>
-      <c r="AA9" s="30"/>
-      <c r="AB9" s="30"/>
-      <c r="AC9" s="30"/>
-      <c r="AD9" s="30"/>
-      <c r="AE9" s="30"/>
-      <c r="AF9" s="30"/>
-      <c r="AG9" s="30"/>
-      <c r="AT9" s="31"/>
-      <c r="AU9" s="31"/>
-      <c r="AV9" s="31"/>
+      <c r="B9" s="19"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="13"/>
+      <c r="L9" s="13"/>
+      <c r="M9" s="13"/>
+      <c r="N9" s="13"/>
+      <c r="O9" s="13"/>
+      <c r="P9" s="13"/>
+      <c r="Q9" s="13"/>
+      <c r="R9" s="13"/>
+      <c r="T9" s="13"/>
+      <c r="U9" s="13"/>
+      <c r="V9" s="13"/>
+      <c r="W9" s="13"/>
+      <c r="X9" s="13"/>
+      <c r="Y9" s="13"/>
+      <c r="Z9" s="13"/>
+      <c r="AA9" s="13"/>
+      <c r="AB9" s="13"/>
+      <c r="AC9" s="13"/>
+      <c r="AD9" s="13"/>
+      <c r="AE9" s="13"/>
+      <c r="AF9" s="13"/>
+      <c r="AG9" s="13"/>
+      <c r="AT9" s="14"/>
+      <c r="AU9" s="14"/>
+      <c r="AV9" s="14"/>
       <c r="AW9" s="15" t="s">
         <v>27</v>
       </c>
@@ -1888,41 +1884,41 @@
       <c r="BQ9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="BR9" s="28"/>
+      <c r="BR9" s="19"/>
     </row>
     <row r="10" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="28"/>
-      <c r="E10" s="30"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="30"/>
-      <c r="K10" s="30"/>
-      <c r="L10" s="30"/>
-      <c r="M10" s="30"/>
-      <c r="N10" s="30"/>
-      <c r="O10" s="30"/>
-      <c r="P10" s="30"/>
-      <c r="Q10" s="30"/>
-      <c r="R10" s="30"/>
-      <c r="T10" s="30"/>
-      <c r="U10" s="30"/>
-      <c r="V10" s="30"/>
-      <c r="W10" s="30"/>
-      <c r="X10" s="30"/>
-      <c r="Y10" s="30"/>
-      <c r="Z10" s="30"/>
-      <c r="AA10" s="30"/>
-      <c r="AB10" s="30"/>
-      <c r="AC10" s="30"/>
-      <c r="AD10" s="30"/>
-      <c r="AE10" s="30"/>
-      <c r="AF10" s="30"/>
-      <c r="AG10" s="30"/>
-      <c r="AT10" s="31"/>
-      <c r="AU10" s="31"/>
-      <c r="AV10" s="31"/>
+      <c r="B10" s="19"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="13"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="13"/>
+      <c r="R10" s="13"/>
+      <c r="T10" s="13"/>
+      <c r="U10" s="13"/>
+      <c r="V10" s="13"/>
+      <c r="W10" s="13"/>
+      <c r="X10" s="13"/>
+      <c r="Y10" s="13"/>
+      <c r="Z10" s="13"/>
+      <c r="AA10" s="13"/>
+      <c r="AB10" s="13"/>
+      <c r="AC10" s="13"/>
+      <c r="AD10" s="13"/>
+      <c r="AE10" s="13"/>
+      <c r="AF10" s="13"/>
+      <c r="AG10" s="13"/>
+      <c r="AT10" s="14"/>
+      <c r="AU10" s="14"/>
+      <c r="AV10" s="14"/>
       <c r="AW10" s="15" t="s">
         <v>35</v>
       </c>
@@ -1960,41 +1956,41 @@
       <c r="BQ10" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="BR10" s="28"/>
+      <c r="BR10" s="19"/>
     </row>
     <row r="11" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="28"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="30"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="30"/>
-      <c r="I11" s="30"/>
-      <c r="J11" s="30"/>
-      <c r="K11" s="30"/>
-      <c r="L11" s="30"/>
-      <c r="M11" s="30"/>
-      <c r="N11" s="30"/>
-      <c r="O11" s="30"/>
-      <c r="P11" s="30"/>
-      <c r="Q11" s="30"/>
-      <c r="R11" s="30"/>
-      <c r="T11" s="30"/>
-      <c r="U11" s="30"/>
-      <c r="V11" s="30"/>
-      <c r="W11" s="30"/>
-      <c r="X11" s="30"/>
-      <c r="Y11" s="30"/>
-      <c r="Z11" s="30"/>
-      <c r="AA11" s="30"/>
-      <c r="AB11" s="30"/>
-      <c r="AC11" s="30"/>
-      <c r="AD11" s="30"/>
-      <c r="AE11" s="30"/>
-      <c r="AF11" s="30"/>
-      <c r="AG11" s="30"/>
-      <c r="AT11" s="31"/>
-      <c r="AU11" s="31"/>
-      <c r="AV11" s="31"/>
+      <c r="B11" s="19"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="13"/>
+      <c r="M11" s="13"/>
+      <c r="N11" s="13"/>
+      <c r="O11" s="13"/>
+      <c r="P11" s="13"/>
+      <c r="Q11" s="13"/>
+      <c r="R11" s="13"/>
+      <c r="T11" s="13"/>
+      <c r="U11" s="13"/>
+      <c r="V11" s="13"/>
+      <c r="W11" s="13"/>
+      <c r="X11" s="13"/>
+      <c r="Y11" s="13"/>
+      <c r="Z11" s="13"/>
+      <c r="AA11" s="13"/>
+      <c r="AB11" s="13"/>
+      <c r="AC11" s="13"/>
+      <c r="AD11" s="13"/>
+      <c r="AE11" s="13"/>
+      <c r="AF11" s="13"/>
+      <c r="AG11" s="13"/>
+      <c r="AT11" s="14"/>
+      <c r="AU11" s="14"/>
+      <c r="AV11" s="14"/>
       <c r="AW11" s="15" t="s">
         <v>43</v>
       </c>
@@ -2032,10 +2028,10 @@
       <c r="BQ11" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="BR11" s="28"/>
+      <c r="BR11" s="19"/>
     </row>
     <row r="12" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="28"/>
+      <c r="B12" s="19"/>
       <c r="AW12" s="15" t="s">
         <v>51</v>
       </c>
@@ -2073,10 +2069,10 @@
       <c r="BQ12" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="BR12" s="28"/>
+      <c r="BR12" s="19"/>
     </row>
     <row r="13" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="28"/>
+      <c r="B13" s="19"/>
       <c r="AW13" s="15" t="s">
         <v>59</v>
       </c>
@@ -2114,10 +2110,10 @@
       <c r="BQ13" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="BR13" s="28"/>
+      <c r="BR13" s="19"/>
     </row>
     <row r="14" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="28"/>
+      <c r="B14" s="19"/>
       <c r="AW14" s="15" t="s">
         <v>67</v>
       </c>
@@ -2155,10 +2151,10 @@
       <c r="BQ14" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="BR14" s="28"/>
+      <c r="BR14" s="19"/>
     </row>
     <row r="15" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B15" s="28"/>
+      <c r="B15" s="19"/>
       <c r="AW15" s="15" t="s">
         <v>75</v>
       </c>
@@ -2196,10 +2192,10 @@
       <c r="BQ15" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="BR15" s="28"/>
+      <c r="BR15" s="19"/>
     </row>
     <row r="16" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="24"/>
+      <c r="B16" s="20"/>
       <c r="AW16" s="15" t="s">
         <v>84</v>
       </c>
@@ -2237,44 +2233,44 @@
       <c r="BQ16" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="BR16" s="24"/>
+      <c r="BR16" s="20"/>
     </row>
     <row r="17" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="29" t="s">
-        <v>233</v>
-      </c>
-      <c r="F17" s="30"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
-      <c r="I17" s="30"/>
-      <c r="J17" s="30"/>
-      <c r="K17" s="30"/>
-      <c r="L17" s="30"/>
-      <c r="M17" s="30"/>
-      <c r="N17" s="30"/>
-      <c r="O17" s="30"/>
-      <c r="P17" s="30"/>
-      <c r="Q17" s="30"/>
-      <c r="R17" s="30"/>
-      <c r="T17" s="29" t="s">
+      <c r="E17" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="13"/>
+      <c r="M17" s="13"/>
+      <c r="N17" s="13"/>
+      <c r="O17" s="13"/>
+      <c r="P17" s="13"/>
+      <c r="Q17" s="13"/>
+      <c r="R17" s="13"/>
+      <c r="T17" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="U17" s="30"/>
-      <c r="V17" s="30"/>
-      <c r="W17" s="30"/>
-      <c r="X17" s="30"/>
-      <c r="Y17" s="30"/>
-      <c r="Z17" s="30"/>
-      <c r="AA17" s="30"/>
-      <c r="AB17" s="30"/>
-      <c r="AC17" s="30"/>
-      <c r="AD17" s="30"/>
-      <c r="AE17" s="30"/>
-      <c r="AF17" s="30"/>
-      <c r="AG17" s="30"/>
+      <c r="U17" s="13"/>
+      <c r="V17" s="13"/>
+      <c r="W17" s="13"/>
+      <c r="X17" s="13"/>
+      <c r="Y17" s="13"/>
+      <c r="Z17" s="13"/>
+      <c r="AA17" s="13"/>
+      <c r="AB17" s="13"/>
+      <c r="AC17" s="13"/>
+      <c r="AD17" s="13"/>
+      <c r="AE17" s="13"/>
+      <c r="AF17" s="13"/>
+      <c r="AG17" s="13"/>
       <c r="AW17" s="15" t="s">
         <v>92</v>
       </c>
@@ -2312,40 +2308,40 @@
       <c r="BQ17" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="BR17" s="23" t="s">
+      <c r="BR17" s="18" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="18" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B18" s="28"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="30"/>
-      <c r="K18" s="30"/>
-      <c r="L18" s="30"/>
-      <c r="M18" s="30"/>
-      <c r="N18" s="30"/>
-      <c r="O18" s="30"/>
-      <c r="P18" s="30"/>
-      <c r="Q18" s="30"/>
-      <c r="R18" s="30"/>
-      <c r="T18" s="30"/>
-      <c r="U18" s="30"/>
-      <c r="V18" s="30"/>
-      <c r="W18" s="30"/>
-      <c r="X18" s="30"/>
-      <c r="Y18" s="30"/>
-      <c r="Z18" s="30"/>
-      <c r="AA18" s="30"/>
-      <c r="AB18" s="30"/>
-      <c r="AC18" s="30"/>
-      <c r="AD18" s="30"/>
-      <c r="AE18" s="30"/>
-      <c r="AF18" s="30"/>
-      <c r="AG18" s="30"/>
+      <c r="B18" s="19"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="13"/>
+      <c r="N18" s="13"/>
+      <c r="O18" s="13"/>
+      <c r="P18" s="13"/>
+      <c r="Q18" s="13"/>
+      <c r="R18" s="13"/>
+      <c r="T18" s="13"/>
+      <c r="U18" s="13"/>
+      <c r="V18" s="13"/>
+      <c r="W18" s="13"/>
+      <c r="X18" s="13"/>
+      <c r="Y18" s="13"/>
+      <c r="Z18" s="13"/>
+      <c r="AA18" s="13"/>
+      <c r="AB18" s="13"/>
+      <c r="AC18" s="13"/>
+      <c r="AD18" s="13"/>
+      <c r="AE18" s="13"/>
+      <c r="AF18" s="13"/>
+      <c r="AG18" s="13"/>
       <c r="AW18" s="15" t="s">
         <v>100</v>
       </c>
@@ -2383,38 +2379,38 @@
       <c r="BQ18" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="BR18" s="28"/>
+      <c r="BR18" s="19"/>
     </row>
     <row r="19" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B19" s="28"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="30"/>
-      <c r="K19" s="30"/>
-      <c r="L19" s="30"/>
-      <c r="M19" s="30"/>
-      <c r="N19" s="30"/>
-      <c r="O19" s="30"/>
-      <c r="P19" s="30"/>
-      <c r="Q19" s="30"/>
-      <c r="R19" s="30"/>
-      <c r="T19" s="30"/>
-      <c r="U19" s="30"/>
-      <c r="V19" s="30"/>
-      <c r="W19" s="30"/>
-      <c r="X19" s="30"/>
-      <c r="Y19" s="30"/>
-      <c r="Z19" s="30"/>
-      <c r="AA19" s="30"/>
-      <c r="AB19" s="30"/>
-      <c r="AC19" s="30"/>
-      <c r="AD19" s="30"/>
-      <c r="AE19" s="30"/>
-      <c r="AF19" s="30"/>
-      <c r="AG19" s="30"/>
+      <c r="B19" s="19"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="13"/>
+      <c r="M19" s="13"/>
+      <c r="N19" s="13"/>
+      <c r="O19" s="13"/>
+      <c r="P19" s="13"/>
+      <c r="Q19" s="13"/>
+      <c r="R19" s="13"/>
+      <c r="T19" s="13"/>
+      <c r="U19" s="13"/>
+      <c r="V19" s="13"/>
+      <c r="W19" s="13"/>
+      <c r="X19" s="13"/>
+      <c r="Y19" s="13"/>
+      <c r="Z19" s="13"/>
+      <c r="AA19" s="13"/>
+      <c r="AB19" s="13"/>
+      <c r="AC19" s="13"/>
+      <c r="AD19" s="13"/>
+      <c r="AE19" s="13"/>
+      <c r="AF19" s="13"/>
+      <c r="AG19" s="13"/>
       <c r="AW19" s="15" t="s">
         <v>108</v>
       </c>
@@ -2452,38 +2448,38 @@
       <c r="BQ19" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="BR19" s="28"/>
+      <c r="BR19" s="19"/>
     </row>
     <row r="20" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B20" s="28"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="30"/>
-      <c r="J20" s="30"/>
-      <c r="K20" s="30"/>
-      <c r="L20" s="30"/>
-      <c r="M20" s="30"/>
-      <c r="N20" s="30"/>
-      <c r="O20" s="30"/>
-      <c r="P20" s="30"/>
-      <c r="Q20" s="30"/>
-      <c r="R20" s="30"/>
-      <c r="T20" s="30"/>
-      <c r="U20" s="30"/>
-      <c r="V20" s="30"/>
-      <c r="W20" s="30"/>
-      <c r="X20" s="30"/>
-      <c r="Y20" s="30"/>
-      <c r="Z20" s="30"/>
-      <c r="AA20" s="30"/>
-      <c r="AB20" s="30"/>
-      <c r="AC20" s="30"/>
-      <c r="AD20" s="30"/>
-      <c r="AE20" s="30"/>
-      <c r="AF20" s="30"/>
-      <c r="AG20" s="30"/>
+      <c r="B20" s="19"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="13"/>
+      <c r="M20" s="13"/>
+      <c r="N20" s="13"/>
+      <c r="O20" s="13"/>
+      <c r="P20" s="13"/>
+      <c r="Q20" s="13"/>
+      <c r="R20" s="13"/>
+      <c r="T20" s="13"/>
+      <c r="U20" s="13"/>
+      <c r="V20" s="13"/>
+      <c r="W20" s="13"/>
+      <c r="X20" s="13"/>
+      <c r="Y20" s="13"/>
+      <c r="Z20" s="13"/>
+      <c r="AA20" s="13"/>
+      <c r="AB20" s="13"/>
+      <c r="AC20" s="13"/>
+      <c r="AD20" s="13"/>
+      <c r="AE20" s="13"/>
+      <c r="AF20" s="13"/>
+      <c r="AG20" s="13"/>
       <c r="AW20" s="15" t="s">
         <v>116</v>
       </c>
@@ -2521,10 +2517,10 @@
       <c r="BQ20" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="BR20" s="28"/>
+      <c r="BR20" s="19"/>
     </row>
     <row r="21" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B21" s="28"/>
+      <c r="B21" s="19"/>
       <c r="AW21" s="15" t="s">
         <v>124</v>
       </c>
@@ -2562,10 +2558,10 @@
       <c r="BQ21" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="BR21" s="28"/>
+      <c r="BR21" s="19"/>
     </row>
     <row r="22" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B22" s="28"/>
+      <c r="B22" s="19"/>
       <c r="AW22" s="15" t="s">
         <v>132</v>
       </c>
@@ -2603,10 +2599,10 @@
       <c r="BQ22" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="BR22" s="28"/>
+      <c r="BR22" s="19"/>
     </row>
     <row r="23" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B23" s="28"/>
+      <c r="B23" s="19"/>
       <c r="AW23" s="15" t="s">
         <v>140</v>
       </c>
@@ -2644,10 +2640,10 @@
       <c r="BQ23" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="BR23" s="28"/>
+      <c r="BR23" s="19"/>
     </row>
     <row r="24" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B24" s="28"/>
+      <c r="B24" s="19"/>
       <c r="AW24" s="15" t="s">
         <v>148</v>
       </c>
@@ -2685,27 +2681,27 @@
       <c r="BQ24" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="BR24" s="28"/>
+      <c r="BR24" s="19"/>
     </row>
     <row r="25" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B25" s="28"/>
+      <c r="B25" s="19"/>
       <c r="AW25" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="AX25" s="17"/>
+      <c r="AY25" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="AZ25" s="31"/>
+      <c r="BA25" s="31"/>
+      <c r="BB25" s="32"/>
+      <c r="BC25" s="16" t="s">
         <v>226</v>
-      </c>
-      <c r="AX25" s="17"/>
-      <c r="AY25" s="25" t="s">
-        <v>156</v>
-      </c>
-      <c r="AZ25" s="26"/>
-      <c r="BA25" s="26"/>
-      <c r="BB25" s="27"/>
-      <c r="BC25" s="16" t="s">
-        <v>227</v>
       </c>
       <c r="BD25" s="16"/>
       <c r="BE25" s="17"/>
       <c r="BF25" s="15" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="BG25" s="16"/>
       <c r="BH25" s="16"/>
@@ -2716,7 +2712,7 @@
         <v>157</v>
       </c>
       <c r="BM25" s="15" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="BN25" s="16"/>
       <c r="BO25" s="17"/>
@@ -2726,42 +2722,42 @@
       <c r="BQ25" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="BR25" s="28"/>
+      <c r="BR25" s="19"/>
     </row>
     <row r="26" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B26" s="28"/>
-      <c r="E26" s="29" t="s">
-        <v>234</v>
-      </c>
-      <c r="F26" s="30"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="30"/>
-      <c r="I26" s="30"/>
-      <c r="J26" s="30"/>
-      <c r="K26" s="30"/>
-      <c r="L26" s="30"/>
-      <c r="M26" s="30"/>
-      <c r="N26" s="30"/>
-      <c r="O26" s="30"/>
-      <c r="P26" s="30"/>
-      <c r="Q26" s="30"/>
-      <c r="R26" s="30"/>
-      <c r="T26" s="29" t="s">
+      <c r="B26" s="19"/>
+      <c r="E26" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
+      <c r="L26" s="13"/>
+      <c r="M26" s="13"/>
+      <c r="N26" s="13"/>
+      <c r="O26" s="13"/>
+      <c r="P26" s="13"/>
+      <c r="Q26" s="13"/>
+      <c r="R26" s="13"/>
+      <c r="T26" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="U26" s="30"/>
-      <c r="V26" s="30"/>
-      <c r="W26" s="30"/>
-      <c r="X26" s="30"/>
-      <c r="Y26" s="30"/>
-      <c r="Z26" s="30"/>
-      <c r="AA26" s="30"/>
-      <c r="AB26" s="30"/>
-      <c r="AC26" s="30"/>
-      <c r="AD26" s="30"/>
-      <c r="AE26" s="30"/>
-      <c r="AF26" s="30"/>
-      <c r="AG26" s="30"/>
+      <c r="U26" s="13"/>
+      <c r="V26" s="13"/>
+      <c r="W26" s="13"/>
+      <c r="X26" s="13"/>
+      <c r="Y26" s="13"/>
+      <c r="Z26" s="13"/>
+      <c r="AA26" s="13"/>
+      <c r="AB26" s="13"/>
+      <c r="AC26" s="13"/>
+      <c r="AD26" s="13"/>
+      <c r="AE26" s="13"/>
+      <c r="AF26" s="13"/>
+      <c r="AG26" s="13"/>
       <c r="AW26" s="15" t="s">
         <v>160</v>
       </c>
@@ -2799,76 +2795,72 @@
       <c r="BQ26" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="BR26" s="28"/>
+      <c r="BR26" s="19"/>
     </row>
     <row r="27" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B27" s="28"/>
-      <c r="E27" s="30"/>
-      <c r="F27" s="30"/>
-      <c r="G27" s="30"/>
-      <c r="H27" s="30"/>
-      <c r="I27" s="30"/>
-      <c r="J27" s="30"/>
-      <c r="K27" s="30"/>
-      <c r="L27" s="30"/>
-      <c r="M27" s="30"/>
-      <c r="N27" s="30"/>
-      <c r="O27" s="30"/>
-      <c r="P27" s="30"/>
-      <c r="Q27" s="30"/>
-      <c r="R27" s="30"/>
-      <c r="T27" s="30"/>
-      <c r="U27" s="30"/>
-      <c r="V27" s="30"/>
-      <c r="W27" s="30"/>
-      <c r="X27" s="30"/>
-      <c r="Y27" s="30"/>
-      <c r="Z27" s="30"/>
-      <c r="AA27" s="30"/>
-      <c r="AB27" s="30"/>
-      <c r="AC27" s="30"/>
-      <c r="AD27" s="30"/>
-      <c r="AE27" s="30"/>
-      <c r="AF27" s="30"/>
-      <c r="AG27" s="30"/>
+      <c r="B27" s="19"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
+      <c r="J27" s="13"/>
+      <c r="K27" s="13"/>
+      <c r="L27" s="13"/>
+      <c r="M27" s="13"/>
+      <c r="N27" s="13"/>
+      <c r="O27" s="13"/>
+      <c r="P27" s="13"/>
+      <c r="Q27" s="13"/>
+      <c r="R27" s="13"/>
+      <c r="T27" s="13"/>
+      <c r="U27" s="13"/>
+      <c r="V27" s="13"/>
+      <c r="W27" s="13"/>
+      <c r="X27" s="13"/>
+      <c r="Y27" s="13"/>
+      <c r="Z27" s="13"/>
+      <c r="AA27" s="13"/>
+      <c r="AB27" s="13"/>
+      <c r="AC27" s="13"/>
+      <c r="AD27" s="13"/>
+      <c r="AE27" s="13"/>
+      <c r="AF27" s="13"/>
+      <c r="AG27" s="13"/>
       <c r="BQ27" s="6"/>
-      <c r="BR27" s="28"/>
+      <c r="BR27" s="19"/>
     </row>
     <row r="28" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B28" s="28"/>
-      <c r="E28" s="30"/>
-      <c r="F28" s="30"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="30"/>
-      <c r="I28" s="30"/>
-      <c r="J28" s="30"/>
-      <c r="K28" s="30"/>
-      <c r="L28" s="30"/>
-      <c r="M28" s="30"/>
-      <c r="N28" s="30"/>
-      <c r="O28" s="30"/>
-      <c r="P28" s="30"/>
-      <c r="Q28" s="30"/>
-      <c r="R28" s="30"/>
-      <c r="T28" s="30"/>
-      <c r="U28" s="30"/>
-      <c r="V28" s="30"/>
-      <c r="W28" s="30"/>
-      <c r="X28" s="30"/>
-      <c r="Y28" s="30"/>
-      <c r="Z28" s="30"/>
-      <c r="AA28" s="30"/>
-      <c r="AB28" s="30"/>
-      <c r="AC28" s="30"/>
-      <c r="AD28" s="30"/>
-      <c r="AE28" s="30"/>
-      <c r="AF28" s="30"/>
-      <c r="AG28" s="30"/>
-      <c r="AI28" s="32"/>
-      <c r="AJ28" s="33"/>
-      <c r="AK28" s="33"/>
-      <c r="AL28" s="33"/>
-      <c r="AM28" s="33"/>
+      <c r="B28" s="19"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="13"/>
+      <c r="H28" s="13"/>
+      <c r="I28" s="13"/>
+      <c r="J28" s="13"/>
+      <c r="K28" s="13"/>
+      <c r="L28" s="13"/>
+      <c r="M28" s="13"/>
+      <c r="N28" s="13"/>
+      <c r="O28" s="13"/>
+      <c r="P28" s="13"/>
+      <c r="Q28" s="13"/>
+      <c r="R28" s="13"/>
+      <c r="T28" s="13"/>
+      <c r="U28" s="13"/>
+      <c r="V28" s="13"/>
+      <c r="W28" s="13"/>
+      <c r="X28" s="13"/>
+      <c r="Y28" s="13"/>
+      <c r="Z28" s="13"/>
+      <c r="AA28" s="13"/>
+      <c r="AB28" s="13"/>
+      <c r="AC28" s="13"/>
+      <c r="AD28" s="13"/>
+      <c r="AE28" s="13"/>
+      <c r="AF28" s="13"/>
+      <c r="AG28" s="13"/>
+      <c r="AI28" s="11"/>
       <c r="AV28" s="6"/>
       <c r="AW28" s="9"/>
       <c r="AX28" s="9"/>
@@ -2891,362 +2883,357 @@
       <c r="BO28" s="9"/>
       <c r="BP28" s="9"/>
       <c r="BQ28" s="9"/>
-      <c r="BR28" s="28"/>
+      <c r="BR28" s="19"/>
     </row>
     <row r="29" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B29" s="24"/>
-      <c r="E29" s="30"/>
-      <c r="F29" s="30"/>
-      <c r="G29" s="30"/>
-      <c r="H29" s="30"/>
-      <c r="I29" s="30"/>
-      <c r="J29" s="30"/>
-      <c r="K29" s="30"/>
-      <c r="L29" s="30"/>
-      <c r="M29" s="30"/>
-      <c r="N29" s="30"/>
-      <c r="O29" s="30"/>
-      <c r="P29" s="30"/>
-      <c r="Q29" s="30"/>
-      <c r="R29" s="30"/>
-      <c r="T29" s="30"/>
-      <c r="U29" s="30"/>
-      <c r="V29" s="30"/>
-      <c r="W29" s="30"/>
-      <c r="X29" s="30"/>
-      <c r="Y29" s="30"/>
-      <c r="Z29" s="30"/>
-      <c r="AA29" s="30"/>
-      <c r="AB29" s="30"/>
-      <c r="AC29" s="30"/>
-      <c r="AD29" s="30"/>
-      <c r="AE29" s="30"/>
-      <c r="AF29" s="30"/>
-      <c r="AG29" s="30"/>
-      <c r="AI29" s="33"/>
-      <c r="AJ29" s="33"/>
-      <c r="AK29" s="33"/>
-      <c r="AL29" s="33"/>
-      <c r="AM29" s="33"/>
+      <c r="B29" s="20"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+      <c r="H29" s="13"/>
+      <c r="I29" s="13"/>
+      <c r="J29" s="13"/>
+      <c r="K29" s="13"/>
+      <c r="L29" s="13"/>
+      <c r="M29" s="13"/>
+      <c r="N29" s="13"/>
+      <c r="O29" s="13"/>
+      <c r="P29" s="13"/>
+      <c r="Q29" s="13"/>
+      <c r="R29" s="13"/>
+      <c r="T29" s="13"/>
+      <c r="U29" s="13"/>
+      <c r="V29" s="13"/>
+      <c r="W29" s="13"/>
+      <c r="X29" s="13"/>
+      <c r="Y29" s="13"/>
+      <c r="Z29" s="13"/>
+      <c r="AA29" s="13"/>
+      <c r="AB29" s="13"/>
+      <c r="AC29" s="13"/>
+      <c r="AD29" s="13"/>
+      <c r="AE29" s="13"/>
+      <c r="AF29" s="13"/>
+      <c r="AG29" s="13"/>
       <c r="BQ29" s="6"/>
-      <c r="BR29" s="24"/>
+      <c r="BR29" s="20"/>
     </row>
     <row r="30" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B30" s="23" t="s">
+      <c r="B30" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="BR30" s="23" t="s">
+      <c r="BR30" s="18" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="31" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B31" s="28"/>
-      <c r="AW31" s="18" t="s">
+      <c r="B31" s="19"/>
+      <c r="AW31" s="21" t="s">
         <v>169</v>
       </c>
-      <c r="AX31" s="11"/>
-      <c r="AY31" s="11" t="s">
+      <c r="AX31" s="22"/>
+      <c r="AY31" s="22" t="s">
         <v>170</v>
       </c>
-      <c r="AZ31" s="11"/>
-      <c r="BA31" s="11"/>
-      <c r="BB31" s="11"/>
-      <c r="BC31" s="11"/>
-      <c r="BD31" s="11"/>
-      <c r="BE31" s="11"/>
-      <c r="BF31" s="11"/>
-      <c r="BG31" s="11"/>
-      <c r="BH31" s="11"/>
-      <c r="BI31" s="11"/>
-      <c r="BJ31" s="11"/>
-      <c r="BK31" s="11"/>
-      <c r="BL31" s="11"/>
-      <c r="BM31" s="11"/>
-      <c r="BN31" s="11"/>
-      <c r="BO31" s="11"/>
-      <c r="BP31" s="11"/>
-      <c r="BQ31" s="12"/>
-      <c r="BR31" s="28"/>
+      <c r="AZ31" s="22"/>
+      <c r="BA31" s="22"/>
+      <c r="BB31" s="22"/>
+      <c r="BC31" s="22"/>
+      <c r="BD31" s="22"/>
+      <c r="BE31" s="22"/>
+      <c r="BF31" s="22"/>
+      <c r="BG31" s="22"/>
+      <c r="BH31" s="22"/>
+      <c r="BI31" s="22"/>
+      <c r="BJ31" s="22"/>
+      <c r="BK31" s="22"/>
+      <c r="BL31" s="22"/>
+      <c r="BM31" s="22"/>
+      <c r="BN31" s="22"/>
+      <c r="BO31" s="22"/>
+      <c r="BP31" s="22"/>
+      <c r="BQ31" s="23"/>
+      <c r="BR31" s="19"/>
     </row>
     <row r="32" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B32" s="28"/>
-      <c r="AW32" s="22"/>
-      <c r="AX32" s="13"/>
-      <c r="AY32" s="13"/>
-      <c r="AZ32" s="13"/>
-      <c r="BA32" s="13"/>
-      <c r="BB32" s="13"/>
-      <c r="BC32" s="13"/>
-      <c r="BD32" s="13"/>
-      <c r="BE32" s="13"/>
-      <c r="BF32" s="13"/>
-      <c r="BG32" s="13"/>
-      <c r="BH32" s="13"/>
-      <c r="BI32" s="13"/>
-      <c r="BJ32" s="13"/>
-      <c r="BK32" s="13"/>
-      <c r="BL32" s="13"/>
-      <c r="BM32" s="13"/>
-      <c r="BN32" s="13"/>
-      <c r="BO32" s="13"/>
-      <c r="BP32" s="13"/>
-      <c r="BQ32" s="14"/>
-      <c r="BR32" s="28"/>
+      <c r="B32" s="19"/>
+      <c r="AW32" s="27"/>
+      <c r="AX32" s="28"/>
+      <c r="AY32" s="28"/>
+      <c r="AZ32" s="28"/>
+      <c r="BA32" s="28"/>
+      <c r="BB32" s="28"/>
+      <c r="BC32" s="28"/>
+      <c r="BD32" s="28"/>
+      <c r="BE32" s="28"/>
+      <c r="BF32" s="28"/>
+      <c r="BG32" s="28"/>
+      <c r="BH32" s="28"/>
+      <c r="BI32" s="28"/>
+      <c r="BJ32" s="28"/>
+      <c r="BK32" s="28"/>
+      <c r="BL32" s="28"/>
+      <c r="BM32" s="28"/>
+      <c r="BN32" s="28"/>
+      <c r="BO32" s="28"/>
+      <c r="BP32" s="28"/>
+      <c r="BQ32" s="29"/>
+      <c r="BR32" s="19"/>
     </row>
     <row r="33" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B33" s="28"/>
-      <c r="AW33" s="22"/>
-      <c r="AX33" s="13"/>
-      <c r="AY33" s="13"/>
-      <c r="AZ33" s="13"/>
-      <c r="BA33" s="13"/>
-      <c r="BB33" s="13"/>
-      <c r="BC33" s="13"/>
-      <c r="BD33" s="13"/>
-      <c r="BE33" s="13"/>
-      <c r="BF33" s="13"/>
-      <c r="BG33" s="13"/>
-      <c r="BH33" s="13"/>
-      <c r="BI33" s="13"/>
-      <c r="BJ33" s="13"/>
-      <c r="BK33" s="13"/>
-      <c r="BL33" s="13"/>
-      <c r="BM33" s="13"/>
-      <c r="BN33" s="13"/>
-      <c r="BO33" s="13"/>
-      <c r="BP33" s="13"/>
-      <c r="BQ33" s="14"/>
-      <c r="BR33" s="28"/>
+      <c r="B33" s="19"/>
+      <c r="AW33" s="27"/>
+      <c r="AX33" s="28"/>
+      <c r="AY33" s="28"/>
+      <c r="AZ33" s="28"/>
+      <c r="BA33" s="28"/>
+      <c r="BB33" s="28"/>
+      <c r="BC33" s="28"/>
+      <c r="BD33" s="28"/>
+      <c r="BE33" s="28"/>
+      <c r="BF33" s="28"/>
+      <c r="BG33" s="28"/>
+      <c r="BH33" s="28"/>
+      <c r="BI33" s="28"/>
+      <c r="BJ33" s="28"/>
+      <c r="BK33" s="28"/>
+      <c r="BL33" s="28"/>
+      <c r="BM33" s="28"/>
+      <c r="BN33" s="28"/>
+      <c r="BO33" s="28"/>
+      <c r="BP33" s="28"/>
+      <c r="BQ33" s="29"/>
+      <c r="BR33" s="19"/>
     </row>
     <row r="34" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B34" s="28"/>
-      <c r="AW34" s="22"/>
-      <c r="AX34" s="13"/>
-      <c r="AY34" s="13"/>
-      <c r="AZ34" s="13"/>
-      <c r="BA34" s="13"/>
-      <c r="BB34" s="13"/>
-      <c r="BC34" s="13"/>
-      <c r="BD34" s="13"/>
-      <c r="BE34" s="13"/>
-      <c r="BF34" s="13"/>
-      <c r="BG34" s="13"/>
-      <c r="BH34" s="13"/>
-      <c r="BI34" s="13"/>
-      <c r="BJ34" s="13"/>
-      <c r="BK34" s="13"/>
-      <c r="BL34" s="13"/>
-      <c r="BM34" s="13"/>
-      <c r="BN34" s="13"/>
-      <c r="BO34" s="13"/>
-      <c r="BP34" s="13"/>
-      <c r="BQ34" s="14"/>
-      <c r="BR34" s="28"/>
+      <c r="B34" s="19"/>
+      <c r="AW34" s="27"/>
+      <c r="AX34" s="28"/>
+      <c r="AY34" s="28"/>
+      <c r="AZ34" s="28"/>
+      <c r="BA34" s="28"/>
+      <c r="BB34" s="28"/>
+      <c r="BC34" s="28"/>
+      <c r="BD34" s="28"/>
+      <c r="BE34" s="28"/>
+      <c r="BF34" s="28"/>
+      <c r="BG34" s="28"/>
+      <c r="BH34" s="28"/>
+      <c r="BI34" s="28"/>
+      <c r="BJ34" s="28"/>
+      <c r="BK34" s="28"/>
+      <c r="BL34" s="28"/>
+      <c r="BM34" s="28"/>
+      <c r="BN34" s="28"/>
+      <c r="BO34" s="28"/>
+      <c r="BP34" s="28"/>
+      <c r="BQ34" s="29"/>
+      <c r="BR34" s="19"/>
     </row>
     <row r="35" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B35" s="28"/>
-      <c r="E35" s="29" t="s">
-        <v>235</v>
-      </c>
-      <c r="F35" s="30"/>
-      <c r="G35" s="30"/>
-      <c r="H35" s="30"/>
-      <c r="I35" s="30"/>
-      <c r="J35" s="30"/>
-      <c r="K35" s="30"/>
-      <c r="L35" s="30"/>
-      <c r="M35" s="30"/>
-      <c r="N35" s="30"/>
-      <c r="O35" s="30"/>
-      <c r="P35" s="30"/>
-      <c r="Q35" s="30"/>
-      <c r="R35" s="30"/>
-      <c r="T35" s="29" t="s">
+      <c r="B35" s="19"/>
+      <c r="E35" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="F35" s="13"/>
+      <c r="G35" s="13"/>
+      <c r="H35" s="13"/>
+      <c r="I35" s="13"/>
+      <c r="J35" s="13"/>
+      <c r="K35" s="13"/>
+      <c r="L35" s="13"/>
+      <c r="M35" s="13"/>
+      <c r="N35" s="13"/>
+      <c r="O35" s="13"/>
+      <c r="P35" s="13"/>
+      <c r="Q35" s="13"/>
+      <c r="R35" s="13"/>
+      <c r="T35" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="U35" s="30"/>
-      <c r="V35" s="30"/>
-      <c r="W35" s="30"/>
-      <c r="X35" s="30"/>
-      <c r="Y35" s="30"/>
-      <c r="Z35" s="30"/>
-      <c r="AA35" s="30"/>
-      <c r="AB35" s="30"/>
-      <c r="AC35" s="30"/>
-      <c r="AD35" s="30"/>
-      <c r="AE35" s="30"/>
-      <c r="AF35" s="30"/>
-      <c r="AG35" s="30"/>
-      <c r="AW35" s="22"/>
-      <c r="AX35" s="13"/>
-      <c r="AY35" s="13"/>
-      <c r="AZ35" s="13"/>
-      <c r="BA35" s="13"/>
-      <c r="BB35" s="13"/>
-      <c r="BC35" s="13"/>
-      <c r="BD35" s="13"/>
-      <c r="BE35" s="13"/>
-      <c r="BF35" s="13"/>
-      <c r="BG35" s="13"/>
-      <c r="BH35" s="13"/>
-      <c r="BI35" s="13"/>
-      <c r="BJ35" s="13"/>
-      <c r="BK35" s="13"/>
-      <c r="BL35" s="13"/>
-      <c r="BM35" s="13"/>
-      <c r="BN35" s="13"/>
-      <c r="BO35" s="13"/>
-      <c r="BP35" s="13"/>
-      <c r="BQ35" s="14"/>
-      <c r="BR35" s="28"/>
+      <c r="U35" s="13"/>
+      <c r="V35" s="13"/>
+      <c r="W35" s="13"/>
+      <c r="X35" s="13"/>
+      <c r="Y35" s="13"/>
+      <c r="Z35" s="13"/>
+      <c r="AA35" s="13"/>
+      <c r="AB35" s="13"/>
+      <c r="AC35" s="13"/>
+      <c r="AD35" s="13"/>
+      <c r="AE35" s="13"/>
+      <c r="AF35" s="13"/>
+      <c r="AG35" s="13"/>
+      <c r="AW35" s="27"/>
+      <c r="AX35" s="28"/>
+      <c r="AY35" s="28"/>
+      <c r="AZ35" s="28"/>
+      <c r="BA35" s="28"/>
+      <c r="BB35" s="28"/>
+      <c r="BC35" s="28"/>
+      <c r="BD35" s="28"/>
+      <c r="BE35" s="28"/>
+      <c r="BF35" s="28"/>
+      <c r="BG35" s="28"/>
+      <c r="BH35" s="28"/>
+      <c r="BI35" s="28"/>
+      <c r="BJ35" s="28"/>
+      <c r="BK35" s="28"/>
+      <c r="BL35" s="28"/>
+      <c r="BM35" s="28"/>
+      <c r="BN35" s="28"/>
+      <c r="BO35" s="28"/>
+      <c r="BP35" s="28"/>
+      <c r="BQ35" s="29"/>
+      <c r="BR35" s="19"/>
     </row>
     <row r="36" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B36" s="28"/>
-      <c r="E36" s="30"/>
-      <c r="F36" s="30"/>
-      <c r="G36" s="30"/>
-      <c r="H36" s="30"/>
-      <c r="I36" s="30"/>
-      <c r="J36" s="30"/>
-      <c r="K36" s="30"/>
-      <c r="L36" s="30"/>
-      <c r="M36" s="30"/>
-      <c r="N36" s="30"/>
-      <c r="O36" s="30"/>
-      <c r="P36" s="30"/>
-      <c r="Q36" s="30"/>
-      <c r="R36" s="30"/>
-      <c r="T36" s="30"/>
-      <c r="U36" s="30"/>
-      <c r="V36" s="30"/>
-      <c r="W36" s="30"/>
-      <c r="X36" s="30"/>
-      <c r="Y36" s="30"/>
-      <c r="Z36" s="30"/>
-      <c r="AA36" s="30"/>
-      <c r="AB36" s="30"/>
-      <c r="AC36" s="30"/>
-      <c r="AD36" s="30"/>
-      <c r="AE36" s="30"/>
-      <c r="AF36" s="30"/>
-      <c r="AG36" s="30"/>
-      <c r="AW36" s="19"/>
-      <c r="AX36" s="20"/>
-      <c r="AY36" s="20"/>
-      <c r="AZ36" s="20"/>
-      <c r="BA36" s="20"/>
-      <c r="BB36" s="20"/>
-      <c r="BC36" s="20"/>
-      <c r="BD36" s="20"/>
-      <c r="BE36" s="20"/>
-      <c r="BF36" s="20"/>
-      <c r="BG36" s="20"/>
-      <c r="BH36" s="20"/>
-      <c r="BI36" s="20"/>
-      <c r="BJ36" s="20"/>
-      <c r="BK36" s="20"/>
-      <c r="BL36" s="20"/>
-      <c r="BM36" s="20"/>
-      <c r="BN36" s="20"/>
-      <c r="BO36" s="20"/>
-      <c r="BP36" s="20"/>
-      <c r="BQ36" s="21"/>
-      <c r="BR36" s="28"/>
+      <c r="B36" s="19"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
+      <c r="G36" s="13"/>
+      <c r="H36" s="13"/>
+      <c r="I36" s="13"/>
+      <c r="J36" s="13"/>
+      <c r="K36" s="13"/>
+      <c r="L36" s="13"/>
+      <c r="M36" s="13"/>
+      <c r="N36" s="13"/>
+      <c r="O36" s="13"/>
+      <c r="P36" s="13"/>
+      <c r="Q36" s="13"/>
+      <c r="R36" s="13"/>
+      <c r="T36" s="13"/>
+      <c r="U36" s="13"/>
+      <c r="V36" s="13"/>
+      <c r="W36" s="13"/>
+      <c r="X36" s="13"/>
+      <c r="Y36" s="13"/>
+      <c r="Z36" s="13"/>
+      <c r="AA36" s="13"/>
+      <c r="AB36" s="13"/>
+      <c r="AC36" s="13"/>
+      <c r="AD36" s="13"/>
+      <c r="AE36" s="13"/>
+      <c r="AF36" s="13"/>
+      <c r="AG36" s="13"/>
+      <c r="AW36" s="24"/>
+      <c r="AX36" s="25"/>
+      <c r="AY36" s="25"/>
+      <c r="AZ36" s="25"/>
+      <c r="BA36" s="25"/>
+      <c r="BB36" s="25"/>
+      <c r="BC36" s="25"/>
+      <c r="BD36" s="25"/>
+      <c r="BE36" s="25"/>
+      <c r="BF36" s="25"/>
+      <c r="BG36" s="25"/>
+      <c r="BH36" s="25"/>
+      <c r="BI36" s="25"/>
+      <c r="BJ36" s="25"/>
+      <c r="BK36" s="25"/>
+      <c r="BL36" s="25"/>
+      <c r="BM36" s="25"/>
+      <c r="BN36" s="25"/>
+      <c r="BO36" s="25"/>
+      <c r="BP36" s="25"/>
+      <c r="BQ36" s="26"/>
+      <c r="BR36" s="19"/>
     </row>
     <row r="37" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B37" s="28"/>
-      <c r="E37" s="30"/>
-      <c r="F37" s="30"/>
-      <c r="G37" s="30"/>
-      <c r="H37" s="30"/>
-      <c r="I37" s="30"/>
-      <c r="J37" s="30"/>
-      <c r="K37" s="30"/>
-      <c r="L37" s="30"/>
-      <c r="M37" s="30"/>
-      <c r="N37" s="30"/>
-      <c r="O37" s="30"/>
-      <c r="P37" s="30"/>
-      <c r="Q37" s="30"/>
-      <c r="R37" s="30"/>
-      <c r="T37" s="30"/>
-      <c r="U37" s="30"/>
-      <c r="V37" s="30"/>
-      <c r="W37" s="30"/>
-      <c r="X37" s="30"/>
-      <c r="Y37" s="30"/>
-      <c r="Z37" s="30"/>
-      <c r="AA37" s="30"/>
-      <c r="AB37" s="30"/>
-      <c r="AC37" s="30"/>
-      <c r="AD37" s="30"/>
-      <c r="AE37" s="30"/>
-      <c r="AF37" s="30"/>
-      <c r="AG37" s="30"/>
-      <c r="BR37" s="28"/>
+      <c r="B37" s="19"/>
+      <c r="E37" s="13"/>
+      <c r="F37" s="13"/>
+      <c r="G37" s="13"/>
+      <c r="H37" s="13"/>
+      <c r="I37" s="13"/>
+      <c r="J37" s="13"/>
+      <c r="K37" s="13"/>
+      <c r="L37" s="13"/>
+      <c r="M37" s="13"/>
+      <c r="N37" s="13"/>
+      <c r="O37" s="13"/>
+      <c r="P37" s="13"/>
+      <c r="Q37" s="13"/>
+      <c r="R37" s="13"/>
+      <c r="T37" s="13"/>
+      <c r="U37" s="13"/>
+      <c r="V37" s="13"/>
+      <c r="W37" s="13"/>
+      <c r="X37" s="13"/>
+      <c r="Y37" s="13"/>
+      <c r="Z37" s="13"/>
+      <c r="AA37" s="13"/>
+      <c r="AB37" s="13"/>
+      <c r="AC37" s="13"/>
+      <c r="AD37" s="13"/>
+      <c r="AE37" s="13"/>
+      <c r="AF37" s="13"/>
+      <c r="AG37" s="13"/>
+      <c r="BR37" s="19"/>
     </row>
     <row r="38" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B38" s="28"/>
-      <c r="E38" s="30"/>
-      <c r="F38" s="30"/>
-      <c r="G38" s="30"/>
-      <c r="H38" s="30"/>
-      <c r="I38" s="30"/>
-      <c r="J38" s="30"/>
-      <c r="K38" s="30"/>
-      <c r="L38" s="30"/>
-      <c r="M38" s="30"/>
-      <c r="N38" s="30"/>
-      <c r="O38" s="30"/>
-      <c r="P38" s="30"/>
-      <c r="Q38" s="30"/>
-      <c r="R38" s="30"/>
-      <c r="T38" s="30"/>
-      <c r="U38" s="30"/>
-      <c r="V38" s="30"/>
-      <c r="W38" s="30"/>
-      <c r="X38" s="30"/>
-      <c r="Y38" s="30"/>
-      <c r="Z38" s="30"/>
-      <c r="AA38" s="30"/>
-      <c r="AB38" s="30"/>
-      <c r="AC38" s="30"/>
-      <c r="AD38" s="30"/>
-      <c r="AE38" s="30"/>
-      <c r="AF38" s="30"/>
-      <c r="AG38" s="30"/>
-      <c r="BR38" s="28"/>
+      <c r="B38" s="19"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="13"/>
+      <c r="G38" s="13"/>
+      <c r="H38" s="13"/>
+      <c r="I38" s="13"/>
+      <c r="J38" s="13"/>
+      <c r="K38" s="13"/>
+      <c r="L38" s="13"/>
+      <c r="M38" s="13"/>
+      <c r="N38" s="13"/>
+      <c r="O38" s="13"/>
+      <c r="P38" s="13"/>
+      <c r="Q38" s="13"/>
+      <c r="R38" s="13"/>
+      <c r="T38" s="13"/>
+      <c r="U38" s="13"/>
+      <c r="V38" s="13"/>
+      <c r="W38" s="13"/>
+      <c r="X38" s="13"/>
+      <c r="Y38" s="13"/>
+      <c r="Z38" s="13"/>
+      <c r="AA38" s="13"/>
+      <c r="AB38" s="13"/>
+      <c r="AC38" s="13"/>
+      <c r="AD38" s="13"/>
+      <c r="AE38" s="13"/>
+      <c r="AF38" s="13"/>
+      <c r="AG38" s="13"/>
+      <c r="BR38" s="19"/>
     </row>
     <row r="39" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B39" s="28"/>
-      <c r="E39" s="30"/>
-      <c r="F39" s="30"/>
-      <c r="G39" s="30"/>
-      <c r="H39" s="30"/>
-      <c r="I39" s="30"/>
-      <c r="J39" s="30"/>
-      <c r="K39" s="30"/>
-      <c r="L39" s="30"/>
-      <c r="M39" s="30"/>
-      <c r="N39" s="30"/>
-      <c r="O39" s="30"/>
-      <c r="P39" s="30"/>
-      <c r="Q39" s="30"/>
-      <c r="R39" s="30"/>
-      <c r="T39" s="30"/>
-      <c r="U39" s="30"/>
-      <c r="V39" s="30"/>
-      <c r="W39" s="30"/>
-      <c r="X39" s="30"/>
-      <c r="Y39" s="30"/>
-      <c r="Z39" s="30"/>
-      <c r="AA39" s="30"/>
-      <c r="AB39" s="30"/>
-      <c r="AC39" s="30"/>
-      <c r="AD39" s="30"/>
-      <c r="AE39" s="30"/>
-      <c r="AF39" s="30"/>
-      <c r="AG39" s="30"/>
+      <c r="B39" s="19"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="13"/>
+      <c r="H39" s="13"/>
+      <c r="I39" s="13"/>
+      <c r="J39" s="13"/>
+      <c r="K39" s="13"/>
+      <c r="L39" s="13"/>
+      <c r="M39" s="13"/>
+      <c r="N39" s="13"/>
+      <c r="O39" s="13"/>
+      <c r="P39" s="13"/>
+      <c r="Q39" s="13"/>
+      <c r="R39" s="13"/>
+      <c r="T39" s="13"/>
+      <c r="U39" s="13"/>
+      <c r="V39" s="13"/>
+      <c r="W39" s="13"/>
+      <c r="X39" s="13"/>
+      <c r="Y39" s="13"/>
+      <c r="Z39" s="13"/>
+      <c r="AA39" s="13"/>
+      <c r="AB39" s="13"/>
+      <c r="AC39" s="13"/>
+      <c r="AD39" s="13"/>
+      <c r="AE39" s="13"/>
+      <c r="AF39" s="13"/>
+      <c r="AG39" s="13"/>
       <c r="AW39" s="1" t="s">
         <v>173</v>
       </c>
@@ -3280,10 +3267,10 @@
       </c>
       <c r="BP39" s="16"/>
       <c r="BQ39" s="17"/>
-      <c r="BR39" s="28"/>
+      <c r="BR39" s="19"/>
     </row>
     <row r="40" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B40" s="28"/>
+      <c r="B40" s="19"/>
       <c r="AW40" s="5" t="s">
         <v>179</v>
       </c>
@@ -3317,10 +3304,10 @@
       </c>
       <c r="BP40" s="16"/>
       <c r="BQ40" s="17"/>
-      <c r="BR40" s="28"/>
+      <c r="BR40" s="19"/>
     </row>
     <row r="41" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B41" s="28"/>
+      <c r="B41" s="19"/>
       <c r="AW41" s="5" t="s">
         <v>185</v>
       </c>
@@ -3354,10 +3341,10 @@
       </c>
       <c r="BP41" s="16"/>
       <c r="BQ41" s="17"/>
-      <c r="BR41" s="28"/>
+      <c r="BR41" s="19"/>
     </row>
     <row r="42" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B42" s="28"/>
+      <c r="B42" s="19"/>
       <c r="AW42" s="5" t="s">
         <v>191</v>
       </c>
@@ -3391,76 +3378,76 @@
       </c>
       <c r="BP42" s="16"/>
       <c r="BQ42" s="17"/>
-      <c r="BR42" s="28"/>
+      <c r="BR42" s="19"/>
     </row>
     <row r="43" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B43" s="24"/>
-      <c r="AW43" s="23" t="s">
+      <c r="B43" s="20"/>
+      <c r="AW43" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="AX43" s="18" t="s">
+      <c r="AX43" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="AY43" s="11"/>
-      <c r="AZ43" s="12"/>
-      <c r="BA43" s="18" t="s">
+      <c r="AY43" s="22"/>
+      <c r="AZ43" s="23"/>
+      <c r="BA43" s="21" t="s">
         <v>199</v>
       </c>
-      <c r="BB43" s="11"/>
-      <c r="BC43" s="11"/>
-      <c r="BD43" s="11"/>
-      <c r="BE43" s="11"/>
-      <c r="BF43" s="11"/>
-      <c r="BG43" s="11"/>
-      <c r="BH43" s="12"/>
-      <c r="BI43" s="18" t="s">
+      <c r="BB43" s="22"/>
+      <c r="BC43" s="22"/>
+      <c r="BD43" s="22"/>
+      <c r="BE43" s="22"/>
+      <c r="BF43" s="22"/>
+      <c r="BG43" s="22"/>
+      <c r="BH43" s="23"/>
+      <c r="BI43" s="21" t="s">
         <v>200</v>
       </c>
-      <c r="BJ43" s="11"/>
-      <c r="BK43" s="12"/>
-      <c r="BL43" s="18" t="s">
+      <c r="BJ43" s="22"/>
+      <c r="BK43" s="23"/>
+      <c r="BL43" s="21" t="s">
         <v>201</v>
       </c>
-      <c r="BM43" s="11"/>
-      <c r="BN43" s="12"/>
-      <c r="BO43" s="18" t="s">
+      <c r="BM43" s="22"/>
+      <c r="BN43" s="23"/>
+      <c r="BO43" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="BP43" s="11"/>
-      <c r="BQ43" s="12"/>
-      <c r="BR43" s="24"/>
+      <c r="BP43" s="22"/>
+      <c r="BQ43" s="23"/>
+      <c r="BR43" s="20"/>
     </row>
     <row r="44" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B44" s="23" t="s">
+      <c r="B44" s="18" t="s">
         <v>203</v>
       </c>
-      <c r="AW44" s="24"/>
-      <c r="AX44" s="19"/>
-      <c r="AY44" s="20"/>
-      <c r="AZ44" s="21"/>
-      <c r="BA44" s="19"/>
-      <c r="BB44" s="20"/>
-      <c r="BC44" s="20"/>
-      <c r="BD44" s="20"/>
-      <c r="BE44" s="20"/>
-      <c r="BF44" s="20"/>
-      <c r="BG44" s="20"/>
-      <c r="BH44" s="21"/>
-      <c r="BI44" s="19"/>
-      <c r="BJ44" s="20"/>
-      <c r="BK44" s="21"/>
-      <c r="BL44" s="19"/>
-      <c r="BM44" s="20"/>
-      <c r="BN44" s="21"/>
-      <c r="BO44" s="19"/>
-      <c r="BP44" s="20"/>
-      <c r="BQ44" s="21"/>
-      <c r="BR44" s="23" t="s">
+      <c r="AW44" s="20"/>
+      <c r="AX44" s="24"/>
+      <c r="AY44" s="25"/>
+      <c r="AZ44" s="26"/>
+      <c r="BA44" s="24"/>
+      <c r="BB44" s="25"/>
+      <c r="BC44" s="25"/>
+      <c r="BD44" s="25"/>
+      <c r="BE44" s="25"/>
+      <c r="BF44" s="25"/>
+      <c r="BG44" s="25"/>
+      <c r="BH44" s="26"/>
+      <c r="BI44" s="24"/>
+      <c r="BJ44" s="25"/>
+      <c r="BK44" s="26"/>
+      <c r="BL44" s="24"/>
+      <c r="BM44" s="25"/>
+      <c r="BN44" s="26"/>
+      <c r="BO44" s="24"/>
+      <c r="BP44" s="25"/>
+      <c r="BQ44" s="26"/>
+      <c r="BR44" s="18" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="45" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B45" s="28"/>
+      <c r="B45" s="19"/>
       <c r="AW45" s="5" t="s">
         <v>204</v>
       </c>
@@ -3494,10 +3481,10 @@
       </c>
       <c r="BP45" s="16"/>
       <c r="BQ45" s="17"/>
-      <c r="BR45" s="28"/>
+      <c r="BR45" s="19"/>
     </row>
     <row r="46" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B46" s="28"/>
+      <c r="B46" s="19"/>
       <c r="AW46" s="15" t="s">
         <v>210</v>
       </c>
@@ -3525,42 +3512,42 @@
       <c r="BO46" s="16"/>
       <c r="BP46" s="16"/>
       <c r="BQ46" s="17"/>
-      <c r="BR46" s="28"/>
+      <c r="BR46" s="19"/>
     </row>
     <row r="47" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B47" s="28"/>
-      <c r="E47" s="29" t="s">
-        <v>236</v>
-      </c>
-      <c r="F47" s="30"/>
-      <c r="G47" s="30"/>
-      <c r="H47" s="30"/>
-      <c r="I47" s="30"/>
-      <c r="J47" s="30"/>
-      <c r="K47" s="30"/>
-      <c r="L47" s="30"/>
-      <c r="M47" s="30"/>
-      <c r="N47" s="30"/>
-      <c r="O47" s="30"/>
-      <c r="P47" s="30"/>
-      <c r="Q47" s="30"/>
-      <c r="R47" s="30"/>
-      <c r="T47" s="29" t="s">
-        <v>237</v>
-      </c>
-      <c r="U47" s="30"/>
-      <c r="V47" s="30"/>
-      <c r="W47" s="30"/>
-      <c r="X47" s="30"/>
-      <c r="Y47" s="30"/>
-      <c r="Z47" s="30"/>
-      <c r="AA47" s="30"/>
-      <c r="AB47" s="30"/>
-      <c r="AC47" s="30"/>
-      <c r="AD47" s="30"/>
-      <c r="AE47" s="30"/>
-      <c r="AF47" s="30"/>
-      <c r="AG47" s="30"/>
+      <c r="B47" s="19"/>
+      <c r="E47" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="F47" s="13"/>
+      <c r="G47" s="13"/>
+      <c r="H47" s="13"/>
+      <c r="I47" s="13"/>
+      <c r="J47" s="13"/>
+      <c r="K47" s="13"/>
+      <c r="L47" s="13"/>
+      <c r="M47" s="13"/>
+      <c r="N47" s="13"/>
+      <c r="O47" s="13"/>
+      <c r="P47" s="13"/>
+      <c r="Q47" s="13"/>
+      <c r="R47" s="13"/>
+      <c r="T47" s="12" t="s">
+        <v>235</v>
+      </c>
+      <c r="U47" s="13"/>
+      <c r="V47" s="13"/>
+      <c r="W47" s="13"/>
+      <c r="X47" s="13"/>
+      <c r="Y47" s="13"/>
+      <c r="Z47" s="13"/>
+      <c r="AA47" s="13"/>
+      <c r="AB47" s="13"/>
+      <c r="AC47" s="13"/>
+      <c r="AD47" s="13"/>
+      <c r="AE47" s="13"/>
+      <c r="AF47" s="13"/>
+      <c r="AG47" s="13"/>
       <c r="AW47" s="15" t="s">
         <v>213</v>
       </c>
@@ -3588,352 +3575,350 @@
       <c r="BO47" s="16"/>
       <c r="BP47" s="16"/>
       <c r="BQ47" s="17"/>
-      <c r="BR47" s="28"/>
+      <c r="BR47" s="19"/>
     </row>
     <row r="48" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B48" s="28"/>
-      <c r="E48" s="30"/>
-      <c r="F48" s="30"/>
-      <c r="G48" s="30"/>
-      <c r="H48" s="30"/>
-      <c r="I48" s="30"/>
-      <c r="J48" s="30"/>
-      <c r="K48" s="30"/>
-      <c r="L48" s="30"/>
-      <c r="M48" s="30"/>
-      <c r="N48" s="30"/>
-      <c r="O48" s="30"/>
-      <c r="P48" s="30"/>
-      <c r="Q48" s="30"/>
-      <c r="R48" s="30"/>
-      <c r="T48" s="30"/>
-      <c r="U48" s="30"/>
-      <c r="V48" s="30"/>
-      <c r="W48" s="30"/>
-      <c r="X48" s="30"/>
-      <c r="Y48" s="30"/>
-      <c r="Z48" s="30"/>
-      <c r="AA48" s="30"/>
-      <c r="AB48" s="30"/>
-      <c r="AC48" s="30"/>
-      <c r="AD48" s="30"/>
-      <c r="AE48" s="30"/>
-      <c r="AF48" s="30"/>
-      <c r="AG48" s="30"/>
-      <c r="AW48" s="18" t="s">
+      <c r="B48" s="19"/>
+      <c r="E48" s="13"/>
+      <c r="F48" s="13"/>
+      <c r="G48" s="13"/>
+      <c r="H48" s="13"/>
+      <c r="I48" s="13"/>
+      <c r="J48" s="13"/>
+      <c r="K48" s="13"/>
+      <c r="L48" s="13"/>
+      <c r="M48" s="13"/>
+      <c r="N48" s="13"/>
+      <c r="O48" s="13"/>
+      <c r="P48" s="13"/>
+      <c r="Q48" s="13"/>
+      <c r="R48" s="13"/>
+      <c r="T48" s="13"/>
+      <c r="U48" s="13"/>
+      <c r="V48" s="13"/>
+      <c r="W48" s="13"/>
+      <c r="X48" s="13"/>
+      <c r="Y48" s="13"/>
+      <c r="Z48" s="13"/>
+      <c r="AA48" s="13"/>
+      <c r="AB48" s="13"/>
+      <c r="AC48" s="13"/>
+      <c r="AD48" s="13"/>
+      <c r="AE48" s="13"/>
+      <c r="AF48" s="13"/>
+      <c r="AG48" s="13"/>
+      <c r="AW48" s="21" t="s">
         <v>216</v>
       </c>
-      <c r="AX48" s="11"/>
-      <c r="AY48" s="11"/>
-      <c r="AZ48" s="11"/>
-      <c r="BA48" s="11"/>
-      <c r="BB48" s="11"/>
-      <c r="BC48" s="11"/>
-      <c r="BD48" s="12"/>
-      <c r="BE48" s="18" t="s">
+      <c r="AX48" s="22"/>
+      <c r="AY48" s="22"/>
+      <c r="AZ48" s="22"/>
+      <c r="BA48" s="22"/>
+      <c r="BB48" s="22"/>
+      <c r="BC48" s="22"/>
+      <c r="BD48" s="23"/>
+      <c r="BE48" s="21" t="s">
         <v>217</v>
       </c>
-      <c r="BF48" s="11"/>
-      <c r="BG48" s="11"/>
-      <c r="BH48" s="11"/>
-      <c r="BI48" s="11"/>
-      <c r="BJ48" s="11"/>
-      <c r="BK48" s="11"/>
-      <c r="BL48" s="11"/>
-      <c r="BM48" s="11"/>
-      <c r="BN48" s="11"/>
-      <c r="BO48" s="11"/>
-      <c r="BP48" s="11"/>
-      <c r="BQ48" s="12"/>
-      <c r="BR48" s="28"/>
+      <c r="BF48" s="22"/>
+      <c r="BG48" s="22"/>
+      <c r="BH48" s="22"/>
+      <c r="BI48" s="22"/>
+      <c r="BJ48" s="22"/>
+      <c r="BK48" s="22"/>
+      <c r="BL48" s="22"/>
+      <c r="BM48" s="22"/>
+      <c r="BN48" s="22"/>
+      <c r="BO48" s="22"/>
+      <c r="BP48" s="22"/>
+      <c r="BQ48" s="23"/>
+      <c r="BR48" s="19"/>
     </row>
     <row r="49" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B49" s="28"/>
-      <c r="E49" s="30"/>
-      <c r="F49" s="30"/>
-      <c r="G49" s="30"/>
-      <c r="H49" s="30"/>
-      <c r="I49" s="30"/>
-      <c r="J49" s="30"/>
-      <c r="K49" s="30"/>
-      <c r="L49" s="30"/>
-      <c r="M49" s="30"/>
-      <c r="N49" s="30"/>
-      <c r="O49" s="30"/>
-      <c r="P49" s="30"/>
-      <c r="Q49" s="30"/>
-      <c r="R49" s="30"/>
-      <c r="T49" s="30"/>
-      <c r="U49" s="30"/>
-      <c r="V49" s="30"/>
-      <c r="W49" s="30"/>
-      <c r="X49" s="30"/>
-      <c r="Y49" s="30"/>
-      <c r="Z49" s="30"/>
-      <c r="AA49" s="30"/>
-      <c r="AB49" s="30"/>
-      <c r="AC49" s="30"/>
-      <c r="AD49" s="30"/>
-      <c r="AE49" s="30"/>
-      <c r="AF49" s="30"/>
-      <c r="AG49" s="30"/>
-      <c r="AW49" s="22" t="s">
+      <c r="B49" s="19"/>
+      <c r="E49" s="13"/>
+      <c r="F49" s="13"/>
+      <c r="G49" s="13"/>
+      <c r="H49" s="13"/>
+      <c r="I49" s="13"/>
+      <c r="J49" s="13"/>
+      <c r="K49" s="13"/>
+      <c r="L49" s="13"/>
+      <c r="M49" s="13"/>
+      <c r="N49" s="13"/>
+      <c r="O49" s="13"/>
+      <c r="P49" s="13"/>
+      <c r="Q49" s="13"/>
+      <c r="R49" s="13"/>
+      <c r="T49" s="13"/>
+      <c r="U49" s="13"/>
+      <c r="V49" s="13"/>
+      <c r="W49" s="13"/>
+      <c r="X49" s="13"/>
+      <c r="Y49" s="13"/>
+      <c r="Z49" s="13"/>
+      <c r="AA49" s="13"/>
+      <c r="AB49" s="13"/>
+      <c r="AC49" s="13"/>
+      <c r="AD49" s="13"/>
+      <c r="AE49" s="13"/>
+      <c r="AF49" s="13"/>
+      <c r="AG49" s="13"/>
+      <c r="AW49" s="27"/>
+      <c r="AX49" s="28"/>
+      <c r="AY49" s="28"/>
+      <c r="AZ49" s="28"/>
+      <c r="BA49" s="28"/>
+      <c r="BB49" s="28"/>
+      <c r="BC49" s="28"/>
+      <c r="BD49" s="29"/>
+      <c r="BE49" s="24"/>
+      <c r="BF49" s="25"/>
+      <c r="BG49" s="25"/>
+      <c r="BH49" s="25"/>
+      <c r="BI49" s="25"/>
+      <c r="BJ49" s="25"/>
+      <c r="BK49" s="25"/>
+      <c r="BL49" s="25"/>
+      <c r="BM49" s="25"/>
+      <c r="BN49" s="25"/>
+      <c r="BO49" s="25"/>
+      <c r="BP49" s="25"/>
+      <c r="BQ49" s="26"/>
+      <c r="BR49" s="19"/>
+    </row>
+    <row r="50" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B50" s="19"/>
+      <c r="E50" s="13"/>
+      <c r="F50" s="13"/>
+      <c r="G50" s="13"/>
+      <c r="H50" s="13"/>
+      <c r="I50" s="13"/>
+      <c r="J50" s="13"/>
+      <c r="K50" s="13"/>
+      <c r="L50" s="13"/>
+      <c r="M50" s="13"/>
+      <c r="N50" s="13"/>
+      <c r="O50" s="13"/>
+      <c r="P50" s="13"/>
+      <c r="Q50" s="13"/>
+      <c r="R50" s="13"/>
+      <c r="T50" s="13"/>
+      <c r="U50" s="13"/>
+      <c r="V50" s="13"/>
+      <c r="W50" s="13"/>
+      <c r="X50" s="13"/>
+      <c r="Y50" s="13"/>
+      <c r="Z50" s="13"/>
+      <c r="AA50" s="13"/>
+      <c r="AB50" s="13"/>
+      <c r="AC50" s="13"/>
+      <c r="AD50" s="13"/>
+      <c r="AE50" s="13"/>
+      <c r="AF50" s="13"/>
+      <c r="AG50" s="13"/>
+      <c r="AW50" s="27"/>
+      <c r="AX50" s="28"/>
+      <c r="AY50" s="28"/>
+      <c r="AZ50" s="28"/>
+      <c r="BA50" s="28"/>
+      <c r="BB50" s="28"/>
+      <c r="BC50" s="28"/>
+      <c r="BD50" s="29"/>
+      <c r="BE50" s="21" t="s">
         <v>218</v>
       </c>
-      <c r="AX49" s="13"/>
-      <c r="AY49" s="13"/>
-      <c r="AZ49" s="13"/>
-      <c r="BA49" s="13"/>
-      <c r="BB49" s="13"/>
-      <c r="BC49" s="13"/>
-      <c r="BD49" s="14"/>
-      <c r="BE49" s="19"/>
-      <c r="BF49" s="20"/>
-      <c r="BG49" s="20"/>
-      <c r="BH49" s="20"/>
-      <c r="BI49" s="20"/>
-      <c r="BJ49" s="20"/>
-      <c r="BK49" s="20"/>
-      <c r="BL49" s="20"/>
-      <c r="BM49" s="20"/>
-      <c r="BN49" s="20"/>
-      <c r="BO49" s="20"/>
-      <c r="BP49" s="20"/>
-      <c r="BQ49" s="21"/>
-      <c r="BR49" s="28"/>
-    </row>
-    <row r="50" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B50" s="28"/>
-      <c r="E50" s="30"/>
-      <c r="F50" s="30"/>
-      <c r="G50" s="30"/>
-      <c r="H50" s="30"/>
-      <c r="I50" s="30"/>
-      <c r="J50" s="30"/>
-      <c r="K50" s="30"/>
-      <c r="L50" s="30"/>
-      <c r="M50" s="30"/>
-      <c r="N50" s="30"/>
-      <c r="O50" s="30"/>
-      <c r="P50" s="30"/>
-      <c r="Q50" s="30"/>
-      <c r="R50" s="30"/>
-      <c r="T50" s="30"/>
-      <c r="U50" s="30"/>
-      <c r="V50" s="30"/>
-      <c r="W50" s="30"/>
-      <c r="X50" s="30"/>
-      <c r="Y50" s="30"/>
-      <c r="Z50" s="30"/>
-      <c r="AA50" s="30"/>
-      <c r="AB50" s="30"/>
-      <c r="AC50" s="30"/>
-      <c r="AD50" s="30"/>
-      <c r="AE50" s="30"/>
-      <c r="AF50" s="30"/>
-      <c r="AG50" s="30"/>
-      <c r="AW50" s="22"/>
-      <c r="AX50" s="13"/>
-      <c r="AY50" s="13"/>
-      <c r="AZ50" s="13"/>
-      <c r="BA50" s="13"/>
-      <c r="BB50" s="13"/>
-      <c r="BC50" s="13"/>
-      <c r="BD50" s="14"/>
-      <c r="BE50" s="18" t="s">
+      <c r="BF50" s="22"/>
+      <c r="BG50" s="22"/>
+      <c r="BH50" s="22"/>
+      <c r="BI50" s="22"/>
+      <c r="BJ50" s="22"/>
+      <c r="BK50" s="22"/>
+      <c r="BL50" s="22"/>
+      <c r="BM50" s="22"/>
+      <c r="BN50" s="22"/>
+      <c r="BO50" s="22"/>
+      <c r="BP50" s="22"/>
+      <c r="BQ50" s="23"/>
+      <c r="BR50" s="19"/>
+    </row>
+    <row r="51" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B51" s="19"/>
+      <c r="E51" s="13"/>
+      <c r="F51" s="13"/>
+      <c r="G51" s="13"/>
+      <c r="H51" s="13"/>
+      <c r="I51" s="13"/>
+      <c r="J51" s="13"/>
+      <c r="K51" s="13"/>
+      <c r="L51" s="13"/>
+      <c r="M51" s="13"/>
+      <c r="N51" s="13"/>
+      <c r="O51" s="13"/>
+      <c r="P51" s="13"/>
+      <c r="Q51" s="13"/>
+      <c r="R51" s="13"/>
+      <c r="T51" s="13"/>
+      <c r="U51" s="13"/>
+      <c r="V51" s="13"/>
+      <c r="W51" s="13"/>
+      <c r="X51" s="13"/>
+      <c r="Y51" s="13"/>
+      <c r="Z51" s="13"/>
+      <c r="AA51" s="13"/>
+      <c r="AB51" s="13"/>
+      <c r="AC51" s="13"/>
+      <c r="AD51" s="13"/>
+      <c r="AE51" s="13"/>
+      <c r="AF51" s="13"/>
+      <c r="AG51" s="13"/>
+      <c r="AW51" s="24"/>
+      <c r="AX51" s="25"/>
+      <c r="AY51" s="25"/>
+      <c r="AZ51" s="25"/>
+      <c r="BA51" s="25"/>
+      <c r="BB51" s="25"/>
+      <c r="BC51" s="25"/>
+      <c r="BD51" s="26"/>
+      <c r="BE51" s="24"/>
+      <c r="BF51" s="25"/>
+      <c r="BG51" s="25"/>
+      <c r="BH51" s="25"/>
+      <c r="BI51" s="25"/>
+      <c r="BJ51" s="25"/>
+      <c r="BK51" s="25"/>
+      <c r="BL51" s="25"/>
+      <c r="BM51" s="25"/>
+      <c r="BN51" s="25"/>
+      <c r="BO51" s="25"/>
+      <c r="BP51" s="25"/>
+      <c r="BQ51" s="26"/>
+      <c r="BR51" s="19"/>
+    </row>
+    <row r="52" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B52" s="19"/>
+      <c r="AW52" s="21" t="s">
         <v>219</v>
       </c>
-      <c r="BF50" s="11"/>
-      <c r="BG50" s="11"/>
-      <c r="BH50" s="11"/>
-      <c r="BI50" s="11"/>
-      <c r="BJ50" s="11"/>
-      <c r="BK50" s="11"/>
-      <c r="BL50" s="11"/>
-      <c r="BM50" s="11"/>
-      <c r="BN50" s="11"/>
-      <c r="BO50" s="11"/>
-      <c r="BP50" s="11"/>
-      <c r="BQ50" s="12"/>
-      <c r="BR50" s="28"/>
-    </row>
-    <row r="51" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B51" s="28"/>
-      <c r="E51" s="30"/>
-      <c r="F51" s="30"/>
-      <c r="G51" s="30"/>
-      <c r="H51" s="30"/>
-      <c r="I51" s="30"/>
-      <c r="J51" s="30"/>
-      <c r="K51" s="30"/>
-      <c r="L51" s="30"/>
-      <c r="M51" s="30"/>
-      <c r="N51" s="30"/>
-      <c r="O51" s="30"/>
-      <c r="P51" s="30"/>
-      <c r="Q51" s="30"/>
-      <c r="R51" s="30"/>
-      <c r="T51" s="30"/>
-      <c r="U51" s="30"/>
-      <c r="V51" s="30"/>
-      <c r="W51" s="30"/>
-      <c r="X51" s="30"/>
-      <c r="Y51" s="30"/>
-      <c r="Z51" s="30"/>
-      <c r="AA51" s="30"/>
-      <c r="AB51" s="30"/>
-      <c r="AC51" s="30"/>
-      <c r="AD51" s="30"/>
-      <c r="AE51" s="30"/>
-      <c r="AF51" s="30"/>
-      <c r="AG51" s="30"/>
-      <c r="AW51" s="19"/>
-      <c r="AX51" s="20"/>
-      <c r="AY51" s="20"/>
-      <c r="AZ51" s="20"/>
-      <c r="BA51" s="20"/>
-      <c r="BB51" s="20"/>
-      <c r="BC51" s="20"/>
-      <c r="BD51" s="21"/>
-      <c r="BE51" s="19"/>
-      <c r="BF51" s="20"/>
-      <c r="BG51" s="20"/>
-      <c r="BH51" s="20"/>
-      <c r="BI51" s="20"/>
-      <c r="BJ51" s="20"/>
-      <c r="BK51" s="20"/>
-      <c r="BL51" s="20"/>
-      <c r="BM51" s="20"/>
-      <c r="BN51" s="20"/>
-      <c r="BO51" s="20"/>
-      <c r="BP51" s="20"/>
-      <c r="BQ51" s="21"/>
-      <c r="BR51" s="28"/>
-    </row>
-    <row r="52" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B52" s="28"/>
-      <c r="AW52" s="18" t="s">
+      <c r="AX52" s="22"/>
+      <c r="AY52" s="22"/>
+      <c r="AZ52" s="22"/>
+      <c r="BA52" s="22"/>
+      <c r="BB52" s="22"/>
+      <c r="BC52" s="22"/>
+      <c r="BD52" s="23"/>
+      <c r="BE52" s="21" t="s">
         <v>220</v>
       </c>
-      <c r="AX52" s="11"/>
-      <c r="AY52" s="11"/>
-      <c r="AZ52" s="11"/>
-      <c r="BA52" s="11"/>
-      <c r="BB52" s="11"/>
-      <c r="BC52" s="11"/>
-      <c r="BD52" s="12"/>
-      <c r="BE52" s="18" t="s">
+      <c r="BF52" s="22"/>
+      <c r="BG52" s="22"/>
+      <c r="BH52" s="22"/>
+      <c r="BI52" s="22"/>
+      <c r="BJ52" s="22"/>
+      <c r="BK52" s="22"/>
+      <c r="BL52" s="22"/>
+      <c r="BM52" s="22"/>
+      <c r="BN52" s="22"/>
+      <c r="BO52" s="22"/>
+      <c r="BP52" s="22"/>
+      <c r="BQ52" s="23"/>
+      <c r="BR52" s="19"/>
+    </row>
+    <row r="53" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B53" s="19"/>
+      <c r="AW53" s="27" t="s">
         <v>221</v>
       </c>
-      <c r="BF52" s="11"/>
-      <c r="BG52" s="11"/>
-      <c r="BH52" s="11"/>
-      <c r="BI52" s="11"/>
-      <c r="BJ52" s="11"/>
-      <c r="BK52" s="11"/>
-      <c r="BL52" s="11"/>
-      <c r="BM52" s="11"/>
-      <c r="BN52" s="11"/>
-      <c r="BO52" s="11"/>
-      <c r="BP52" s="11"/>
-      <c r="BQ52" s="12"/>
-      <c r="BR52" s="28"/>
-    </row>
-    <row r="53" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B53" s="28"/>
-      <c r="AW53" s="22" t="s">
+      <c r="AX53" s="28"/>
+      <c r="AY53" s="28"/>
+      <c r="AZ53" s="28"/>
+      <c r="BA53" s="28"/>
+      <c r="BB53" s="28"/>
+      <c r="BC53" s="28"/>
+      <c r="BD53" s="29"/>
+      <c r="BE53" s="27"/>
+      <c r="BF53" s="28"/>
+      <c r="BG53" s="28"/>
+      <c r="BH53" s="28"/>
+      <c r="BI53" s="28"/>
+      <c r="BJ53" s="28"/>
+      <c r="BK53" s="28"/>
+      <c r="BL53" s="28"/>
+      <c r="BM53" s="28"/>
+      <c r="BN53" s="28"/>
+      <c r="BO53" s="28"/>
+      <c r="BP53" s="28"/>
+      <c r="BQ53" s="29"/>
+      <c r="BR53" s="19"/>
+    </row>
+    <row r="54" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B54" s="19"/>
+      <c r="AW54" s="27"/>
+      <c r="AX54" s="28"/>
+      <c r="AY54" s="28"/>
+      <c r="AZ54" s="28"/>
+      <c r="BA54" s="28"/>
+      <c r="BB54" s="28"/>
+      <c r="BC54" s="28"/>
+      <c r="BD54" s="29"/>
+      <c r="BE54" s="27"/>
+      <c r="BF54" s="28"/>
+      <c r="BG54" s="28"/>
+      <c r="BH54" s="28"/>
+      <c r="BI54" s="28"/>
+      <c r="BJ54" s="28"/>
+      <c r="BK54" s="28"/>
+      <c r="BL54" s="28"/>
+      <c r="BM54" s="28"/>
+      <c r="BN54" s="28"/>
+      <c r="BO54" s="28"/>
+      <c r="BP54" s="28"/>
+      <c r="BQ54" s="29"/>
+      <c r="BR54" s="19"/>
+    </row>
+    <row r="55" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B55" s="19"/>
+      <c r="AW55" s="24"/>
+      <c r="AX55" s="25"/>
+      <c r="AY55" s="25"/>
+      <c r="AZ55" s="25"/>
+      <c r="BA55" s="25"/>
+      <c r="BB55" s="25"/>
+      <c r="BC55" s="25"/>
+      <c r="BD55" s="26"/>
+      <c r="BE55" s="24"/>
+      <c r="BF55" s="25"/>
+      <c r="BG55" s="25"/>
+      <c r="BH55" s="25"/>
+      <c r="BI55" s="25"/>
+      <c r="BJ55" s="25"/>
+      <c r="BK55" s="25"/>
+      <c r="BL55" s="25"/>
+      <c r="BM55" s="25"/>
+      <c r="BN55" s="25"/>
+      <c r="BO55" s="25"/>
+      <c r="BP55" s="25"/>
+      <c r="BQ55" s="26"/>
+      <c r="BR55" s="19"/>
+    </row>
+    <row r="56" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B56" s="20"/>
+      <c r="K56" s="12"/>
+      <c r="L56" s="13"/>
+      <c r="M56" s="13"/>
+      <c r="N56" s="13"/>
+      <c r="O56" s="13"/>
+      <c r="AI56" s="12"/>
+      <c r="AJ56" s="13"/>
+      <c r="AK56" s="13"/>
+      <c r="AL56" s="13"/>
+      <c r="AM56" s="13"/>
+      <c r="AW56" s="15" t="s">
         <v>222</v>
-      </c>
-      <c r="AX53" s="13"/>
-      <c r="AY53" s="13"/>
-      <c r="AZ53" s="13"/>
-      <c r="BA53" s="13"/>
-      <c r="BB53" s="13"/>
-      <c r="BC53" s="13"/>
-      <c r="BD53" s="14"/>
-      <c r="BE53" s="22"/>
-      <c r="BF53" s="13"/>
-      <c r="BG53" s="13"/>
-      <c r="BH53" s="13"/>
-      <c r="BI53" s="13"/>
-      <c r="BJ53" s="13"/>
-      <c r="BK53" s="13"/>
-      <c r="BL53" s="13"/>
-      <c r="BM53" s="13"/>
-      <c r="BN53" s="13"/>
-      <c r="BO53" s="13"/>
-      <c r="BP53" s="13"/>
-      <c r="BQ53" s="14"/>
-      <c r="BR53" s="28"/>
-    </row>
-    <row r="54" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B54" s="28"/>
-      <c r="AW54" s="22"/>
-      <c r="AX54" s="13"/>
-      <c r="AY54" s="13"/>
-      <c r="AZ54" s="13"/>
-      <c r="BA54" s="13"/>
-      <c r="BB54" s="13"/>
-      <c r="BC54" s="13"/>
-      <c r="BD54" s="14"/>
-      <c r="BE54" s="22"/>
-      <c r="BF54" s="13"/>
-      <c r="BG54" s="13"/>
-      <c r="BH54" s="13"/>
-      <c r="BI54" s="13"/>
-      <c r="BJ54" s="13"/>
-      <c r="BK54" s="13"/>
-      <c r="BL54" s="13"/>
-      <c r="BM54" s="13"/>
-      <c r="BN54" s="13"/>
-      <c r="BO54" s="13"/>
-      <c r="BP54" s="13"/>
-      <c r="BQ54" s="14"/>
-      <c r="BR54" s="28"/>
-    </row>
-    <row r="55" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B55" s="28"/>
-      <c r="AW55" s="19"/>
-      <c r="AX55" s="20"/>
-      <c r="AY55" s="20"/>
-      <c r="AZ55" s="20"/>
-      <c r="BA55" s="20"/>
-      <c r="BB55" s="20"/>
-      <c r="BC55" s="20"/>
-      <c r="BD55" s="21"/>
-      <c r="BE55" s="19"/>
-      <c r="BF55" s="20"/>
-      <c r="BG55" s="20"/>
-      <c r="BH55" s="20"/>
-      <c r="BI55" s="20"/>
-      <c r="BJ55" s="20"/>
-      <c r="BK55" s="20"/>
-      <c r="BL55" s="20"/>
-      <c r="BM55" s="20"/>
-      <c r="BN55" s="20"/>
-      <c r="BO55" s="20"/>
-      <c r="BP55" s="20"/>
-      <c r="BQ55" s="21"/>
-      <c r="BR55" s="28"/>
-    </row>
-    <row r="56" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B56" s="24"/>
-      <c r="K56" s="29"/>
-      <c r="L56" s="30"/>
-      <c r="M56" s="30"/>
-      <c r="N56" s="30"/>
-      <c r="O56" s="30"/>
-      <c r="AI56" s="29"/>
-      <c r="AJ56" s="30"/>
-      <c r="AK56" s="30"/>
-      <c r="AL56" s="30"/>
-      <c r="AM56" s="30"/>
-      <c r="AW56" s="15" t="s">
-        <v>223</v>
       </c>
       <c r="AX56" s="16"/>
       <c r="AY56" s="16" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AZ56" s="16"/>
       <c r="BA56" s="16"/>
@@ -3953,7 +3938,7 @@
       <c r="BO56" s="16"/>
       <c r="BP56" s="16"/>
       <c r="BQ56" s="17"/>
-      <c r="BR56" s="24"/>
+      <c r="BR56" s="20"/>
     </row>
     <row r="57" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="C57" s="15">
@@ -4039,39 +4024,138 @@
     <row r="58" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <mergeCells count="191">
-    <mergeCell ref="E47:R51"/>
-    <mergeCell ref="T47:AG51"/>
-    <mergeCell ref="AT3:AV11"/>
-    <mergeCell ref="E7:R11"/>
-    <mergeCell ref="T7:AG11"/>
-    <mergeCell ref="E17:R20"/>
-    <mergeCell ref="T17:AG20"/>
-    <mergeCell ref="E26:R29"/>
-    <mergeCell ref="T26:AG29"/>
-    <mergeCell ref="E35:R39"/>
-    <mergeCell ref="T35:AG39"/>
-    <mergeCell ref="AW56:AX56"/>
-    <mergeCell ref="BM25:BO25"/>
-    <mergeCell ref="Y57:AI57"/>
-    <mergeCell ref="BL39:BN39"/>
-    <mergeCell ref="C2:L2"/>
-    <mergeCell ref="BO41:BQ41"/>
-    <mergeCell ref="BF16:BK16"/>
-    <mergeCell ref="AY10:BB10"/>
-    <mergeCell ref="AW11:AX11"/>
-    <mergeCell ref="AY11:BB11"/>
-    <mergeCell ref="BC11:BE11"/>
-    <mergeCell ref="BF11:BK11"/>
-    <mergeCell ref="BM11:BO11"/>
-    <mergeCell ref="AY17:BB17"/>
-    <mergeCell ref="AW24:AX24"/>
-    <mergeCell ref="BF24:BK24"/>
-    <mergeCell ref="BC20:BE20"/>
-    <mergeCell ref="AY15:BB15"/>
-    <mergeCell ref="AW22:AX22"/>
-    <mergeCell ref="BA41:BH41"/>
-    <mergeCell ref="AW26:AX26"/>
-    <mergeCell ref="AY26:BB26"/>
+    <mergeCell ref="M2:X2"/>
+    <mergeCell ref="AU2:BF2"/>
+    <mergeCell ref="AW18:AX18"/>
+    <mergeCell ref="BC8:BE8"/>
+    <mergeCell ref="BI43:BK44"/>
+    <mergeCell ref="AU57:BF57"/>
+    <mergeCell ref="AW9:AX9"/>
+    <mergeCell ref="BC22:BE22"/>
+    <mergeCell ref="BA47:BH47"/>
+    <mergeCell ref="BG2:BQ2"/>
+    <mergeCell ref="AJ2:AT2"/>
+    <mergeCell ref="AY56:BQ56"/>
+    <mergeCell ref="Y2:AI2"/>
+    <mergeCell ref="BF9:BK9"/>
+    <mergeCell ref="AY8:BB8"/>
+    <mergeCell ref="AW17:AX17"/>
+    <mergeCell ref="BO43:BQ44"/>
+    <mergeCell ref="BG57:BQ57"/>
+    <mergeCell ref="BC7:BE7"/>
+    <mergeCell ref="BC15:BE15"/>
+    <mergeCell ref="BA40:BH40"/>
+    <mergeCell ref="AW19:AX19"/>
+    <mergeCell ref="AW53:BD55"/>
+    <mergeCell ref="B3:B16"/>
+    <mergeCell ref="BC9:BE9"/>
+    <mergeCell ref="AY18:BB18"/>
+    <mergeCell ref="BI47:BQ47"/>
+    <mergeCell ref="AW21:AX21"/>
+    <mergeCell ref="AJ57:AT57"/>
+    <mergeCell ref="BC19:BE19"/>
+    <mergeCell ref="AX41:AZ41"/>
+    <mergeCell ref="BM24:BO24"/>
+    <mergeCell ref="BI39:BK39"/>
+    <mergeCell ref="BC21:BE21"/>
+    <mergeCell ref="AX43:AZ44"/>
+    <mergeCell ref="AY19:BB19"/>
+    <mergeCell ref="AY13:BB13"/>
+    <mergeCell ref="AX40:AZ40"/>
+    <mergeCell ref="AY22:BB22"/>
+    <mergeCell ref="BA43:BH44"/>
+    <mergeCell ref="BL40:BN40"/>
+    <mergeCell ref="BC12:BE12"/>
+    <mergeCell ref="BL43:BN44"/>
+    <mergeCell ref="C3:D5"/>
+    <mergeCell ref="C57:L57"/>
+    <mergeCell ref="AW48:BD48"/>
+    <mergeCell ref="AW3:BQ4"/>
+    <mergeCell ref="BE52:BQ55"/>
+    <mergeCell ref="M57:X57"/>
+    <mergeCell ref="AX42:AZ42"/>
+    <mergeCell ref="AW43:AW44"/>
+    <mergeCell ref="BR30:BR43"/>
+    <mergeCell ref="BM8:BO8"/>
+    <mergeCell ref="AX39:AZ39"/>
+    <mergeCell ref="BM16:BO16"/>
+    <mergeCell ref="BA46:BH46"/>
+    <mergeCell ref="K56:O56"/>
+    <mergeCell ref="BA39:BH39"/>
+    <mergeCell ref="BM10:BO10"/>
+    <mergeCell ref="AW31:AX36"/>
+    <mergeCell ref="BE48:BQ49"/>
+    <mergeCell ref="BL42:BN42"/>
+    <mergeCell ref="AI56:AM56"/>
+    <mergeCell ref="AY23:BB23"/>
+    <mergeCell ref="AX45:AZ45"/>
+    <mergeCell ref="BI42:BK42"/>
+    <mergeCell ref="BF21:BK21"/>
+    <mergeCell ref="BO45:BQ45"/>
+    <mergeCell ref="BR44:BR56"/>
+    <mergeCell ref="BI46:BQ46"/>
+    <mergeCell ref="BM23:BO23"/>
+    <mergeCell ref="BE50:BQ51"/>
+    <mergeCell ref="AY5:BB6"/>
+    <mergeCell ref="B17:B29"/>
+    <mergeCell ref="AY9:BB9"/>
+    <mergeCell ref="AW25:AX25"/>
+    <mergeCell ref="AW7:AX7"/>
+    <mergeCell ref="AW15:AX15"/>
+    <mergeCell ref="B44:B56"/>
+    <mergeCell ref="BL41:BN41"/>
+    <mergeCell ref="BA42:BH42"/>
+    <mergeCell ref="AW49:BD51"/>
+    <mergeCell ref="BI45:BK45"/>
+    <mergeCell ref="BC16:BE16"/>
+    <mergeCell ref="BF20:BK20"/>
+    <mergeCell ref="AW20:AX20"/>
+    <mergeCell ref="B30:B43"/>
+    <mergeCell ref="AW47:AZ47"/>
+    <mergeCell ref="BF10:BK10"/>
+    <mergeCell ref="AW10:AX10"/>
+    <mergeCell ref="BF17:BK17"/>
+    <mergeCell ref="AW23:AX23"/>
+    <mergeCell ref="BM5:BO6"/>
+    <mergeCell ref="AW5:AX6"/>
+    <mergeCell ref="BC18:BE18"/>
+    <mergeCell ref="AW13:AX13"/>
+    <mergeCell ref="BA45:BH45"/>
+    <mergeCell ref="AW8:AX8"/>
+    <mergeCell ref="BL45:BN45"/>
+    <mergeCell ref="BF8:BK8"/>
+    <mergeCell ref="BI40:BK40"/>
+    <mergeCell ref="AW46:AZ46"/>
+    <mergeCell ref="BC26:BE26"/>
+    <mergeCell ref="BF26:BK26"/>
+    <mergeCell ref="BM26:BO26"/>
+    <mergeCell ref="BI41:BK41"/>
+    <mergeCell ref="BF15:BK15"/>
+    <mergeCell ref="AY14:BB14"/>
+    <mergeCell ref="AY25:BB25"/>
+    <mergeCell ref="AY31:BQ36"/>
+    <mergeCell ref="AY12:BB12"/>
+    <mergeCell ref="BC14:BE14"/>
+    <mergeCell ref="BM22:BO22"/>
+    <mergeCell ref="AW14:AX14"/>
+    <mergeCell ref="BC10:BE10"/>
+    <mergeCell ref="BM17:BO17"/>
+    <mergeCell ref="BC23:BE23"/>
+    <mergeCell ref="BF18:BK18"/>
+    <mergeCell ref="AW12:AX12"/>
+    <mergeCell ref="BF5:BK6"/>
+    <mergeCell ref="BC17:BE17"/>
+    <mergeCell ref="AY24:BB24"/>
+    <mergeCell ref="BC5:BE6"/>
+    <mergeCell ref="BO42:BQ42"/>
+    <mergeCell ref="BP5:BP6"/>
+    <mergeCell ref="BO40:BQ40"/>
+    <mergeCell ref="BQ5:BQ6"/>
+    <mergeCell ref="BM21:BO21"/>
+    <mergeCell ref="BF13:BK13"/>
+    <mergeCell ref="BL5:BL6"/>
+    <mergeCell ref="AY7:BB7"/>
+    <mergeCell ref="BM14:BO14"/>
     <mergeCell ref="BR17:BR29"/>
     <mergeCell ref="BM9:BO9"/>
     <mergeCell ref="AY16:BB16"/>
@@ -4096,140 +4180,41 @@
     <mergeCell ref="BC13:BE13"/>
     <mergeCell ref="BM13:BO13"/>
     <mergeCell ref="AY20:BB20"/>
+    <mergeCell ref="AW56:AX56"/>
+    <mergeCell ref="BM25:BO25"/>
+    <mergeCell ref="Y57:AI57"/>
+    <mergeCell ref="BL39:BN39"/>
+    <mergeCell ref="C2:L2"/>
+    <mergeCell ref="BO41:BQ41"/>
+    <mergeCell ref="BF16:BK16"/>
+    <mergeCell ref="AY10:BB10"/>
+    <mergeCell ref="AW11:AX11"/>
+    <mergeCell ref="AY11:BB11"/>
+    <mergeCell ref="BC11:BE11"/>
+    <mergeCell ref="BF11:BK11"/>
+    <mergeCell ref="BM11:BO11"/>
+    <mergeCell ref="AY17:BB17"/>
+    <mergeCell ref="AW24:AX24"/>
+    <mergeCell ref="BF24:BK24"/>
+    <mergeCell ref="BC20:BE20"/>
+    <mergeCell ref="AY15:BB15"/>
+    <mergeCell ref="AW22:AX22"/>
+    <mergeCell ref="BA41:BH41"/>
+    <mergeCell ref="AW26:AX26"/>
+    <mergeCell ref="AY26:BB26"/>
     <mergeCell ref="AW52:BD52"/>
     <mergeCell ref="AW16:AX16"/>
-    <mergeCell ref="BF5:BK6"/>
-    <mergeCell ref="BC17:BE17"/>
-    <mergeCell ref="AY24:BB24"/>
-    <mergeCell ref="BC5:BE6"/>
-    <mergeCell ref="BO42:BQ42"/>
-    <mergeCell ref="BP5:BP6"/>
-    <mergeCell ref="BO40:BQ40"/>
-    <mergeCell ref="BQ5:BQ6"/>
-    <mergeCell ref="BM21:BO21"/>
-    <mergeCell ref="BF13:BK13"/>
-    <mergeCell ref="AW13:AX13"/>
-    <mergeCell ref="BA45:BH45"/>
-    <mergeCell ref="AW8:AX8"/>
-    <mergeCell ref="BL45:BN45"/>
-    <mergeCell ref="BF8:BK8"/>
-    <mergeCell ref="BI40:BK40"/>
-    <mergeCell ref="AW46:AZ46"/>
-    <mergeCell ref="BC26:BE26"/>
-    <mergeCell ref="BF26:BK26"/>
-    <mergeCell ref="BM26:BO26"/>
-    <mergeCell ref="BE50:BQ51"/>
-    <mergeCell ref="AY5:BB6"/>
-    <mergeCell ref="B17:B29"/>
-    <mergeCell ref="AY9:BB9"/>
-    <mergeCell ref="AW25:AX25"/>
-    <mergeCell ref="AW7:AX7"/>
-    <mergeCell ref="AW15:AX15"/>
-    <mergeCell ref="B44:B56"/>
-    <mergeCell ref="BL41:BN41"/>
-    <mergeCell ref="BA42:BH42"/>
-    <mergeCell ref="AW49:BD51"/>
-    <mergeCell ref="BI45:BK45"/>
-    <mergeCell ref="BC16:BE16"/>
-    <mergeCell ref="BF20:BK20"/>
-    <mergeCell ref="AW20:AX20"/>
-    <mergeCell ref="B30:B43"/>
-    <mergeCell ref="AW47:AZ47"/>
-    <mergeCell ref="BF10:BK10"/>
-    <mergeCell ref="AW10:AX10"/>
-    <mergeCell ref="BF17:BK17"/>
-    <mergeCell ref="AW23:AX23"/>
-    <mergeCell ref="BM5:BO6"/>
-    <mergeCell ref="AW5:AX6"/>
-    <mergeCell ref="BC18:BE18"/>
-    <mergeCell ref="BI41:BK41"/>
-    <mergeCell ref="BE52:BQ55"/>
-    <mergeCell ref="M57:X57"/>
-    <mergeCell ref="AX42:AZ42"/>
-    <mergeCell ref="AW43:AW44"/>
-    <mergeCell ref="BR30:BR43"/>
-    <mergeCell ref="BM8:BO8"/>
-    <mergeCell ref="AX39:AZ39"/>
-    <mergeCell ref="BM16:BO16"/>
-    <mergeCell ref="BA46:BH46"/>
-    <mergeCell ref="K56:O56"/>
-    <mergeCell ref="BA39:BH39"/>
-    <mergeCell ref="BM10:BO10"/>
-    <mergeCell ref="AW31:AX36"/>
-    <mergeCell ref="BE48:BQ49"/>
-    <mergeCell ref="BL42:BN42"/>
-    <mergeCell ref="AI56:AM56"/>
-    <mergeCell ref="AY23:BB23"/>
-    <mergeCell ref="AX45:AZ45"/>
-    <mergeCell ref="BI42:BK42"/>
-    <mergeCell ref="BF21:BK21"/>
-    <mergeCell ref="BO45:BQ45"/>
-    <mergeCell ref="BR44:BR56"/>
-    <mergeCell ref="B3:B16"/>
-    <mergeCell ref="BC9:BE9"/>
-    <mergeCell ref="AY18:BB18"/>
-    <mergeCell ref="BI47:BQ47"/>
-    <mergeCell ref="AW21:AX21"/>
-    <mergeCell ref="AJ57:AT57"/>
-    <mergeCell ref="BC19:BE19"/>
-    <mergeCell ref="AX41:AZ41"/>
-    <mergeCell ref="BM24:BO24"/>
-    <mergeCell ref="BI39:BK39"/>
-    <mergeCell ref="BC21:BE21"/>
-    <mergeCell ref="AX43:AZ44"/>
-    <mergeCell ref="AY19:BB19"/>
-    <mergeCell ref="AY13:BB13"/>
-    <mergeCell ref="AX40:AZ40"/>
-    <mergeCell ref="AY22:BB22"/>
-    <mergeCell ref="BA43:BH44"/>
-    <mergeCell ref="BL40:BN40"/>
-    <mergeCell ref="BC12:BE12"/>
-    <mergeCell ref="BL43:BN44"/>
-    <mergeCell ref="C3:D5"/>
-    <mergeCell ref="C57:L57"/>
-    <mergeCell ref="AW48:BD48"/>
-    <mergeCell ref="AW3:BQ4"/>
-    <mergeCell ref="BI46:BQ46"/>
-    <mergeCell ref="BM23:BO23"/>
-    <mergeCell ref="BF15:BK15"/>
-    <mergeCell ref="BL5:BL6"/>
-    <mergeCell ref="AY14:BB14"/>
-    <mergeCell ref="AY25:BB25"/>
-    <mergeCell ref="AY31:BQ36"/>
-    <mergeCell ref="AY12:BB12"/>
-    <mergeCell ref="BC14:BE14"/>
-    <mergeCell ref="BM22:BO22"/>
-    <mergeCell ref="AW14:AX14"/>
-    <mergeCell ref="AY7:BB7"/>
-    <mergeCell ref="BC10:BE10"/>
-    <mergeCell ref="BM17:BO17"/>
-    <mergeCell ref="BC23:BE23"/>
-    <mergeCell ref="BF18:BK18"/>
-    <mergeCell ref="AW12:AX12"/>
-    <mergeCell ref="BM14:BO14"/>
-    <mergeCell ref="M2:X2"/>
-    <mergeCell ref="AU2:BF2"/>
-    <mergeCell ref="AW18:AX18"/>
-    <mergeCell ref="BC8:BE8"/>
-    <mergeCell ref="BI43:BK44"/>
-    <mergeCell ref="AU57:BF57"/>
-    <mergeCell ref="AW9:AX9"/>
-    <mergeCell ref="BC22:BE22"/>
-    <mergeCell ref="BA47:BH47"/>
-    <mergeCell ref="BG2:BQ2"/>
-    <mergeCell ref="AJ2:AT2"/>
-    <mergeCell ref="AY56:BQ56"/>
-    <mergeCell ref="Y2:AI2"/>
-    <mergeCell ref="BF9:BK9"/>
-    <mergeCell ref="AY8:BB8"/>
-    <mergeCell ref="AW17:AX17"/>
-    <mergeCell ref="BO43:BQ44"/>
-    <mergeCell ref="BG57:BQ57"/>
-    <mergeCell ref="BC7:BE7"/>
-    <mergeCell ref="BC15:BE15"/>
-    <mergeCell ref="BA40:BH40"/>
-    <mergeCell ref="AW19:AX19"/>
-    <mergeCell ref="AW53:BD55"/>
+    <mergeCell ref="E47:R51"/>
+    <mergeCell ref="T47:AG51"/>
+    <mergeCell ref="AT3:AV11"/>
+    <mergeCell ref="E7:R11"/>
+    <mergeCell ref="T7:AG11"/>
+    <mergeCell ref="E17:R20"/>
+    <mergeCell ref="T17:AG20"/>
+    <mergeCell ref="E26:R29"/>
+    <mergeCell ref="T26:AG29"/>
+    <mergeCell ref="E35:R39"/>
+    <mergeCell ref="T35:AG39"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
[auto] session sync 2026-07-21T02:20:50Z
</commit_message>
<xml_diff>
--- a/가공도_도면_1.xlsx
+++ b/가공도_도면_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\duddl\Desktop\Project\a2z\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{660380A4-5322-4233-9727-47280CFCE2E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDEB2998-C9AF-484C-A642-9381DB1EC01C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1920" yWindow="720" windowWidth="20256" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="231">
   <si>
     <t>A</t>
   </si>
@@ -527,9 +527,6 @@
   </si>
   <si>
     <t>C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note : </t>
   </si>
   <si>
     <t>{Input_164}</t>
@@ -994,9 +991,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1015,15 +1009,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1031,6 +1016,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1044,15 +1050,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1518,189 +1515,189 @@
       <c r="BR2" s="2"/>
     </row>
     <row r="3" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="29" t="s">
-        <v>224</v>
-      </c>
-      <c r="D3" s="30"/>
+      <c r="C3" s="32" t="s">
+        <v>223</v>
+      </c>
+      <c r="D3" s="33"/>
       <c r="Y3" s="3"/>
-      <c r="AT3" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="AU3" s="18"/>
-      <c r="AV3" s="19"/>
-      <c r="AW3" s="17" t="s">
+      <c r="AT3" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="AU3" s="17"/>
+      <c r="AV3" s="18"/>
+      <c r="AW3" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="AX3" s="18"/>
-      <c r="AY3" s="18"/>
-      <c r="AZ3" s="18"/>
-      <c r="BA3" s="18"/>
-      <c r="BB3" s="18"/>
-      <c r="BC3" s="18"/>
-      <c r="BD3" s="18"/>
-      <c r="BE3" s="18"/>
-      <c r="BF3" s="18"/>
-      <c r="BG3" s="18"/>
-      <c r="BH3" s="18"/>
-      <c r="BI3" s="18"/>
-      <c r="BJ3" s="18"/>
-      <c r="BK3" s="18"/>
-      <c r="BL3" s="18"/>
-      <c r="BM3" s="18"/>
-      <c r="BN3" s="18"/>
-      <c r="BO3" s="18"/>
-      <c r="BP3" s="18"/>
-      <c r="BQ3" s="19"/>
-      <c r="BR3" s="23" t="s">
+      <c r="AX3" s="17"/>
+      <c r="AY3" s="17"/>
+      <c r="AZ3" s="17"/>
+      <c r="BA3" s="17"/>
+      <c r="BB3" s="17"/>
+      <c r="BC3" s="17"/>
+      <c r="BD3" s="17"/>
+      <c r="BE3" s="17"/>
+      <c r="BF3" s="17"/>
+      <c r="BG3" s="17"/>
+      <c r="BH3" s="17"/>
+      <c r="BI3" s="17"/>
+      <c r="BJ3" s="17"/>
+      <c r="BK3" s="17"/>
+      <c r="BL3" s="17"/>
+      <c r="BM3" s="17"/>
+      <c r="BN3" s="17"/>
+      <c r="BO3" s="17"/>
+      <c r="BP3" s="17"/>
+      <c r="BQ3" s="18"/>
+      <c r="BR3" s="25" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="24"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="32"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="35"/>
       <c r="E4" s="3"/>
       <c r="AA4" s="3"/>
-      <c r="AT4" s="27"/>
-      <c r="AU4" s="27"/>
-      <c r="AV4" s="28"/>
-      <c r="AW4" s="20"/>
-      <c r="AX4" s="21"/>
-      <c r="AY4" s="21"/>
-      <c r="AZ4" s="21"/>
-      <c r="BA4" s="21"/>
-      <c r="BB4" s="21"/>
-      <c r="BC4" s="21"/>
-      <c r="BD4" s="21"/>
-      <c r="BE4" s="21"/>
-      <c r="BF4" s="21"/>
-      <c r="BG4" s="21"/>
-      <c r="BH4" s="21"/>
-      <c r="BI4" s="21"/>
-      <c r="BJ4" s="21"/>
-      <c r="BK4" s="21"/>
-      <c r="BL4" s="21"/>
-      <c r="BM4" s="21"/>
-      <c r="BN4" s="21"/>
-      <c r="BO4" s="21"/>
-      <c r="BP4" s="21"/>
-      <c r="BQ4" s="22"/>
-      <c r="BR4" s="24"/>
+      <c r="AT4" s="23"/>
+      <c r="AU4" s="23"/>
+      <c r="AV4" s="24"/>
+      <c r="AW4" s="19"/>
+      <c r="AX4" s="20"/>
+      <c r="AY4" s="20"/>
+      <c r="AZ4" s="20"/>
+      <c r="BA4" s="20"/>
+      <c r="BB4" s="20"/>
+      <c r="BC4" s="20"/>
+      <c r="BD4" s="20"/>
+      <c r="BE4" s="20"/>
+      <c r="BF4" s="20"/>
+      <c r="BG4" s="20"/>
+      <c r="BH4" s="20"/>
+      <c r="BI4" s="20"/>
+      <c r="BJ4" s="20"/>
+      <c r="BK4" s="20"/>
+      <c r="BL4" s="20"/>
+      <c r="BM4" s="20"/>
+      <c r="BN4" s="20"/>
+      <c r="BO4" s="20"/>
+      <c r="BP4" s="20"/>
+      <c r="BQ4" s="21"/>
+      <c r="BR4" s="31"/>
     </row>
     <row r="5" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="24"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="32"/>
-      <c r="AT5" s="27"/>
-      <c r="AU5" s="27"/>
-      <c r="AV5" s="28"/>
-      <c r="AW5" s="17" t="s">
-        <v>218</v>
-      </c>
-      <c r="AX5" s="19"/>
-      <c r="AY5" s="17" t="s">
+      <c r="B5" s="31"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="35"/>
+      <c r="AT5" s="23"/>
+      <c r="AU5" s="23"/>
+      <c r="AV5" s="24"/>
+      <c r="AW5" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="AX5" s="18"/>
+      <c r="AY5" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="AZ5" s="18"/>
-      <c r="BA5" s="18"/>
-      <c r="BB5" s="19"/>
-      <c r="BC5" s="17" t="s">
+      <c r="AZ5" s="17"/>
+      <c r="BA5" s="17"/>
+      <c r="BB5" s="18"/>
+      <c r="BC5" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="BD5" s="18"/>
-      <c r="BE5" s="19"/>
-      <c r="BF5" s="17" t="s">
+      <c r="BD5" s="17"/>
+      <c r="BE5" s="18"/>
+      <c r="BF5" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="BG5" s="18"/>
-      <c r="BH5" s="18"/>
-      <c r="BI5" s="18"/>
-      <c r="BJ5" s="18"/>
-      <c r="BK5" s="19"/>
-      <c r="BL5" s="23" t="s">
+      <c r="BG5" s="17"/>
+      <c r="BH5" s="17"/>
+      <c r="BI5" s="17"/>
+      <c r="BJ5" s="17"/>
+      <c r="BK5" s="18"/>
+      <c r="BL5" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="BM5" s="17" t="s">
+      <c r="BM5" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="BN5" s="18"/>
-      <c r="BO5" s="19"/>
-      <c r="BP5" s="23" t="s">
+      <c r="BN5" s="17"/>
+      <c r="BO5" s="18"/>
+      <c r="BP5" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="BQ5" s="23" t="s">
+      <c r="BQ5" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="BR5" s="24"/>
+      <c r="BR5" s="31"/>
     </row>
     <row r="6" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="24"/>
-      <c r="AT6" s="27"/>
-      <c r="AU6" s="27"/>
-      <c r="AV6" s="28"/>
-      <c r="AW6" s="20"/>
-      <c r="AX6" s="22"/>
-      <c r="AY6" s="20"/>
-      <c r="AZ6" s="21"/>
-      <c r="BA6" s="21"/>
-      <c r="BB6" s="22"/>
-      <c r="BC6" s="20"/>
-      <c r="BD6" s="21"/>
-      <c r="BE6" s="22"/>
-      <c r="BF6" s="20"/>
-      <c r="BG6" s="21"/>
-      <c r="BH6" s="21"/>
-      <c r="BI6" s="21"/>
-      <c r="BJ6" s="21"/>
-      <c r="BK6" s="22"/>
-      <c r="BL6" s="25"/>
-      <c r="BM6" s="20"/>
-      <c r="BN6" s="21"/>
-      <c r="BO6" s="22"/>
-      <c r="BP6" s="25"/>
-      <c r="BQ6" s="25"/>
-      <c r="BR6" s="24"/>
+      <c r="B6" s="31"/>
+      <c r="AT6" s="23"/>
+      <c r="AU6" s="23"/>
+      <c r="AV6" s="24"/>
+      <c r="AW6" s="19"/>
+      <c r="AX6" s="21"/>
+      <c r="AY6" s="19"/>
+      <c r="AZ6" s="20"/>
+      <c r="BA6" s="20"/>
+      <c r="BB6" s="21"/>
+      <c r="BC6" s="19"/>
+      <c r="BD6" s="20"/>
+      <c r="BE6" s="21"/>
+      <c r="BF6" s="19"/>
+      <c r="BG6" s="20"/>
+      <c r="BH6" s="20"/>
+      <c r="BI6" s="20"/>
+      <c r="BJ6" s="20"/>
+      <c r="BK6" s="21"/>
+      <c r="BL6" s="26"/>
+      <c r="BM6" s="19"/>
+      <c r="BN6" s="20"/>
+      <c r="BO6" s="21"/>
+      <c r="BP6" s="26"/>
+      <c r="BQ6" s="26"/>
+      <c r="BR6" s="31"/>
     </row>
     <row r="7" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="24"/>
-      <c r="E7" s="16" t="s">
-        <v>226</v>
-      </c>
-      <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
-      <c r="H7" s="16"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="16"/>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="16"/>
-      <c r="O7" s="16"/>
-      <c r="P7" s="16"/>
-      <c r="Q7" s="16"/>
-      <c r="R7" s="16"/>
-      <c r="T7" s="16" t="s">
+      <c r="B7" s="31"/>
+      <c r="E7" s="30" t="s">
+        <v>225</v>
+      </c>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="30"/>
+      <c r="K7" s="30"/>
+      <c r="L7" s="30"/>
+      <c r="M7" s="30"/>
+      <c r="N7" s="30"/>
+      <c r="O7" s="30"/>
+      <c r="P7" s="30"/>
+      <c r="Q7" s="30"/>
+      <c r="R7" s="30"/>
+      <c r="T7" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="U7" s="16"/>
-      <c r="V7" s="16"/>
-      <c r="W7" s="16"/>
-      <c r="X7" s="16"/>
-      <c r="Y7" s="16"/>
-      <c r="Z7" s="16"/>
-      <c r="AA7" s="16"/>
-      <c r="AB7" s="16"/>
-      <c r="AC7" s="16"/>
-      <c r="AD7" s="16"/>
-      <c r="AE7" s="16"/>
-      <c r="AF7" s="16"/>
-      <c r="AG7" s="16"/>
-      <c r="AT7" s="27"/>
-      <c r="AU7" s="27"/>
-      <c r="AV7" s="28"/>
+      <c r="U7" s="30"/>
+      <c r="V7" s="30"/>
+      <c r="W7" s="30"/>
+      <c r="X7" s="30"/>
+      <c r="Y7" s="30"/>
+      <c r="Z7" s="30"/>
+      <c r="AA7" s="30"/>
+      <c r="AB7" s="30"/>
+      <c r="AC7" s="30"/>
+      <c r="AD7" s="30"/>
+      <c r="AE7" s="30"/>
+      <c r="AF7" s="30"/>
+      <c r="AG7" s="30"/>
+      <c r="AT7" s="23"/>
+      <c r="AU7" s="23"/>
+      <c r="AV7" s="24"/>
       <c r="AW7" s="13" t="s">
         <v>11</v>
       </c>
@@ -1738,41 +1735,41 @@
       <c r="BQ7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="BR7" s="24"/>
+      <c r="BR7" s="31"/>
     </row>
     <row r="8" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B8" s="24"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="16"/>
-      <c r="P8" s="16"/>
-      <c r="Q8" s="16"/>
-      <c r="R8" s="16"/>
-      <c r="T8" s="16"/>
-      <c r="U8" s="16"/>
-      <c r="V8" s="16"/>
-      <c r="W8" s="16"/>
-      <c r="X8" s="16"/>
-      <c r="Y8" s="16"/>
-      <c r="Z8" s="16"/>
-      <c r="AA8" s="16"/>
-      <c r="AB8" s="16"/>
-      <c r="AC8" s="16"/>
-      <c r="AD8" s="16"/>
-      <c r="AE8" s="16"/>
-      <c r="AF8" s="16"/>
-      <c r="AG8" s="16"/>
-      <c r="AT8" s="27"/>
-      <c r="AU8" s="27"/>
-      <c r="AV8" s="28"/>
+      <c r="B8" s="31"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
+      <c r="M8" s="30"/>
+      <c r="N8" s="30"/>
+      <c r="O8" s="30"/>
+      <c r="P8" s="30"/>
+      <c r="Q8" s="30"/>
+      <c r="R8" s="30"/>
+      <c r="T8" s="30"/>
+      <c r="U8" s="30"/>
+      <c r="V8" s="30"/>
+      <c r="W8" s="30"/>
+      <c r="X8" s="30"/>
+      <c r="Y8" s="30"/>
+      <c r="Z8" s="30"/>
+      <c r="AA8" s="30"/>
+      <c r="AB8" s="30"/>
+      <c r="AC8" s="30"/>
+      <c r="AD8" s="30"/>
+      <c r="AE8" s="30"/>
+      <c r="AF8" s="30"/>
+      <c r="AG8" s="30"/>
+      <c r="AT8" s="23"/>
+      <c r="AU8" s="23"/>
+      <c r="AV8" s="24"/>
       <c r="AW8" s="13" t="s">
         <v>19</v>
       </c>
@@ -1810,38 +1807,38 @@
       <c r="BQ8" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="BR8" s="24"/>
+      <c r="BR8" s="31"/>
     </row>
     <row r="9" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B9" s="24"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="16"/>
-      <c r="P9" s="16"/>
-      <c r="Q9" s="16"/>
-      <c r="R9" s="16"/>
-      <c r="T9" s="16"/>
-      <c r="U9" s="16"/>
-      <c r="V9" s="16"/>
-      <c r="W9" s="16"/>
-      <c r="X9" s="16"/>
-      <c r="Y9" s="16"/>
-      <c r="Z9" s="16"/>
-      <c r="AA9" s="16"/>
-      <c r="AB9" s="16"/>
-      <c r="AC9" s="16"/>
-      <c r="AD9" s="16"/>
-      <c r="AE9" s="16"/>
-      <c r="AF9" s="16"/>
-      <c r="AG9" s="16"/>
+      <c r="B9" s="31"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
+      <c r="K9" s="30"/>
+      <c r="L9" s="30"/>
+      <c r="M9" s="30"/>
+      <c r="N9" s="30"/>
+      <c r="O9" s="30"/>
+      <c r="P9" s="30"/>
+      <c r="Q9" s="30"/>
+      <c r="R9" s="30"/>
+      <c r="T9" s="30"/>
+      <c r="U9" s="30"/>
+      <c r="V9" s="30"/>
+      <c r="W9" s="30"/>
+      <c r="X9" s="30"/>
+      <c r="Y9" s="30"/>
+      <c r="Z9" s="30"/>
+      <c r="AA9" s="30"/>
+      <c r="AB9" s="30"/>
+      <c r="AC9" s="30"/>
+      <c r="AD9" s="30"/>
+      <c r="AE9" s="30"/>
+      <c r="AF9" s="30"/>
+      <c r="AG9" s="30"/>
       <c r="AT9" s="11"/>
       <c r="AU9" s="11"/>
       <c r="AV9" s="12"/>
@@ -1882,38 +1879,38 @@
       <c r="BQ9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="BR9" s="24"/>
+      <c r="BR9" s="31"/>
     </row>
     <row r="10" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="24"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="16"/>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
-      <c r="N10" s="16"/>
-      <c r="O10" s="16"/>
-      <c r="P10" s="16"/>
-      <c r="Q10" s="16"/>
-      <c r="R10" s="16"/>
-      <c r="T10" s="16"/>
-      <c r="U10" s="16"/>
-      <c r="V10" s="16"/>
-      <c r="W10" s="16"/>
-      <c r="X10" s="16"/>
-      <c r="Y10" s="16"/>
-      <c r="Z10" s="16"/>
-      <c r="AA10" s="16"/>
-      <c r="AB10" s="16"/>
-      <c r="AC10" s="16"/>
-      <c r="AD10" s="16"/>
-      <c r="AE10" s="16"/>
-      <c r="AF10" s="16"/>
-      <c r="AG10" s="16"/>
+      <c r="B10" s="31"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
+      <c r="K10" s="30"/>
+      <c r="L10" s="30"/>
+      <c r="M10" s="30"/>
+      <c r="N10" s="30"/>
+      <c r="O10" s="30"/>
+      <c r="P10" s="30"/>
+      <c r="Q10" s="30"/>
+      <c r="R10" s="30"/>
+      <c r="T10" s="30"/>
+      <c r="U10" s="30"/>
+      <c r="V10" s="30"/>
+      <c r="W10" s="30"/>
+      <c r="X10" s="30"/>
+      <c r="Y10" s="30"/>
+      <c r="Z10" s="30"/>
+      <c r="AA10" s="30"/>
+      <c r="AB10" s="30"/>
+      <c r="AC10" s="30"/>
+      <c r="AD10" s="30"/>
+      <c r="AE10" s="30"/>
+      <c r="AF10" s="30"/>
+      <c r="AG10" s="30"/>
       <c r="AT10" s="11"/>
       <c r="AU10" s="11"/>
       <c r="AV10" s="12"/>
@@ -1954,38 +1951,38 @@
       <c r="BQ10" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="BR10" s="24"/>
+      <c r="BR10" s="31"/>
     </row>
     <row r="11" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="24"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="16"/>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="16"/>
-      <c r="O11" s="16"/>
-      <c r="P11" s="16"/>
-      <c r="Q11" s="16"/>
-      <c r="R11" s="16"/>
-      <c r="T11" s="16"/>
-      <c r="U11" s="16"/>
-      <c r="V11" s="16"/>
-      <c r="W11" s="16"/>
-      <c r="X11" s="16"/>
-      <c r="Y11" s="16"/>
-      <c r="Z11" s="16"/>
-      <c r="AA11" s="16"/>
-      <c r="AB11" s="16"/>
-      <c r="AC11" s="16"/>
-      <c r="AD11" s="16"/>
-      <c r="AE11" s="16"/>
-      <c r="AF11" s="16"/>
-      <c r="AG11" s="16"/>
+      <c r="B11" s="31"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="30"/>
+      <c r="J11" s="30"/>
+      <c r="K11" s="30"/>
+      <c r="L11" s="30"/>
+      <c r="M11" s="30"/>
+      <c r="N11" s="30"/>
+      <c r="O11" s="30"/>
+      <c r="P11" s="30"/>
+      <c r="Q11" s="30"/>
+      <c r="R11" s="30"/>
+      <c r="T11" s="30"/>
+      <c r="U11" s="30"/>
+      <c r="V11" s="30"/>
+      <c r="W11" s="30"/>
+      <c r="X11" s="30"/>
+      <c r="Y11" s="30"/>
+      <c r="Z11" s="30"/>
+      <c r="AA11" s="30"/>
+      <c r="AB11" s="30"/>
+      <c r="AC11" s="30"/>
+      <c r="AD11" s="30"/>
+      <c r="AE11" s="30"/>
+      <c r="AF11" s="30"/>
+      <c r="AG11" s="30"/>
       <c r="AT11" s="11"/>
       <c r="AU11" s="11"/>
       <c r="AV11" s="12"/>
@@ -2026,10 +2023,10 @@
       <c r="BQ11" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="BR11" s="24"/>
+      <c r="BR11" s="31"/>
     </row>
     <row r="12" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="24"/>
+      <c r="B12" s="31"/>
       <c r="AW12" s="13" t="s">
         <v>51</v>
       </c>
@@ -2067,10 +2064,10 @@
       <c r="BQ12" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="BR12" s="24"/>
+      <c r="BR12" s="31"/>
     </row>
     <row r="13" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="24"/>
+      <c r="B13" s="31"/>
       <c r="AW13" s="13" t="s">
         <v>59</v>
       </c>
@@ -2108,10 +2105,10 @@
       <c r="BQ13" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="BR13" s="24"/>
+      <c r="BR13" s="31"/>
     </row>
     <row r="14" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="24"/>
+      <c r="B14" s="31"/>
       <c r="AW14" s="13" t="s">
         <v>67</v>
       </c>
@@ -2149,10 +2146,10 @@
       <c r="BQ14" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="BR14" s="24"/>
+      <c r="BR14" s="31"/>
     </row>
     <row r="15" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B15" s="24"/>
+      <c r="B15" s="31"/>
       <c r="AW15" s="13" t="s">
         <v>75</v>
       </c>
@@ -2190,10 +2187,10 @@
       <c r="BQ15" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="BR15" s="24"/>
+      <c r="BR15" s="31"/>
     </row>
     <row r="16" spans="1:71" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="25"/>
+      <c r="B16" s="26"/>
       <c r="AW16" s="13" t="s">
         <v>84</v>
       </c>
@@ -2231,44 +2228,44 @@
       <c r="BQ16" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="BR16" s="25"/>
+      <c r="BR16" s="26"/>
     </row>
     <row r="17" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="16" t="s">
-        <v>227</v>
-      </c>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="16"/>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
-      <c r="N17" s="16"/>
-      <c r="O17" s="16"/>
-      <c r="P17" s="16"/>
-      <c r="Q17" s="16"/>
-      <c r="R17" s="16"/>
-      <c r="T17" s="16" t="s">
+      <c r="E17" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="F17" s="30"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="30"/>
+      <c r="K17" s="30"/>
+      <c r="L17" s="30"/>
+      <c r="M17" s="30"/>
+      <c r="N17" s="30"/>
+      <c r="O17" s="30"/>
+      <c r="P17" s="30"/>
+      <c r="Q17" s="30"/>
+      <c r="R17" s="30"/>
+      <c r="T17" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="U17" s="16"/>
-      <c r="V17" s="16"/>
-      <c r="W17" s="16"/>
-      <c r="X17" s="16"/>
-      <c r="Y17" s="16"/>
-      <c r="Z17" s="16"/>
-      <c r="AA17" s="16"/>
-      <c r="AB17" s="16"/>
-      <c r="AC17" s="16"/>
-      <c r="AD17" s="16"/>
-      <c r="AE17" s="16"/>
-      <c r="AF17" s="16"/>
-      <c r="AG17" s="16"/>
+      <c r="U17" s="30"/>
+      <c r="V17" s="30"/>
+      <c r="W17" s="30"/>
+      <c r="X17" s="30"/>
+      <c r="Y17" s="30"/>
+      <c r="Z17" s="30"/>
+      <c r="AA17" s="30"/>
+      <c r="AB17" s="30"/>
+      <c r="AC17" s="30"/>
+      <c r="AD17" s="30"/>
+      <c r="AE17" s="30"/>
+      <c r="AF17" s="30"/>
+      <c r="AG17" s="30"/>
       <c r="AW17" s="13" t="s">
         <v>92</v>
       </c>
@@ -2306,40 +2303,40 @@
       <c r="BQ17" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="BR17" s="23" t="s">
+      <c r="BR17" s="25" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="18" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B18" s="24"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="16"/>
-      <c r="O18" s="16"/>
-      <c r="P18" s="16"/>
-      <c r="Q18" s="16"/>
-      <c r="R18" s="16"/>
-      <c r="T18" s="16"/>
-      <c r="U18" s="16"/>
-      <c r="V18" s="16"/>
-      <c r="W18" s="16"/>
-      <c r="X18" s="16"/>
-      <c r="Y18" s="16"/>
-      <c r="Z18" s="16"/>
-      <c r="AA18" s="16"/>
-      <c r="AB18" s="16"/>
-      <c r="AC18" s="16"/>
-      <c r="AD18" s="16"/>
-      <c r="AE18" s="16"/>
-      <c r="AF18" s="16"/>
-      <c r="AG18" s="16"/>
+      <c r="B18" s="31"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="30"/>
+      <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
+      <c r="M18" s="30"/>
+      <c r="N18" s="30"/>
+      <c r="O18" s="30"/>
+      <c r="P18" s="30"/>
+      <c r="Q18" s="30"/>
+      <c r="R18" s="30"/>
+      <c r="T18" s="30"/>
+      <c r="U18" s="30"/>
+      <c r="V18" s="30"/>
+      <c r="W18" s="30"/>
+      <c r="X18" s="30"/>
+      <c r="Y18" s="30"/>
+      <c r="Z18" s="30"/>
+      <c r="AA18" s="30"/>
+      <c r="AB18" s="30"/>
+      <c r="AC18" s="30"/>
+      <c r="AD18" s="30"/>
+      <c r="AE18" s="30"/>
+      <c r="AF18" s="30"/>
+      <c r="AG18" s="30"/>
       <c r="AW18" s="13" t="s">
         <v>100</v>
       </c>
@@ -2377,38 +2374,38 @@
       <c r="BQ18" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="BR18" s="24"/>
+      <c r="BR18" s="31"/>
     </row>
     <row r="19" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B19" s="24"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="16"/>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="16"/>
-      <c r="O19" s="16"/>
-      <c r="P19" s="16"/>
-      <c r="Q19" s="16"/>
-      <c r="R19" s="16"/>
-      <c r="T19" s="16"/>
-      <c r="U19" s="16"/>
-      <c r="V19" s="16"/>
-      <c r="W19" s="16"/>
-      <c r="X19" s="16"/>
-      <c r="Y19" s="16"/>
-      <c r="Z19" s="16"/>
-      <c r="AA19" s="16"/>
-      <c r="AB19" s="16"/>
-      <c r="AC19" s="16"/>
-      <c r="AD19" s="16"/>
-      <c r="AE19" s="16"/>
-      <c r="AF19" s="16"/>
-      <c r="AG19" s="16"/>
+      <c r="B19" s="31"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="30"/>
+      <c r="J19" s="30"/>
+      <c r="K19" s="30"/>
+      <c r="L19" s="30"/>
+      <c r="M19" s="30"/>
+      <c r="N19" s="30"/>
+      <c r="O19" s="30"/>
+      <c r="P19" s="30"/>
+      <c r="Q19" s="30"/>
+      <c r="R19" s="30"/>
+      <c r="T19" s="30"/>
+      <c r="U19" s="30"/>
+      <c r="V19" s="30"/>
+      <c r="W19" s="30"/>
+      <c r="X19" s="30"/>
+      <c r="Y19" s="30"/>
+      <c r="Z19" s="30"/>
+      <c r="AA19" s="30"/>
+      <c r="AB19" s="30"/>
+      <c r="AC19" s="30"/>
+      <c r="AD19" s="30"/>
+      <c r="AE19" s="30"/>
+      <c r="AF19" s="30"/>
+      <c r="AG19" s="30"/>
       <c r="AW19" s="13" t="s">
         <v>108</v>
       </c>
@@ -2446,38 +2443,38 @@
       <c r="BQ19" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="BR19" s="24"/>
+      <c r="BR19" s="31"/>
     </row>
     <row r="20" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B20" s="24"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="16"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="16"/>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="16"/>
-      <c r="O20" s="16"/>
-      <c r="P20" s="16"/>
-      <c r="Q20" s="16"/>
-      <c r="R20" s="16"/>
-      <c r="T20" s="16"/>
-      <c r="U20" s="16"/>
-      <c r="V20" s="16"/>
-      <c r="W20" s="16"/>
-      <c r="X20" s="16"/>
-      <c r="Y20" s="16"/>
-      <c r="Z20" s="16"/>
-      <c r="AA20" s="16"/>
-      <c r="AB20" s="16"/>
-      <c r="AC20" s="16"/>
-      <c r="AD20" s="16"/>
-      <c r="AE20" s="16"/>
-      <c r="AF20" s="16"/>
-      <c r="AG20" s="16"/>
+      <c r="B20" s="31"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="30"/>
+      <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
+      <c r="M20" s="30"/>
+      <c r="N20" s="30"/>
+      <c r="O20" s="30"/>
+      <c r="P20" s="30"/>
+      <c r="Q20" s="30"/>
+      <c r="R20" s="30"/>
+      <c r="T20" s="30"/>
+      <c r="U20" s="30"/>
+      <c r="V20" s="30"/>
+      <c r="W20" s="30"/>
+      <c r="X20" s="30"/>
+      <c r="Y20" s="30"/>
+      <c r="Z20" s="30"/>
+      <c r="AA20" s="30"/>
+      <c r="AB20" s="30"/>
+      <c r="AC20" s="30"/>
+      <c r="AD20" s="30"/>
+      <c r="AE20" s="30"/>
+      <c r="AF20" s="30"/>
+      <c r="AG20" s="30"/>
       <c r="AW20" s="13" t="s">
         <v>116</v>
       </c>
@@ -2515,10 +2512,10 @@
       <c r="BQ20" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="BR20" s="24"/>
+      <c r="BR20" s="31"/>
     </row>
     <row r="21" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B21" s="24"/>
+      <c r="B21" s="31"/>
       <c r="AW21" s="13" t="s">
         <v>124</v>
       </c>
@@ -2556,10 +2553,10 @@
       <c r="BQ21" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="BR21" s="24"/>
+      <c r="BR21" s="31"/>
     </row>
     <row r="22" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B22" s="24"/>
+      <c r="B22" s="31"/>
       <c r="AW22" s="13" t="s">
         <v>132</v>
       </c>
@@ -2597,10 +2594,10 @@
       <c r="BQ22" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="BR22" s="24"/>
+      <c r="BR22" s="31"/>
     </row>
     <row r="23" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B23" s="24"/>
+      <c r="B23" s="31"/>
       <c r="AW23" s="13" t="s">
         <v>140</v>
       </c>
@@ -2638,10 +2635,10 @@
       <c r="BQ23" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="BR23" s="24"/>
+      <c r="BR23" s="31"/>
     </row>
     <row r="24" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B24" s="24"/>
+      <c r="B24" s="31"/>
       <c r="AW24" s="13" t="s">
         <v>148</v>
       </c>
@@ -2679,27 +2676,27 @@
       <c r="BQ24" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="BR24" s="24"/>
+      <c r="BR24" s="31"/>
     </row>
     <row r="25" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B25" s="24"/>
+      <c r="B25" s="31"/>
       <c r="AW25" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="AX25" s="15"/>
+      <c r="AY25" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="AZ25" s="28"/>
+      <c r="BA25" s="28"/>
+      <c r="BB25" s="29"/>
+      <c r="BC25" s="14" t="s">
         <v>219</v>
-      </c>
-      <c r="AX25" s="15"/>
-      <c r="AY25" s="33" t="s">
-        <v>156</v>
-      </c>
-      <c r="AZ25" s="34"/>
-      <c r="BA25" s="34"/>
-      <c r="BB25" s="35"/>
-      <c r="BC25" s="14" t="s">
-        <v>220</v>
       </c>
       <c r="BD25" s="14"/>
       <c r="BE25" s="15"/>
       <c r="BF25" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="BG25" s="14"/>
       <c r="BH25" s="14"/>
@@ -2710,7 +2707,7 @@
         <v>157</v>
       </c>
       <c r="BM25" s="13" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="BN25" s="14"/>
       <c r="BO25" s="15"/>
@@ -2720,42 +2717,42 @@
       <c r="BQ25" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="BR25" s="24"/>
+      <c r="BR25" s="31"/>
     </row>
     <row r="26" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B26" s="24"/>
-      <c r="E26" s="16" t="s">
-        <v>228</v>
-      </c>
-      <c r="F26" s="16"/>
-      <c r="G26" s="16"/>
-      <c r="H26" s="16"/>
-      <c r="I26" s="16"/>
-      <c r="J26" s="16"/>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
-      <c r="N26" s="16"/>
-      <c r="O26" s="16"/>
-      <c r="P26" s="16"/>
-      <c r="Q26" s="16"/>
-      <c r="R26" s="16"/>
-      <c r="T26" s="16" t="s">
-        <v>171</v>
-      </c>
-      <c r="U26" s="16"/>
-      <c r="V26" s="16"/>
-      <c r="W26" s="16"/>
-      <c r="X26" s="16"/>
-      <c r="Y26" s="16"/>
-      <c r="Z26" s="16"/>
-      <c r="AA26" s="16"/>
-      <c r="AB26" s="16"/>
-      <c r="AC26" s="16"/>
-      <c r="AD26" s="16"/>
-      <c r="AE26" s="16"/>
-      <c r="AF26" s="16"/>
-      <c r="AG26" s="16"/>
+      <c r="B26" s="31"/>
+      <c r="E26" s="30" t="s">
+        <v>227</v>
+      </c>
+      <c r="F26" s="30"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="30"/>
+      <c r="I26" s="30"/>
+      <c r="J26" s="30"/>
+      <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
+      <c r="M26" s="30"/>
+      <c r="N26" s="30"/>
+      <c r="O26" s="30"/>
+      <c r="P26" s="30"/>
+      <c r="Q26" s="30"/>
+      <c r="R26" s="30"/>
+      <c r="T26" s="30" t="s">
+        <v>170</v>
+      </c>
+      <c r="U26" s="30"/>
+      <c r="V26" s="30"/>
+      <c r="W26" s="30"/>
+      <c r="X26" s="30"/>
+      <c r="Y26" s="30"/>
+      <c r="Z26" s="30"/>
+      <c r="AA26" s="30"/>
+      <c r="AB26" s="30"/>
+      <c r="AC26" s="30"/>
+      <c r="AD26" s="30"/>
+      <c r="AE26" s="30"/>
+      <c r="AF26" s="30"/>
+      <c r="AG26" s="30"/>
       <c r="AW26" s="13" t="s">
         <v>160</v>
       </c>
@@ -2793,71 +2790,71 @@
       <c r="BQ26" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="BR26" s="24"/>
+      <c r="BR26" s="31"/>
     </row>
     <row r="27" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B27" s="24"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="16"/>
-      <c r="H27" s="16"/>
-      <c r="I27" s="16"/>
-      <c r="J27" s="16"/>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="16"/>
-      <c r="O27" s="16"/>
-      <c r="P27" s="16"/>
-      <c r="Q27" s="16"/>
-      <c r="R27" s="16"/>
-      <c r="T27" s="16"/>
-      <c r="U27" s="16"/>
-      <c r="V27" s="16"/>
-      <c r="W27" s="16"/>
-      <c r="X27" s="16"/>
-      <c r="Y27" s="16"/>
-      <c r="Z27" s="16"/>
-      <c r="AA27" s="16"/>
-      <c r="AB27" s="16"/>
-      <c r="AC27" s="16"/>
-      <c r="AD27" s="16"/>
-      <c r="AE27" s="16"/>
-      <c r="AF27" s="16"/>
-      <c r="AG27" s="16"/>
+      <c r="B27" s="31"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="30"/>
+      <c r="I27" s="30"/>
+      <c r="J27" s="30"/>
+      <c r="K27" s="30"/>
+      <c r="L27" s="30"/>
+      <c r="M27" s="30"/>
+      <c r="N27" s="30"/>
+      <c r="O27" s="30"/>
+      <c r="P27" s="30"/>
+      <c r="Q27" s="30"/>
+      <c r="R27" s="30"/>
+      <c r="T27" s="30"/>
+      <c r="U27" s="30"/>
+      <c r="V27" s="30"/>
+      <c r="W27" s="30"/>
+      <c r="X27" s="30"/>
+      <c r="Y27" s="30"/>
+      <c r="Z27" s="30"/>
+      <c r="AA27" s="30"/>
+      <c r="AB27" s="30"/>
+      <c r="AC27" s="30"/>
+      <c r="AD27" s="30"/>
+      <c r="AE27" s="30"/>
+      <c r="AF27" s="30"/>
+      <c r="AG27" s="30"/>
       <c r="BQ27" s="6"/>
-      <c r="BR27" s="24"/>
+      <c r="BR27" s="31"/>
     </row>
     <row r="28" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B28" s="24"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="16"/>
-      <c r="I28" s="16"/>
-      <c r="J28" s="16"/>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="16"/>
-      <c r="O28" s="16"/>
-      <c r="P28" s="16"/>
-      <c r="Q28" s="16"/>
-      <c r="R28" s="16"/>
-      <c r="T28" s="16"/>
-      <c r="U28" s="16"/>
-      <c r="V28" s="16"/>
-      <c r="W28" s="16"/>
-      <c r="X28" s="16"/>
-      <c r="Y28" s="16"/>
-      <c r="Z28" s="16"/>
-      <c r="AA28" s="16"/>
-      <c r="AB28" s="16"/>
-      <c r="AC28" s="16"/>
-      <c r="AD28" s="16"/>
-      <c r="AE28" s="16"/>
-      <c r="AF28" s="16"/>
-      <c r="AG28" s="16"/>
+      <c r="B28" s="31"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="30"/>
+      <c r="I28" s="30"/>
+      <c r="J28" s="30"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
+      <c r="M28" s="30"/>
+      <c r="N28" s="30"/>
+      <c r="O28" s="30"/>
+      <c r="P28" s="30"/>
+      <c r="Q28" s="30"/>
+      <c r="R28" s="30"/>
+      <c r="T28" s="30"/>
+      <c r="U28" s="30"/>
+      <c r="V28" s="30"/>
+      <c r="W28" s="30"/>
+      <c r="X28" s="30"/>
+      <c r="Y28" s="30"/>
+      <c r="Z28" s="30"/>
+      <c r="AA28" s="30"/>
+      <c r="AB28" s="30"/>
+      <c r="AC28" s="30"/>
+      <c r="AD28" s="30"/>
+      <c r="AE28" s="30"/>
+      <c r="AF28" s="30"/>
+      <c r="AG28" s="30"/>
       <c r="AI28" s="3"/>
       <c r="AV28" s="6"/>
       <c r="AW28" s="9"/>
@@ -2881,369 +2878,367 @@
       <c r="BO28" s="9"/>
       <c r="BP28" s="9"/>
       <c r="BQ28" s="9"/>
-      <c r="BR28" s="24"/>
+      <c r="BR28" s="31"/>
     </row>
     <row r="29" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B29" s="25"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-      <c r="H29" s="16"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="16"/>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="16"/>
-      <c r="O29" s="16"/>
-      <c r="P29" s="16"/>
-      <c r="Q29" s="16"/>
-      <c r="R29" s="16"/>
-      <c r="T29" s="16"/>
-      <c r="U29" s="16"/>
-      <c r="V29" s="16"/>
-      <c r="W29" s="16"/>
-      <c r="X29" s="16"/>
-      <c r="Y29" s="16"/>
-      <c r="Z29" s="16"/>
-      <c r="AA29" s="16"/>
-      <c r="AB29" s="16"/>
-      <c r="AC29" s="16"/>
-      <c r="AD29" s="16"/>
-      <c r="AE29" s="16"/>
-      <c r="AF29" s="16"/>
-      <c r="AG29" s="16"/>
+      <c r="B29" s="26"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="30"/>
+      <c r="K29" s="30"/>
+      <c r="L29" s="30"/>
+      <c r="M29" s="30"/>
+      <c r="N29" s="30"/>
+      <c r="O29" s="30"/>
+      <c r="P29" s="30"/>
+      <c r="Q29" s="30"/>
+      <c r="R29" s="30"/>
+      <c r="T29" s="30"/>
+      <c r="U29" s="30"/>
+      <c r="V29" s="30"/>
+      <c r="W29" s="30"/>
+      <c r="X29" s="30"/>
+      <c r="Y29" s="30"/>
+      <c r="Z29" s="30"/>
+      <c r="AA29" s="30"/>
+      <c r="AB29" s="30"/>
+      <c r="AC29" s="30"/>
+      <c r="AD29" s="30"/>
+      <c r="AE29" s="30"/>
+      <c r="AF29" s="30"/>
+      <c r="AG29" s="30"/>
       <c r="BQ29" s="6"/>
-      <c r="BR29" s="25"/>
+      <c r="BR29" s="26"/>
     </row>
     <row r="30" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B30" s="23" t="s">
+      <c r="B30" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="BR30" s="23" t="s">
+      <c r="BR30" s="25" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="31" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B31" s="24"/>
-      <c r="AW31" s="17" t="s">
+      <c r="B31" s="31"/>
+      <c r="AW31" s="16"/>
+      <c r="AX31" s="17"/>
+      <c r="AY31" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="AX31" s="18"/>
-      <c r="AY31" s="18" t="s">
-        <v>170</v>
-      </c>
-      <c r="AZ31" s="18"/>
-      <c r="BA31" s="18"/>
-      <c r="BB31" s="18"/>
-      <c r="BC31" s="18"/>
-      <c r="BD31" s="18"/>
-      <c r="BE31" s="18"/>
-      <c r="BF31" s="18"/>
-      <c r="BG31" s="18"/>
-      <c r="BH31" s="18"/>
-      <c r="BI31" s="18"/>
-      <c r="BJ31" s="18"/>
-      <c r="BK31" s="18"/>
-      <c r="BL31" s="18"/>
-      <c r="BM31" s="18"/>
-      <c r="BN31" s="18"/>
-      <c r="BO31" s="18"/>
-      <c r="BP31" s="18"/>
-      <c r="BQ31" s="19"/>
-      <c r="BR31" s="24"/>
+      <c r="AZ31" s="17"/>
+      <c r="BA31" s="17"/>
+      <c r="BB31" s="17"/>
+      <c r="BC31" s="17"/>
+      <c r="BD31" s="17"/>
+      <c r="BE31" s="17"/>
+      <c r="BF31" s="17"/>
+      <c r="BG31" s="17"/>
+      <c r="BH31" s="17"/>
+      <c r="BI31" s="17"/>
+      <c r="BJ31" s="17"/>
+      <c r="BK31" s="17"/>
+      <c r="BL31" s="17"/>
+      <c r="BM31" s="17"/>
+      <c r="BN31" s="17"/>
+      <c r="BO31" s="17"/>
+      <c r="BP31" s="17"/>
+      <c r="BQ31" s="18"/>
+      <c r="BR31" s="31"/>
     </row>
     <row r="32" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B32" s="24"/>
+      <c r="B32" s="31"/>
       <c r="E32" s="3"/>
       <c r="AA32" s="3"/>
-      <c r="AW32" s="26"/>
-      <c r="AX32" s="27"/>
-      <c r="AY32" s="27"/>
-      <c r="AZ32" s="27"/>
-      <c r="BA32" s="27"/>
-      <c r="BB32" s="27"/>
-      <c r="BC32" s="27"/>
-      <c r="BD32" s="27"/>
-      <c r="BE32" s="27"/>
-      <c r="BF32" s="27"/>
-      <c r="BG32" s="27"/>
-      <c r="BH32" s="27"/>
-      <c r="BI32" s="27"/>
-      <c r="BJ32" s="27"/>
-      <c r="BK32" s="27"/>
-      <c r="BL32" s="27"/>
-      <c r="BM32" s="27"/>
-      <c r="BN32" s="27"/>
-      <c r="BO32" s="27"/>
-      <c r="BP32" s="27"/>
-      <c r="BQ32" s="28"/>
-      <c r="BR32" s="24"/>
+      <c r="AW32" s="22"/>
+      <c r="AX32" s="23"/>
+      <c r="AY32" s="23"/>
+      <c r="AZ32" s="23"/>
+      <c r="BA32" s="23"/>
+      <c r="BB32" s="23"/>
+      <c r="BC32" s="23"/>
+      <c r="BD32" s="23"/>
+      <c r="BE32" s="23"/>
+      <c r="BF32" s="23"/>
+      <c r="BG32" s="23"/>
+      <c r="BH32" s="23"/>
+      <c r="BI32" s="23"/>
+      <c r="BJ32" s="23"/>
+      <c r="BK32" s="23"/>
+      <c r="BL32" s="23"/>
+      <c r="BM32" s="23"/>
+      <c r="BN32" s="23"/>
+      <c r="BO32" s="23"/>
+      <c r="BP32" s="23"/>
+      <c r="BQ32" s="24"/>
+      <c r="BR32" s="31"/>
     </row>
     <row r="33" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B33" s="24"/>
-      <c r="AW33" s="26"/>
-      <c r="AX33" s="27"/>
-      <c r="AY33" s="27"/>
-      <c r="AZ33" s="27"/>
-      <c r="BA33" s="27"/>
-      <c r="BB33" s="27"/>
-      <c r="BC33" s="27"/>
-      <c r="BD33" s="27"/>
-      <c r="BE33" s="27"/>
-      <c r="BF33" s="27"/>
-      <c r="BG33" s="27"/>
-      <c r="BH33" s="27"/>
-      <c r="BI33" s="27"/>
-      <c r="BJ33" s="27"/>
-      <c r="BK33" s="27"/>
-      <c r="BL33" s="27"/>
-      <c r="BM33" s="27"/>
-      <c r="BN33" s="27"/>
-      <c r="BO33" s="27"/>
-      <c r="BP33" s="27"/>
-      <c r="BQ33" s="28"/>
-      <c r="BR33" s="24"/>
+      <c r="B33" s="31"/>
+      <c r="AW33" s="22"/>
+      <c r="AX33" s="23"/>
+      <c r="AY33" s="23"/>
+      <c r="AZ33" s="23"/>
+      <c r="BA33" s="23"/>
+      <c r="BB33" s="23"/>
+      <c r="BC33" s="23"/>
+      <c r="BD33" s="23"/>
+      <c r="BE33" s="23"/>
+      <c r="BF33" s="23"/>
+      <c r="BG33" s="23"/>
+      <c r="BH33" s="23"/>
+      <c r="BI33" s="23"/>
+      <c r="BJ33" s="23"/>
+      <c r="BK33" s="23"/>
+      <c r="BL33" s="23"/>
+      <c r="BM33" s="23"/>
+      <c r="BN33" s="23"/>
+      <c r="BO33" s="23"/>
+      <c r="BP33" s="23"/>
+      <c r="BQ33" s="24"/>
+      <c r="BR33" s="31"/>
     </row>
     <row r="34" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B34" s="24"/>
-      <c r="AW34" s="26"/>
-      <c r="AX34" s="27"/>
-      <c r="AY34" s="27"/>
-      <c r="AZ34" s="27"/>
-      <c r="BA34" s="27"/>
-      <c r="BB34" s="27"/>
-      <c r="BC34" s="27"/>
-      <c r="BD34" s="27"/>
-      <c r="BE34" s="27"/>
-      <c r="BF34" s="27"/>
-      <c r="BG34" s="27"/>
-      <c r="BH34" s="27"/>
-      <c r="BI34" s="27"/>
-      <c r="BJ34" s="27"/>
-      <c r="BK34" s="27"/>
-      <c r="BL34" s="27"/>
-      <c r="BM34" s="27"/>
-      <c r="BN34" s="27"/>
-      <c r="BO34" s="27"/>
-      <c r="BP34" s="27"/>
-      <c r="BQ34" s="28"/>
-      <c r="BR34" s="24"/>
+      <c r="B34" s="31"/>
+      <c r="AW34" s="22"/>
+      <c r="AX34" s="23"/>
+      <c r="AY34" s="23"/>
+      <c r="AZ34" s="23"/>
+      <c r="BA34" s="23"/>
+      <c r="BB34" s="23"/>
+      <c r="BC34" s="23"/>
+      <c r="BD34" s="23"/>
+      <c r="BE34" s="23"/>
+      <c r="BF34" s="23"/>
+      <c r="BG34" s="23"/>
+      <c r="BH34" s="23"/>
+      <c r="BI34" s="23"/>
+      <c r="BJ34" s="23"/>
+      <c r="BK34" s="23"/>
+      <c r="BL34" s="23"/>
+      <c r="BM34" s="23"/>
+      <c r="BN34" s="23"/>
+      <c r="BO34" s="23"/>
+      <c r="BP34" s="23"/>
+      <c r="BQ34" s="24"/>
+      <c r="BR34" s="31"/>
     </row>
     <row r="35" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B35" s="24"/>
-      <c r="E35" s="16" t="s">
-        <v>229</v>
-      </c>
-      <c r="F35" s="16"/>
-      <c r="G35" s="16"/>
-      <c r="H35" s="16"/>
-      <c r="I35" s="16"/>
-      <c r="J35" s="16"/>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="16"/>
-      <c r="O35" s="16"/>
-      <c r="P35" s="16"/>
-      <c r="Q35" s="16"/>
-      <c r="R35" s="16"/>
-      <c r="T35" s="16" t="s">
+      <c r="B35" s="31"/>
+      <c r="E35" s="30" t="s">
+        <v>228</v>
+      </c>
+      <c r="F35" s="30"/>
+      <c r="G35" s="30"/>
+      <c r="H35" s="30"/>
+      <c r="I35" s="30"/>
+      <c r="J35" s="30"/>
+      <c r="K35" s="30"/>
+      <c r="L35" s="30"/>
+      <c r="M35" s="30"/>
+      <c r="N35" s="30"/>
+      <c r="O35" s="30"/>
+      <c r="P35" s="30"/>
+      <c r="Q35" s="30"/>
+      <c r="R35" s="30"/>
+      <c r="T35" s="30" t="s">
+        <v>171</v>
+      </c>
+      <c r="U35" s="30"/>
+      <c r="V35" s="30"/>
+      <c r="W35" s="30"/>
+      <c r="X35" s="30"/>
+      <c r="Y35" s="30"/>
+      <c r="Z35" s="30"/>
+      <c r="AA35" s="30"/>
+      <c r="AB35" s="30"/>
+      <c r="AC35" s="30"/>
+      <c r="AD35" s="30"/>
+      <c r="AE35" s="30"/>
+      <c r="AF35" s="30"/>
+      <c r="AG35" s="30"/>
+      <c r="AW35" s="22"/>
+      <c r="AX35" s="23"/>
+      <c r="AY35" s="23"/>
+      <c r="AZ35" s="23"/>
+      <c r="BA35" s="23"/>
+      <c r="BB35" s="23"/>
+      <c r="BC35" s="23"/>
+      <c r="BD35" s="23"/>
+      <c r="BE35" s="23"/>
+      <c r="BF35" s="23"/>
+      <c r="BG35" s="23"/>
+      <c r="BH35" s="23"/>
+      <c r="BI35" s="23"/>
+      <c r="BJ35" s="23"/>
+      <c r="BK35" s="23"/>
+      <c r="BL35" s="23"/>
+      <c r="BM35" s="23"/>
+      <c r="BN35" s="23"/>
+      <c r="BO35" s="23"/>
+      <c r="BP35" s="23"/>
+      <c r="BQ35" s="24"/>
+      <c r="BR35" s="31"/>
+    </row>
+    <row r="36" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B36" s="31"/>
+      <c r="E36" s="30"/>
+      <c r="F36" s="30"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="30"/>
+      <c r="I36" s="30"/>
+      <c r="J36" s="30"/>
+      <c r="K36" s="30"/>
+      <c r="L36" s="30"/>
+      <c r="M36" s="30"/>
+      <c r="N36" s="30"/>
+      <c r="O36" s="30"/>
+      <c r="P36" s="30"/>
+      <c r="Q36" s="30"/>
+      <c r="R36" s="30"/>
+      <c r="T36" s="30"/>
+      <c r="U36" s="30"/>
+      <c r="V36" s="30"/>
+      <c r="W36" s="30"/>
+      <c r="X36" s="30"/>
+      <c r="Y36" s="30"/>
+      <c r="Z36" s="30"/>
+      <c r="AA36" s="30"/>
+      <c r="AB36" s="30"/>
+      <c r="AC36" s="30"/>
+      <c r="AD36" s="30"/>
+      <c r="AE36" s="30"/>
+      <c r="AF36" s="30"/>
+      <c r="AG36" s="30"/>
+      <c r="AW36" s="19"/>
+      <c r="AX36" s="20"/>
+      <c r="AY36" s="20"/>
+      <c r="AZ36" s="20"/>
+      <c r="BA36" s="20"/>
+      <c r="BB36" s="20"/>
+      <c r="BC36" s="20"/>
+      <c r="BD36" s="20"/>
+      <c r="BE36" s="20"/>
+      <c r="BF36" s="20"/>
+      <c r="BG36" s="20"/>
+      <c r="BH36" s="20"/>
+      <c r="BI36" s="20"/>
+      <c r="BJ36" s="20"/>
+      <c r="BK36" s="20"/>
+      <c r="BL36" s="20"/>
+      <c r="BM36" s="20"/>
+      <c r="BN36" s="20"/>
+      <c r="BO36" s="20"/>
+      <c r="BP36" s="20"/>
+      <c r="BQ36" s="21"/>
+      <c r="BR36" s="31"/>
+    </row>
+    <row r="37" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B37" s="31"/>
+      <c r="E37" s="30"/>
+      <c r="F37" s="30"/>
+      <c r="G37" s="30"/>
+      <c r="H37" s="30"/>
+      <c r="I37" s="30"/>
+      <c r="J37" s="30"/>
+      <c r="K37" s="30"/>
+      <c r="L37" s="30"/>
+      <c r="M37" s="30"/>
+      <c r="N37" s="30"/>
+      <c r="O37" s="30"/>
+      <c r="P37" s="30"/>
+      <c r="Q37" s="30"/>
+      <c r="R37" s="30"/>
+      <c r="T37" s="30"/>
+      <c r="U37" s="30"/>
+      <c r="V37" s="30"/>
+      <c r="W37" s="30"/>
+      <c r="X37" s="30"/>
+      <c r="Y37" s="30"/>
+      <c r="Z37" s="30"/>
+      <c r="AA37" s="30"/>
+      <c r="AB37" s="30"/>
+      <c r="AC37" s="30"/>
+      <c r="AD37" s="30"/>
+      <c r="AE37" s="30"/>
+      <c r="AF37" s="30"/>
+      <c r="AG37" s="30"/>
+      <c r="BR37" s="31"/>
+    </row>
+    <row r="38" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B38" s="31"/>
+      <c r="E38" s="30"/>
+      <c r="F38" s="30"/>
+      <c r="G38" s="30"/>
+      <c r="H38" s="30"/>
+      <c r="I38" s="30"/>
+      <c r="J38" s="30"/>
+      <c r="K38" s="30"/>
+      <c r="L38" s="30"/>
+      <c r="M38" s="30"/>
+      <c r="N38" s="30"/>
+      <c r="O38" s="30"/>
+      <c r="P38" s="30"/>
+      <c r="Q38" s="30"/>
+      <c r="R38" s="30"/>
+      <c r="T38" s="30"/>
+      <c r="U38" s="30"/>
+      <c r="V38" s="30"/>
+      <c r="W38" s="30"/>
+      <c r="X38" s="30"/>
+      <c r="Y38" s="30"/>
+      <c r="Z38" s="30"/>
+      <c r="AA38" s="30"/>
+      <c r="AB38" s="30"/>
+      <c r="AC38" s="30"/>
+      <c r="AD38" s="30"/>
+      <c r="AE38" s="30"/>
+      <c r="AF38" s="30"/>
+      <c r="AG38" s="30"/>
+      <c r="BR38" s="31"/>
+    </row>
+    <row r="39" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B39" s="31"/>
+      <c r="E39" s="30"/>
+      <c r="F39" s="30"/>
+      <c r="G39" s="30"/>
+      <c r="H39" s="30"/>
+      <c r="I39" s="30"/>
+      <c r="J39" s="30"/>
+      <c r="K39" s="30"/>
+      <c r="L39" s="30"/>
+      <c r="M39" s="30"/>
+      <c r="N39" s="30"/>
+      <c r="O39" s="30"/>
+      <c r="P39" s="30"/>
+      <c r="Q39" s="30"/>
+      <c r="R39" s="30"/>
+      <c r="T39" s="30"/>
+      <c r="U39" s="30"/>
+      <c r="V39" s="30"/>
+      <c r="W39" s="30"/>
+      <c r="X39" s="30"/>
+      <c r="Y39" s="30"/>
+      <c r="Z39" s="30"/>
+      <c r="AA39" s="30"/>
+      <c r="AB39" s="30"/>
+      <c r="AC39" s="30"/>
+      <c r="AD39" s="30"/>
+      <c r="AE39" s="30"/>
+      <c r="AF39" s="30"/>
+      <c r="AG39" s="30"/>
+      <c r="AW39" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="U35" s="16"/>
-      <c r="V35" s="16"/>
-      <c r="W35" s="16"/>
-      <c r="X35" s="16"/>
-      <c r="Y35" s="16"/>
-      <c r="Z35" s="16"/>
-      <c r="AA35" s="16"/>
-      <c r="AB35" s="16"/>
-      <c r="AC35" s="16"/>
-      <c r="AD35" s="16"/>
-      <c r="AE35" s="16"/>
-      <c r="AF35" s="16"/>
-      <c r="AG35" s="16"/>
-      <c r="AW35" s="26"/>
-      <c r="AX35" s="27"/>
-      <c r="AY35" s="27"/>
-      <c r="AZ35" s="27"/>
-      <c r="BA35" s="27"/>
-      <c r="BB35" s="27"/>
-      <c r="BC35" s="27"/>
-      <c r="BD35" s="27"/>
-      <c r="BE35" s="27"/>
-      <c r="BF35" s="27"/>
-      <c r="BG35" s="27"/>
-      <c r="BH35" s="27"/>
-      <c r="BI35" s="27"/>
-      <c r="BJ35" s="27"/>
-      <c r="BK35" s="27"/>
-      <c r="BL35" s="27"/>
-      <c r="BM35" s="27"/>
-      <c r="BN35" s="27"/>
-      <c r="BO35" s="27"/>
-      <c r="BP35" s="27"/>
-      <c r="BQ35" s="28"/>
-      <c r="BR35" s="24"/>
-    </row>
-    <row r="36" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B36" s="24"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="16"/>
-      <c r="G36" s="16"/>
-      <c r="H36" s="16"/>
-      <c r="I36" s="16"/>
-      <c r="J36" s="16"/>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16"/>
-      <c r="M36" s="16"/>
-      <c r="N36" s="16"/>
-      <c r="O36" s="16"/>
-      <c r="P36" s="16"/>
-      <c r="Q36" s="16"/>
-      <c r="R36" s="16"/>
-      <c r="T36" s="16"/>
-      <c r="U36" s="16"/>
-      <c r="V36" s="16"/>
-      <c r="W36" s="16"/>
-      <c r="X36" s="16"/>
-      <c r="Y36" s="16"/>
-      <c r="Z36" s="16"/>
-      <c r="AA36" s="16"/>
-      <c r="AB36" s="16"/>
-      <c r="AC36" s="16"/>
-      <c r="AD36" s="16"/>
-      <c r="AE36" s="16"/>
-      <c r="AF36" s="16"/>
-      <c r="AG36" s="16"/>
-      <c r="AW36" s="20"/>
-      <c r="AX36" s="21"/>
-      <c r="AY36" s="21"/>
-      <c r="AZ36" s="21"/>
-      <c r="BA36" s="21"/>
-      <c r="BB36" s="21"/>
-      <c r="BC36" s="21"/>
-      <c r="BD36" s="21"/>
-      <c r="BE36" s="21"/>
-      <c r="BF36" s="21"/>
-      <c r="BG36" s="21"/>
-      <c r="BH36" s="21"/>
-      <c r="BI36" s="21"/>
-      <c r="BJ36" s="21"/>
-      <c r="BK36" s="21"/>
-      <c r="BL36" s="21"/>
-      <c r="BM36" s="21"/>
-      <c r="BN36" s="21"/>
-      <c r="BO36" s="21"/>
-      <c r="BP36" s="21"/>
-      <c r="BQ36" s="22"/>
-      <c r="BR36" s="24"/>
-    </row>
-    <row r="37" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B37" s="24"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
-      <c r="G37" s="16"/>
-      <c r="H37" s="16"/>
-      <c r="I37" s="16"/>
-      <c r="J37" s="16"/>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="16"/>
-      <c r="N37" s="16"/>
-      <c r="O37" s="16"/>
-      <c r="P37" s="16"/>
-      <c r="Q37" s="16"/>
-      <c r="R37" s="16"/>
-      <c r="T37" s="16"/>
-      <c r="U37" s="16"/>
-      <c r="V37" s="16"/>
-      <c r="W37" s="16"/>
-      <c r="X37" s="16"/>
-      <c r="Y37" s="16"/>
-      <c r="Z37" s="16"/>
-      <c r="AA37" s="16"/>
-      <c r="AB37" s="16"/>
-      <c r="AC37" s="16"/>
-      <c r="AD37" s="16"/>
-      <c r="AE37" s="16"/>
-      <c r="AF37" s="16"/>
-      <c r="AG37" s="16"/>
-      <c r="BR37" s="24"/>
-    </row>
-    <row r="38" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B38" s="24"/>
-      <c r="E38" s="16"/>
-      <c r="F38" s="16"/>
-      <c r="G38" s="16"/>
-      <c r="H38" s="16"/>
-      <c r="I38" s="16"/>
-      <c r="J38" s="16"/>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
-      <c r="N38" s="16"/>
-      <c r="O38" s="16"/>
-      <c r="P38" s="16"/>
-      <c r="Q38" s="16"/>
-      <c r="R38" s="16"/>
-      <c r="T38" s="16"/>
-      <c r="U38" s="16"/>
-      <c r="V38" s="16"/>
-      <c r="W38" s="16"/>
-      <c r="X38" s="16"/>
-      <c r="Y38" s="16"/>
-      <c r="Z38" s="16"/>
-      <c r="AA38" s="16"/>
-      <c r="AB38" s="16"/>
-      <c r="AC38" s="16"/>
-      <c r="AD38" s="16"/>
-      <c r="AE38" s="16"/>
-      <c r="AF38" s="16"/>
-      <c r="AG38" s="16"/>
-      <c r="BR38" s="24"/>
-    </row>
-    <row r="39" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B39" s="24"/>
-      <c r="E39" s="16"/>
-      <c r="F39" s="16"/>
-      <c r="G39" s="16"/>
-      <c r="H39" s="16"/>
-      <c r="I39" s="16"/>
-      <c r="J39" s="16"/>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="16"/>
-      <c r="O39" s="16"/>
-      <c r="P39" s="16"/>
-      <c r="Q39" s="16"/>
-      <c r="R39" s="16"/>
-      <c r="T39" s="16"/>
-      <c r="U39" s="16"/>
-      <c r="V39" s="16"/>
-      <c r="W39" s="16"/>
-      <c r="X39" s="16"/>
-      <c r="Y39" s="16"/>
-      <c r="Z39" s="16"/>
-      <c r="AA39" s="16"/>
-      <c r="AB39" s="16"/>
-      <c r="AC39" s="16"/>
-      <c r="AD39" s="16"/>
-      <c r="AE39" s="16"/>
-      <c r="AF39" s="16"/>
-      <c r="AG39" s="16"/>
-      <c r="AW39" s="1" t="s">
+      <c r="AX39" s="13" t="s">
         <v>173</v>
-      </c>
-      <c r="AX39" s="13" t="s">
-        <v>174</v>
       </c>
       <c r="AY39" s="14"/>
       <c r="AZ39" s="15"/>
       <c r="BA39" s="13" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="BB39" s="14"/>
       <c r="BC39" s="14"/>
@@ -3253,34 +3248,34 @@
       <c r="BG39" s="14"/>
       <c r="BH39" s="15"/>
       <c r="BI39" s="13" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="BJ39" s="14"/>
       <c r="BK39" s="15"/>
       <c r="BL39" s="13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="BM39" s="14"/>
       <c r="BN39" s="15"/>
       <c r="BO39" s="13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="BP39" s="14"/>
       <c r="BQ39" s="15"/>
-      <c r="BR39" s="24"/>
+      <c r="BR39" s="31"/>
     </row>
     <row r="40" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B40" s="24"/>
+      <c r="B40" s="31"/>
       <c r="AW40" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="AX40" s="13" t="s">
         <v>179</v>
-      </c>
-      <c r="AX40" s="13" t="s">
-        <v>180</v>
       </c>
       <c r="AY40" s="14"/>
       <c r="AZ40" s="15"/>
       <c r="BA40" s="13" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="BB40" s="14"/>
       <c r="BC40" s="14"/>
@@ -3290,34 +3285,34 @@
       <c r="BG40" s="14"/>
       <c r="BH40" s="15"/>
       <c r="BI40" s="13" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="BJ40" s="14"/>
       <c r="BK40" s="15"/>
       <c r="BL40" s="13" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="BM40" s="14"/>
       <c r="BN40" s="15"/>
       <c r="BO40" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="BP40" s="14"/>
       <c r="BQ40" s="15"/>
-      <c r="BR40" s="24"/>
+      <c r="BR40" s="31"/>
     </row>
     <row r="41" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B41" s="24"/>
+      <c r="B41" s="31"/>
       <c r="AW41" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="AX41" s="13" t="s">
         <v>185</v>
-      </c>
-      <c r="AX41" s="13" t="s">
-        <v>186</v>
       </c>
       <c r="AY41" s="14"/>
       <c r="AZ41" s="15"/>
       <c r="BA41" s="13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="BB41" s="14"/>
       <c r="BC41" s="14"/>
@@ -3327,34 +3322,34 @@
       <c r="BG41" s="14"/>
       <c r="BH41" s="15"/>
       <c r="BI41" s="13" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="BJ41" s="14"/>
       <c r="BK41" s="15"/>
       <c r="BL41" s="13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="BM41" s="14"/>
       <c r="BN41" s="15"/>
       <c r="BO41" s="13" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="BP41" s="14"/>
       <c r="BQ41" s="15"/>
-      <c r="BR41" s="24"/>
+      <c r="BR41" s="31"/>
     </row>
     <row r="42" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B42" s="24"/>
+      <c r="B42" s="31"/>
       <c r="AW42" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="AX42" s="13" t="s">
         <v>191</v>
-      </c>
-      <c r="AX42" s="13" t="s">
-        <v>192</v>
       </c>
       <c r="AY42" s="14"/>
       <c r="AZ42" s="15"/>
       <c r="BA42" s="13" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="BB42" s="14"/>
       <c r="BC42" s="14"/>
@@ -3364,90 +3359,90 @@
       <c r="BG42" s="14"/>
       <c r="BH42" s="15"/>
       <c r="BI42" s="13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="BJ42" s="14"/>
       <c r="BK42" s="15"/>
       <c r="BL42" s="13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="BM42" s="14"/>
       <c r="BN42" s="15"/>
       <c r="BO42" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="BP42" s="14"/>
       <c r="BQ42" s="15"/>
-      <c r="BR42" s="24"/>
+      <c r="BR42" s="31"/>
     </row>
     <row r="43" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B43" s="25"/>
-      <c r="AW43" s="23" t="s">
+      <c r="B43" s="26"/>
+      <c r="AW43" s="25" t="s">
+        <v>196</v>
+      </c>
+      <c r="AX43" s="16"/>
+      <c r="AY43" s="17"/>
+      <c r="AZ43" s="18"/>
+      <c r="BA43" s="16"/>
+      <c r="BB43" s="17"/>
+      <c r="BC43" s="17"/>
+      <c r="BD43" s="17"/>
+      <c r="BE43" s="17"/>
+      <c r="BF43" s="17"/>
+      <c r="BG43" s="17"/>
+      <c r="BH43" s="18"/>
+      <c r="BI43" s="16"/>
+      <c r="BJ43" s="17"/>
+      <c r="BK43" s="18"/>
+      <c r="BL43" s="16"/>
+      <c r="BM43" s="17"/>
+      <c r="BN43" s="18"/>
+      <c r="BO43" s="16"/>
+      <c r="BP43" s="17"/>
+      <c r="BQ43" s="18"/>
+      <c r="BR43" s="26"/>
+    </row>
+    <row r="44" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B44" s="25" t="s">
         <v>197</v>
       </c>
-      <c r="AX43" s="17"/>
-      <c r="AY43" s="18"/>
-      <c r="AZ43" s="19"/>
-      <c r="BA43" s="17"/>
-      <c r="BB43" s="18"/>
-      <c r="BC43" s="18"/>
-      <c r="BD43" s="18"/>
-      <c r="BE43" s="18"/>
-      <c r="BF43" s="18"/>
-      <c r="BG43" s="18"/>
-      <c r="BH43" s="19"/>
-      <c r="BI43" s="17"/>
-      <c r="BJ43" s="18"/>
-      <c r="BK43" s="19"/>
-      <c r="BL43" s="17"/>
-      <c r="BM43" s="18"/>
-      <c r="BN43" s="19"/>
-      <c r="BO43" s="17"/>
-      <c r="BP43" s="18"/>
-      <c r="BQ43" s="19"/>
-      <c r="BR43" s="25"/>
-    </row>
-    <row r="44" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B44" s="23" t="s">
+      <c r="AW44" s="26"/>
+      <c r="AX44" s="19"/>
+      <c r="AY44" s="20"/>
+      <c r="AZ44" s="21"/>
+      <c r="BA44" s="19"/>
+      <c r="BB44" s="20"/>
+      <c r="BC44" s="20"/>
+      <c r="BD44" s="20"/>
+      <c r="BE44" s="20"/>
+      <c r="BF44" s="20"/>
+      <c r="BG44" s="20"/>
+      <c r="BH44" s="21"/>
+      <c r="BI44" s="19"/>
+      <c r="BJ44" s="20"/>
+      <c r="BK44" s="21"/>
+      <c r="BL44" s="19"/>
+      <c r="BM44" s="20"/>
+      <c r="BN44" s="21"/>
+      <c r="BO44" s="19"/>
+      <c r="BP44" s="20"/>
+      <c r="BQ44" s="21"/>
+      <c r="BR44" s="25" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="45" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B45" s="31"/>
+      <c r="AW45" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="AW44" s="25"/>
-      <c r="AX44" s="20"/>
-      <c r="AY44" s="21"/>
-      <c r="AZ44" s="22"/>
-      <c r="BA44" s="20"/>
-      <c r="BB44" s="21"/>
-      <c r="BC44" s="21"/>
-      <c r="BD44" s="21"/>
-      <c r="BE44" s="21"/>
-      <c r="BF44" s="21"/>
-      <c r="BG44" s="21"/>
-      <c r="BH44" s="22"/>
-      <c r="BI44" s="20"/>
-      <c r="BJ44" s="21"/>
-      <c r="BK44" s="22"/>
-      <c r="BL44" s="20"/>
-      <c r="BM44" s="21"/>
-      <c r="BN44" s="22"/>
-      <c r="BO44" s="20"/>
-      <c r="BP44" s="21"/>
-      <c r="BQ44" s="22"/>
-      <c r="BR44" s="23" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="45" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B45" s="24"/>
-      <c r="AW45" s="5" t="s">
+      <c r="AX45" s="13" t="s">
         <v>199</v>
-      </c>
-      <c r="AX45" s="13" t="s">
-        <v>200</v>
       </c>
       <c r="AY45" s="14"/>
       <c r="AZ45" s="15"/>
       <c r="BA45" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="BB45" s="14"/>
       <c r="BC45" s="14"/>
@@ -3457,32 +3452,32 @@
       <c r="BG45" s="14"/>
       <c r="BH45" s="15"/>
       <c r="BI45" s="13" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="BJ45" s="14"/>
       <c r="BK45" s="15"/>
       <c r="BL45" s="13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="BM45" s="14"/>
       <c r="BN45" s="15"/>
       <c r="BO45" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="BP45" s="14"/>
       <c r="BQ45" s="15"/>
-      <c r="BR45" s="24"/>
+      <c r="BR45" s="31"/>
     </row>
     <row r="46" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B46" s="24"/>
+      <c r="B46" s="31"/>
       <c r="AW46" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="AX46" s="14"/>
       <c r="AY46" s="14"/>
       <c r="AZ46" s="15"/>
       <c r="BA46" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="BB46" s="14"/>
       <c r="BC46" s="14"/>
@@ -3492,7 +3487,7 @@
       <c r="BG46" s="14"/>
       <c r="BH46" s="15"/>
       <c r="BI46" s="13" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="BJ46" s="14"/>
       <c r="BK46" s="14"/>
@@ -3502,50 +3497,50 @@
       <c r="BO46" s="14"/>
       <c r="BP46" s="14"/>
       <c r="BQ46" s="15"/>
-      <c r="BR46" s="24"/>
+      <c r="BR46" s="31"/>
     </row>
     <row r="47" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B47" s="24"/>
-      <c r="E47" s="16" t="s">
-        <v>230</v>
-      </c>
-      <c r="F47" s="16"/>
-      <c r="G47" s="16"/>
-      <c r="H47" s="16"/>
-      <c r="I47" s="16"/>
-      <c r="J47" s="16"/>
-      <c r="K47" s="16"/>
-      <c r="L47" s="16"/>
-      <c r="M47" s="16"/>
-      <c r="N47" s="16"/>
-      <c r="O47" s="16"/>
-      <c r="P47" s="16"/>
-      <c r="Q47" s="16"/>
-      <c r="R47" s="16"/>
-      <c r="T47" s="16" t="s">
-        <v>225</v>
-      </c>
-      <c r="U47" s="16"/>
-      <c r="V47" s="16"/>
-      <c r="W47" s="16"/>
-      <c r="X47" s="16"/>
-      <c r="Y47" s="16"/>
-      <c r="Z47" s="16"/>
-      <c r="AA47" s="16"/>
-      <c r="AB47" s="16"/>
-      <c r="AC47" s="16"/>
-      <c r="AD47" s="16"/>
-      <c r="AE47" s="16"/>
-      <c r="AF47" s="16"/>
-      <c r="AG47" s="16"/>
+      <c r="B47" s="31"/>
+      <c r="E47" s="30" t="s">
+        <v>229</v>
+      </c>
+      <c r="F47" s="30"/>
+      <c r="G47" s="30"/>
+      <c r="H47" s="30"/>
+      <c r="I47" s="30"/>
+      <c r="J47" s="30"/>
+      <c r="K47" s="30"/>
+      <c r="L47" s="30"/>
+      <c r="M47" s="30"/>
+      <c r="N47" s="30"/>
+      <c r="O47" s="30"/>
+      <c r="P47" s="30"/>
+      <c r="Q47" s="30"/>
+      <c r="R47" s="30"/>
+      <c r="T47" s="30" t="s">
+        <v>224</v>
+      </c>
+      <c r="U47" s="30"/>
+      <c r="V47" s="30"/>
+      <c r="W47" s="30"/>
+      <c r="X47" s="30"/>
+      <c r="Y47" s="30"/>
+      <c r="Z47" s="30"/>
+      <c r="AA47" s="30"/>
+      <c r="AB47" s="30"/>
+      <c r="AC47" s="30"/>
+      <c r="AD47" s="30"/>
+      <c r="AE47" s="30"/>
+      <c r="AF47" s="30"/>
+      <c r="AG47" s="30"/>
       <c r="AW47" s="13" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="AX47" s="14"/>
       <c r="AY47" s="14"/>
       <c r="AZ47" s="15"/>
       <c r="BA47" s="13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="BB47" s="14"/>
       <c r="BC47" s="14"/>
@@ -3555,7 +3550,7 @@
       <c r="BG47" s="14"/>
       <c r="BH47" s="15"/>
       <c r="BI47" s="13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="BJ47" s="14"/>
       <c r="BK47" s="14"/>
@@ -3565,342 +3560,342 @@
       <c r="BO47" s="14"/>
       <c r="BP47" s="14"/>
       <c r="BQ47" s="15"/>
-      <c r="BR47" s="24"/>
+      <c r="BR47" s="31"/>
     </row>
     <row r="48" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B48" s="24"/>
-      <c r="E48" s="16"/>
-      <c r="F48" s="16"/>
-      <c r="G48" s="16"/>
-      <c r="H48" s="16"/>
-      <c r="I48" s="16"/>
-      <c r="J48" s="16"/>
-      <c r="K48" s="16"/>
-      <c r="L48" s="16"/>
-      <c r="M48" s="16"/>
-      <c r="N48" s="16"/>
-      <c r="O48" s="16"/>
-      <c r="P48" s="16"/>
-      <c r="Q48" s="16"/>
-      <c r="R48" s="16"/>
-      <c r="T48" s="16"/>
-      <c r="U48" s="16"/>
-      <c r="V48" s="16"/>
-      <c r="W48" s="16"/>
-      <c r="X48" s="16"/>
-      <c r="Y48" s="16"/>
-      <c r="Z48" s="16"/>
-      <c r="AA48" s="16"/>
-      <c r="AB48" s="16"/>
-      <c r="AC48" s="16"/>
-      <c r="AD48" s="16"/>
-      <c r="AE48" s="16"/>
-      <c r="AF48" s="16"/>
-      <c r="AG48" s="16"/>
-      <c r="AW48" s="17" t="s">
+      <c r="B48" s="31"/>
+      <c r="E48" s="30"/>
+      <c r="F48" s="30"/>
+      <c r="G48" s="30"/>
+      <c r="H48" s="30"/>
+      <c r="I48" s="30"/>
+      <c r="J48" s="30"/>
+      <c r="K48" s="30"/>
+      <c r="L48" s="30"/>
+      <c r="M48" s="30"/>
+      <c r="N48" s="30"/>
+      <c r="O48" s="30"/>
+      <c r="P48" s="30"/>
+      <c r="Q48" s="30"/>
+      <c r="R48" s="30"/>
+      <c r="T48" s="30"/>
+      <c r="U48" s="30"/>
+      <c r="V48" s="30"/>
+      <c r="W48" s="30"/>
+      <c r="X48" s="30"/>
+      <c r="Y48" s="30"/>
+      <c r="Z48" s="30"/>
+      <c r="AA48" s="30"/>
+      <c r="AB48" s="30"/>
+      <c r="AC48" s="30"/>
+      <c r="AD48" s="30"/>
+      <c r="AE48" s="30"/>
+      <c r="AF48" s="30"/>
+      <c r="AG48" s="30"/>
+      <c r="AW48" s="16" t="s">
+        <v>210</v>
+      </c>
+      <c r="AX48" s="17"/>
+      <c r="AY48" s="17"/>
+      <c r="AZ48" s="17"/>
+      <c r="BA48" s="17"/>
+      <c r="BB48" s="17"/>
+      <c r="BC48" s="17"/>
+      <c r="BD48" s="18"/>
+      <c r="BE48" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="AX48" s="18"/>
-      <c r="AY48" s="18"/>
-      <c r="AZ48" s="18"/>
-      <c r="BA48" s="18"/>
-      <c r="BB48" s="18"/>
-      <c r="BC48" s="18"/>
-      <c r="BD48" s="19"/>
-      <c r="BE48" s="17" t="s">
+      <c r="BF48" s="17"/>
+      <c r="BG48" s="17"/>
+      <c r="BH48" s="17"/>
+      <c r="BI48" s="17"/>
+      <c r="BJ48" s="17"/>
+      <c r="BK48" s="17"/>
+      <c r="BL48" s="17"/>
+      <c r="BM48" s="17"/>
+      <c r="BN48" s="17"/>
+      <c r="BO48" s="17"/>
+      <c r="BP48" s="17"/>
+      <c r="BQ48" s="18"/>
+      <c r="BR48" s="31"/>
+    </row>
+    <row r="49" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B49" s="31"/>
+      <c r="E49" s="30"/>
+      <c r="F49" s="30"/>
+      <c r="G49" s="30"/>
+      <c r="H49" s="30"/>
+      <c r="I49" s="30"/>
+      <c r="J49" s="30"/>
+      <c r="K49" s="30"/>
+      <c r="L49" s="30"/>
+      <c r="M49" s="30"/>
+      <c r="N49" s="30"/>
+      <c r="O49" s="30"/>
+      <c r="P49" s="30"/>
+      <c r="Q49" s="30"/>
+      <c r="R49" s="30"/>
+      <c r="T49" s="30"/>
+      <c r="U49" s="30"/>
+      <c r="V49" s="30"/>
+      <c r="W49" s="30"/>
+      <c r="X49" s="30"/>
+      <c r="Y49" s="30"/>
+      <c r="Z49" s="30"/>
+      <c r="AA49" s="30"/>
+      <c r="AB49" s="30"/>
+      <c r="AC49" s="30"/>
+      <c r="AD49" s="30"/>
+      <c r="AE49" s="30"/>
+      <c r="AF49" s="30"/>
+      <c r="AG49" s="30"/>
+      <c r="AW49" s="22"/>
+      <c r="AX49" s="23"/>
+      <c r="AY49" s="23"/>
+      <c r="AZ49" s="23"/>
+      <c r="BA49" s="23"/>
+      <c r="BB49" s="23"/>
+      <c r="BC49" s="23"/>
+      <c r="BD49" s="24"/>
+      <c r="BE49" s="19"/>
+      <c r="BF49" s="20"/>
+      <c r="BG49" s="20"/>
+      <c r="BH49" s="20"/>
+      <c r="BI49" s="20"/>
+      <c r="BJ49" s="20"/>
+      <c r="BK49" s="20"/>
+      <c r="BL49" s="20"/>
+      <c r="BM49" s="20"/>
+      <c r="BN49" s="20"/>
+      <c r="BO49" s="20"/>
+      <c r="BP49" s="20"/>
+      <c r="BQ49" s="21"/>
+      <c r="BR49" s="31"/>
+    </row>
+    <row r="50" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B50" s="31"/>
+      <c r="E50" s="30"/>
+      <c r="F50" s="30"/>
+      <c r="G50" s="30"/>
+      <c r="H50" s="30"/>
+      <c r="I50" s="30"/>
+      <c r="J50" s="30"/>
+      <c r="K50" s="30"/>
+      <c r="L50" s="30"/>
+      <c r="M50" s="30"/>
+      <c r="N50" s="30"/>
+      <c r="O50" s="30"/>
+      <c r="P50" s="30"/>
+      <c r="Q50" s="30"/>
+      <c r="R50" s="30"/>
+      <c r="T50" s="30"/>
+      <c r="U50" s="30"/>
+      <c r="V50" s="30"/>
+      <c r="W50" s="30"/>
+      <c r="X50" s="30"/>
+      <c r="Y50" s="30"/>
+      <c r="Z50" s="30"/>
+      <c r="AA50" s="30"/>
+      <c r="AB50" s="30"/>
+      <c r="AC50" s="30"/>
+      <c r="AD50" s="30"/>
+      <c r="AE50" s="30"/>
+      <c r="AF50" s="30"/>
+      <c r="AG50" s="30"/>
+      <c r="AW50" s="22"/>
+      <c r="AX50" s="23"/>
+      <c r="AY50" s="23"/>
+      <c r="AZ50" s="23"/>
+      <c r="BA50" s="23"/>
+      <c r="BB50" s="23"/>
+      <c r="BC50" s="23"/>
+      <c r="BD50" s="24"/>
+      <c r="BE50" s="16" t="s">
         <v>212</v>
       </c>
-      <c r="BF48" s="18"/>
-      <c r="BG48" s="18"/>
-      <c r="BH48" s="18"/>
-      <c r="BI48" s="18"/>
-      <c r="BJ48" s="18"/>
-      <c r="BK48" s="18"/>
-      <c r="BL48" s="18"/>
-      <c r="BM48" s="18"/>
-      <c r="BN48" s="18"/>
-      <c r="BO48" s="18"/>
-      <c r="BP48" s="18"/>
-      <c r="BQ48" s="19"/>
-      <c r="BR48" s="24"/>
-    </row>
-    <row r="49" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B49" s="24"/>
-      <c r="E49" s="16"/>
-      <c r="F49" s="16"/>
-      <c r="G49" s="16"/>
-      <c r="H49" s="16"/>
-      <c r="I49" s="16"/>
-      <c r="J49" s="16"/>
-      <c r="K49" s="16"/>
-      <c r="L49" s="16"/>
-      <c r="M49" s="16"/>
-      <c r="N49" s="16"/>
-      <c r="O49" s="16"/>
-      <c r="P49" s="16"/>
-      <c r="Q49" s="16"/>
-      <c r="R49" s="16"/>
-      <c r="T49" s="16"/>
-      <c r="U49" s="16"/>
-      <c r="V49" s="16"/>
-      <c r="W49" s="16"/>
-      <c r="X49" s="16"/>
-      <c r="Y49" s="16"/>
-      <c r="Z49" s="16"/>
-      <c r="AA49" s="16"/>
-      <c r="AB49" s="16"/>
-      <c r="AC49" s="16"/>
-      <c r="AD49" s="16"/>
-      <c r="AE49" s="16"/>
-      <c r="AF49" s="16"/>
-      <c r="AG49" s="16"/>
-      <c r="AW49" s="26"/>
-      <c r="AX49" s="27"/>
-      <c r="AY49" s="27"/>
-      <c r="AZ49" s="27"/>
-      <c r="BA49" s="27"/>
-      <c r="BB49" s="27"/>
-      <c r="BC49" s="27"/>
-      <c r="BD49" s="28"/>
-      <c r="BE49" s="20"/>
-      <c r="BF49" s="21"/>
-      <c r="BG49" s="21"/>
-      <c r="BH49" s="21"/>
-      <c r="BI49" s="21"/>
-      <c r="BJ49" s="21"/>
-      <c r="BK49" s="21"/>
-      <c r="BL49" s="21"/>
-      <c r="BM49" s="21"/>
-      <c r="BN49" s="21"/>
-      <c r="BO49" s="21"/>
-      <c r="BP49" s="21"/>
-      <c r="BQ49" s="22"/>
-      <c r="BR49" s="24"/>
-    </row>
-    <row r="50" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B50" s="24"/>
-      <c r="E50" s="16"/>
-      <c r="F50" s="16"/>
-      <c r="G50" s="16"/>
-      <c r="H50" s="16"/>
-      <c r="I50" s="16"/>
-      <c r="J50" s="16"/>
-      <c r="K50" s="16"/>
-      <c r="L50" s="16"/>
-      <c r="M50" s="16"/>
-      <c r="N50" s="16"/>
-      <c r="O50" s="16"/>
-      <c r="P50" s="16"/>
-      <c r="Q50" s="16"/>
-      <c r="R50" s="16"/>
-      <c r="T50" s="16"/>
-      <c r="U50" s="16"/>
-      <c r="V50" s="16"/>
-      <c r="W50" s="16"/>
-      <c r="X50" s="16"/>
-      <c r="Y50" s="16"/>
-      <c r="Z50" s="16"/>
-      <c r="AA50" s="16"/>
-      <c r="AB50" s="16"/>
-      <c r="AC50" s="16"/>
-      <c r="AD50" s="16"/>
-      <c r="AE50" s="16"/>
-      <c r="AF50" s="16"/>
-      <c r="AG50" s="16"/>
-      <c r="AW50" s="26"/>
-      <c r="AX50" s="27"/>
-      <c r="AY50" s="27"/>
-      <c r="AZ50" s="27"/>
-      <c r="BA50" s="27"/>
-      <c r="BB50" s="27"/>
-      <c r="BC50" s="27"/>
-      <c r="BD50" s="28"/>
-      <c r="BE50" s="17" t="s">
+      <c r="BF50" s="17"/>
+      <c r="BG50" s="17"/>
+      <c r="BH50" s="17"/>
+      <c r="BI50" s="17"/>
+      <c r="BJ50" s="17"/>
+      <c r="BK50" s="17"/>
+      <c r="BL50" s="17"/>
+      <c r="BM50" s="17"/>
+      <c r="BN50" s="17"/>
+      <c r="BO50" s="17"/>
+      <c r="BP50" s="17"/>
+      <c r="BQ50" s="18"/>
+      <c r="BR50" s="31"/>
+    </row>
+    <row r="51" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B51" s="31"/>
+      <c r="E51" s="30"/>
+      <c r="F51" s="30"/>
+      <c r="G51" s="30"/>
+      <c r="H51" s="30"/>
+      <c r="I51" s="30"/>
+      <c r="J51" s="30"/>
+      <c r="K51" s="30"/>
+      <c r="L51" s="30"/>
+      <c r="M51" s="30"/>
+      <c r="N51" s="30"/>
+      <c r="O51" s="30"/>
+      <c r="P51" s="30"/>
+      <c r="Q51" s="30"/>
+      <c r="R51" s="30"/>
+      <c r="T51" s="30"/>
+      <c r="U51" s="30"/>
+      <c r="V51" s="30"/>
+      <c r="W51" s="30"/>
+      <c r="X51" s="30"/>
+      <c r="Y51" s="30"/>
+      <c r="Z51" s="30"/>
+      <c r="AA51" s="30"/>
+      <c r="AB51" s="30"/>
+      <c r="AC51" s="30"/>
+      <c r="AD51" s="30"/>
+      <c r="AE51" s="30"/>
+      <c r="AF51" s="30"/>
+      <c r="AG51" s="30"/>
+      <c r="AW51" s="19"/>
+      <c r="AX51" s="20"/>
+      <c r="AY51" s="20"/>
+      <c r="AZ51" s="20"/>
+      <c r="BA51" s="20"/>
+      <c r="BB51" s="20"/>
+      <c r="BC51" s="20"/>
+      <c r="BD51" s="21"/>
+      <c r="BE51" s="19"/>
+      <c r="BF51" s="20"/>
+      <c r="BG51" s="20"/>
+      <c r="BH51" s="20"/>
+      <c r="BI51" s="20"/>
+      <c r="BJ51" s="20"/>
+      <c r="BK51" s="20"/>
+      <c r="BL51" s="20"/>
+      <c r="BM51" s="20"/>
+      <c r="BN51" s="20"/>
+      <c r="BO51" s="20"/>
+      <c r="BP51" s="20"/>
+      <c r="BQ51" s="21"/>
+      <c r="BR51" s="31"/>
+    </row>
+    <row r="52" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B52" s="31"/>
+      <c r="AW52" s="16" t="s">
         <v>213</v>
       </c>
-      <c r="BF50" s="18"/>
-      <c r="BG50" s="18"/>
-      <c r="BH50" s="18"/>
-      <c r="BI50" s="18"/>
-      <c r="BJ50" s="18"/>
-      <c r="BK50" s="18"/>
-      <c r="BL50" s="18"/>
-      <c r="BM50" s="18"/>
-      <c r="BN50" s="18"/>
-      <c r="BO50" s="18"/>
-      <c r="BP50" s="18"/>
-      <c r="BQ50" s="19"/>
-      <c r="BR50" s="24"/>
-    </row>
-    <row r="51" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B51" s="24"/>
-      <c r="E51" s="16"/>
-      <c r="F51" s="16"/>
-      <c r="G51" s="16"/>
-      <c r="H51" s="16"/>
-      <c r="I51" s="16"/>
-      <c r="J51" s="16"/>
-      <c r="K51" s="16"/>
-      <c r="L51" s="16"/>
-      <c r="M51" s="16"/>
-      <c r="N51" s="16"/>
-      <c r="O51" s="16"/>
-      <c r="P51" s="16"/>
-      <c r="Q51" s="16"/>
-      <c r="R51" s="16"/>
-      <c r="T51" s="16"/>
-      <c r="U51" s="16"/>
-      <c r="V51" s="16"/>
-      <c r="W51" s="16"/>
-      <c r="X51" s="16"/>
-      <c r="Y51" s="16"/>
-      <c r="Z51" s="16"/>
-      <c r="AA51" s="16"/>
-      <c r="AB51" s="16"/>
-      <c r="AC51" s="16"/>
-      <c r="AD51" s="16"/>
-      <c r="AE51" s="16"/>
-      <c r="AF51" s="16"/>
-      <c r="AG51" s="16"/>
-      <c r="AW51" s="20"/>
-      <c r="AX51" s="21"/>
-      <c r="AY51" s="21"/>
-      <c r="AZ51" s="21"/>
-      <c r="BA51" s="21"/>
-      <c r="BB51" s="21"/>
-      <c r="BC51" s="21"/>
-      <c r="BD51" s="22"/>
-      <c r="BE51" s="20"/>
-      <c r="BF51" s="21"/>
-      <c r="BG51" s="21"/>
-      <c r="BH51" s="21"/>
-      <c r="BI51" s="21"/>
-      <c r="BJ51" s="21"/>
-      <c r="BK51" s="21"/>
-      <c r="BL51" s="21"/>
-      <c r="BM51" s="21"/>
-      <c r="BN51" s="21"/>
-      <c r="BO51" s="21"/>
-      <c r="BP51" s="21"/>
-      <c r="BQ51" s="22"/>
-      <c r="BR51" s="24"/>
-    </row>
-    <row r="52" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B52" s="24"/>
-      <c r="AW52" s="17" t="s">
+      <c r="AX52" s="17"/>
+      <c r="AY52" s="17"/>
+      <c r="AZ52" s="17"/>
+      <c r="BA52" s="17"/>
+      <c r="BB52" s="17"/>
+      <c r="BC52" s="17"/>
+      <c r="BD52" s="18"/>
+      <c r="BE52" s="16" t="s">
         <v>214</v>
       </c>
-      <c r="AX52" s="18"/>
-      <c r="AY52" s="18"/>
-      <c r="AZ52" s="18"/>
-      <c r="BA52" s="18"/>
-      <c r="BB52" s="18"/>
-      <c r="BC52" s="18"/>
-      <c r="BD52" s="19"/>
-      <c r="BE52" s="17" t="s">
-        <v>215</v>
-      </c>
-      <c r="BF52" s="18"/>
-      <c r="BG52" s="18"/>
-      <c r="BH52" s="18"/>
-      <c r="BI52" s="18"/>
-      <c r="BJ52" s="18"/>
-      <c r="BK52" s="18"/>
-      <c r="BL52" s="18"/>
-      <c r="BM52" s="18"/>
-      <c r="BN52" s="18"/>
-      <c r="BO52" s="18"/>
-      <c r="BP52" s="18"/>
-      <c r="BQ52" s="19"/>
-      <c r="BR52" s="24"/>
+      <c r="BF52" s="17"/>
+      <c r="BG52" s="17"/>
+      <c r="BH52" s="17"/>
+      <c r="BI52" s="17"/>
+      <c r="BJ52" s="17"/>
+      <c r="BK52" s="17"/>
+      <c r="BL52" s="17"/>
+      <c r="BM52" s="17"/>
+      <c r="BN52" s="17"/>
+      <c r="BO52" s="17"/>
+      <c r="BP52" s="17"/>
+      <c r="BQ52" s="18"/>
+      <c r="BR52" s="31"/>
     </row>
     <row r="53" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B53" s="24"/>
-      <c r="AW53" s="26" t="s">
-        <v>231</v>
-      </c>
-      <c r="AX53" s="27"/>
-      <c r="AY53" s="27"/>
-      <c r="AZ53" s="27"/>
-      <c r="BA53" s="27"/>
-      <c r="BB53" s="27"/>
-      <c r="BC53" s="27"/>
-      <c r="BD53" s="28"/>
-      <c r="BE53" s="26"/>
-      <c r="BF53" s="27"/>
-      <c r="BG53" s="27"/>
-      <c r="BH53" s="27"/>
-      <c r="BI53" s="27"/>
-      <c r="BJ53" s="27"/>
-      <c r="BK53" s="27"/>
-      <c r="BL53" s="27"/>
-      <c r="BM53" s="27"/>
-      <c r="BN53" s="27"/>
-      <c r="BO53" s="27"/>
-      <c r="BP53" s="27"/>
-      <c r="BQ53" s="28"/>
-      <c r="BR53" s="24"/>
+      <c r="B53" s="31"/>
+      <c r="AW53" s="22" t="s">
+        <v>230</v>
+      </c>
+      <c r="AX53" s="23"/>
+      <c r="AY53" s="23"/>
+      <c r="AZ53" s="23"/>
+      <c r="BA53" s="23"/>
+      <c r="BB53" s="23"/>
+      <c r="BC53" s="23"/>
+      <c r="BD53" s="24"/>
+      <c r="BE53" s="22"/>
+      <c r="BF53" s="23"/>
+      <c r="BG53" s="23"/>
+      <c r="BH53" s="23"/>
+      <c r="BI53" s="23"/>
+      <c r="BJ53" s="23"/>
+      <c r="BK53" s="23"/>
+      <c r="BL53" s="23"/>
+      <c r="BM53" s="23"/>
+      <c r="BN53" s="23"/>
+      <c r="BO53" s="23"/>
+      <c r="BP53" s="23"/>
+      <c r="BQ53" s="24"/>
+      <c r="BR53" s="31"/>
     </row>
     <row r="54" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B54" s="24"/>
-      <c r="AW54" s="26"/>
-      <c r="AX54" s="27"/>
-      <c r="AY54" s="27"/>
-      <c r="AZ54" s="27"/>
-      <c r="BA54" s="27"/>
-      <c r="BB54" s="27"/>
-      <c r="BC54" s="27"/>
-      <c r="BD54" s="28"/>
-      <c r="BE54" s="26"/>
-      <c r="BF54" s="27"/>
-      <c r="BG54" s="27"/>
-      <c r="BH54" s="27"/>
-      <c r="BI54" s="27"/>
-      <c r="BJ54" s="27"/>
-      <c r="BK54" s="27"/>
-      <c r="BL54" s="27"/>
-      <c r="BM54" s="27"/>
-      <c r="BN54" s="27"/>
-      <c r="BO54" s="27"/>
-      <c r="BP54" s="27"/>
-      <c r="BQ54" s="28"/>
-      <c r="BR54" s="24"/>
+      <c r="B54" s="31"/>
+      <c r="AW54" s="22"/>
+      <c r="AX54" s="23"/>
+      <c r="AY54" s="23"/>
+      <c r="AZ54" s="23"/>
+      <c r="BA54" s="23"/>
+      <c r="BB54" s="23"/>
+      <c r="BC54" s="23"/>
+      <c r="BD54" s="24"/>
+      <c r="BE54" s="22"/>
+      <c r="BF54" s="23"/>
+      <c r="BG54" s="23"/>
+      <c r="BH54" s="23"/>
+      <c r="BI54" s="23"/>
+      <c r="BJ54" s="23"/>
+      <c r="BK54" s="23"/>
+      <c r="BL54" s="23"/>
+      <c r="BM54" s="23"/>
+      <c r="BN54" s="23"/>
+      <c r="BO54" s="23"/>
+      <c r="BP54" s="23"/>
+      <c r="BQ54" s="24"/>
+      <c r="BR54" s="31"/>
     </row>
     <row r="55" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B55" s="24"/>
-      <c r="AW55" s="20"/>
-      <c r="AX55" s="21"/>
-      <c r="AY55" s="21"/>
-      <c r="AZ55" s="21"/>
-      <c r="BA55" s="21"/>
-      <c r="BB55" s="21"/>
-      <c r="BC55" s="21"/>
-      <c r="BD55" s="22"/>
-      <c r="BE55" s="20"/>
-      <c r="BF55" s="21"/>
-      <c r="BG55" s="21"/>
-      <c r="BH55" s="21"/>
-      <c r="BI55" s="21"/>
-      <c r="BJ55" s="21"/>
-      <c r="BK55" s="21"/>
-      <c r="BL55" s="21"/>
-      <c r="BM55" s="21"/>
-      <c r="BN55" s="21"/>
-      <c r="BO55" s="21"/>
-      <c r="BP55" s="21"/>
-      <c r="BQ55" s="22"/>
-      <c r="BR55" s="24"/>
+      <c r="B55" s="31"/>
+      <c r="AW55" s="19"/>
+      <c r="AX55" s="20"/>
+      <c r="AY55" s="20"/>
+      <c r="AZ55" s="20"/>
+      <c r="BA55" s="20"/>
+      <c r="BB55" s="20"/>
+      <c r="BC55" s="20"/>
+      <c r="BD55" s="21"/>
+      <c r="BE55" s="19"/>
+      <c r="BF55" s="20"/>
+      <c r="BG55" s="20"/>
+      <c r="BH55" s="20"/>
+      <c r="BI55" s="20"/>
+      <c r="BJ55" s="20"/>
+      <c r="BK55" s="20"/>
+      <c r="BL55" s="20"/>
+      <c r="BM55" s="20"/>
+      <c r="BN55" s="20"/>
+      <c r="BO55" s="20"/>
+      <c r="BP55" s="20"/>
+      <c r="BQ55" s="21"/>
+      <c r="BR55" s="31"/>
     </row>
     <row r="56" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B56" s="25"/>
+      <c r="B56" s="26"/>
       <c r="K56" s="3"/>
       <c r="AI56" s="3"/>
       <c r="AW56" s="13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="AX56" s="14"/>
       <c r="AY56" s="14" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="AZ56" s="14"/>
       <c r="BA56" s="14"/>
@@ -3920,7 +3915,7 @@
       <c r="BO56" s="14"/>
       <c r="BP56" s="14"/>
       <c r="BQ56" s="15"/>
-      <c r="BR56" s="25"/>
+      <c r="BR56" s="26"/>
     </row>
     <row r="57" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4">
       <c r="C57" s="13">
@@ -4006,6 +4001,171 @@
     <row r="58" spans="2:70" ht="13.95" customHeight="1" x14ac:dyDescent="0.4"/>
   </sheetData>
   <mergeCells count="189">
+    <mergeCell ref="C2:L2"/>
+    <mergeCell ref="BO41:BQ41"/>
+    <mergeCell ref="BF16:BK16"/>
+    <mergeCell ref="AY10:BB10"/>
+    <mergeCell ref="AW11:AX11"/>
+    <mergeCell ref="AY11:BB11"/>
+    <mergeCell ref="BC11:BE11"/>
+    <mergeCell ref="BF11:BK11"/>
+    <mergeCell ref="BM11:BO11"/>
+    <mergeCell ref="AY17:BB17"/>
+    <mergeCell ref="AW24:AX24"/>
+    <mergeCell ref="BF24:BK24"/>
+    <mergeCell ref="BC20:BE20"/>
+    <mergeCell ref="AY15:BB15"/>
+    <mergeCell ref="AW22:AX22"/>
+    <mergeCell ref="BA41:BH41"/>
+    <mergeCell ref="AW26:AX26"/>
+    <mergeCell ref="E7:R11"/>
+    <mergeCell ref="E17:R20"/>
+    <mergeCell ref="E26:R29"/>
+    <mergeCell ref="E35:R39"/>
+    <mergeCell ref="BM7:BO7"/>
+    <mergeCell ref="BM15:BO15"/>
+    <mergeCell ref="BC25:BE25"/>
+    <mergeCell ref="C57:L57"/>
+    <mergeCell ref="M57:X57"/>
+    <mergeCell ref="Y57:AI57"/>
+    <mergeCell ref="AJ57:AT57"/>
+    <mergeCell ref="AW56:AX56"/>
+    <mergeCell ref="BM25:BO25"/>
+    <mergeCell ref="BL39:BN39"/>
+    <mergeCell ref="E47:R51"/>
+    <mergeCell ref="BA42:BH42"/>
+    <mergeCell ref="AX40:AZ40"/>
+    <mergeCell ref="BA43:BH44"/>
+    <mergeCell ref="BL40:BN40"/>
+    <mergeCell ref="BE50:BQ51"/>
+    <mergeCell ref="AY26:BB26"/>
+    <mergeCell ref="BR17:BR29"/>
+    <mergeCell ref="BM9:BO9"/>
+    <mergeCell ref="AY16:BB16"/>
+    <mergeCell ref="BO39:BQ39"/>
+    <mergeCell ref="BM19:BO19"/>
+    <mergeCell ref="BF14:BK14"/>
+    <mergeCell ref="BF23:BK23"/>
+    <mergeCell ref="BM12:BO12"/>
+    <mergeCell ref="BR3:BR16"/>
+    <mergeCell ref="BF25:BK25"/>
+    <mergeCell ref="BF22:BK22"/>
+    <mergeCell ref="BF12:BK12"/>
+    <mergeCell ref="BM20:BO20"/>
+    <mergeCell ref="BF7:BK7"/>
+    <mergeCell ref="AY21:BB21"/>
+    <mergeCell ref="BM18:BO18"/>
+    <mergeCell ref="BC13:BE13"/>
+    <mergeCell ref="BM13:BO13"/>
+    <mergeCell ref="AY19:BB19"/>
+    <mergeCell ref="AY13:BB13"/>
+    <mergeCell ref="AY22:BB22"/>
+    <mergeCell ref="B30:B43"/>
+    <mergeCell ref="AW47:AZ47"/>
+    <mergeCell ref="BF10:BK10"/>
+    <mergeCell ref="AW10:AX10"/>
+    <mergeCell ref="BF17:BK17"/>
+    <mergeCell ref="AW23:AX23"/>
+    <mergeCell ref="BC18:BE18"/>
+    <mergeCell ref="AW48:BD48"/>
+    <mergeCell ref="BI41:BK41"/>
+    <mergeCell ref="B3:B16"/>
+    <mergeCell ref="BI47:BQ47"/>
+    <mergeCell ref="AW21:AX21"/>
+    <mergeCell ref="BC19:BE19"/>
+    <mergeCell ref="AX41:AZ41"/>
+    <mergeCell ref="BM24:BO24"/>
+    <mergeCell ref="BI39:BK39"/>
+    <mergeCell ref="BC21:BE21"/>
+    <mergeCell ref="AX43:AZ44"/>
+    <mergeCell ref="AY20:BB20"/>
+    <mergeCell ref="AW16:AX16"/>
+    <mergeCell ref="BF5:BK6"/>
+    <mergeCell ref="BC17:BE17"/>
+    <mergeCell ref="AY24:BB24"/>
+    <mergeCell ref="BC5:BE6"/>
+    <mergeCell ref="BR30:BR43"/>
+    <mergeCell ref="BM8:BO8"/>
+    <mergeCell ref="AX39:AZ39"/>
+    <mergeCell ref="BM16:BO16"/>
+    <mergeCell ref="BA46:BH46"/>
+    <mergeCell ref="BA39:BH39"/>
+    <mergeCell ref="BM10:BO10"/>
+    <mergeCell ref="AW31:AX36"/>
+    <mergeCell ref="BE48:BQ49"/>
+    <mergeCell ref="BL42:BN42"/>
+    <mergeCell ref="AY23:BB23"/>
+    <mergeCell ref="AX45:AZ45"/>
+    <mergeCell ref="BI42:BK42"/>
+    <mergeCell ref="BF21:BK21"/>
+    <mergeCell ref="BO45:BQ45"/>
+    <mergeCell ref="BR44:BR56"/>
+    <mergeCell ref="AY9:BB9"/>
+    <mergeCell ref="AW25:AX25"/>
+    <mergeCell ref="AW15:AX15"/>
+    <mergeCell ref="BC9:BE9"/>
+    <mergeCell ref="AY18:BB18"/>
+    <mergeCell ref="AW49:BD51"/>
+    <mergeCell ref="BI45:BK45"/>
+    <mergeCell ref="BC16:BE16"/>
+    <mergeCell ref="T7:AG11"/>
+    <mergeCell ref="B17:B29"/>
+    <mergeCell ref="AW7:AX7"/>
+    <mergeCell ref="B44:B56"/>
+    <mergeCell ref="BL41:BN41"/>
+    <mergeCell ref="T47:AG51"/>
+    <mergeCell ref="C3:D5"/>
+    <mergeCell ref="BM5:BO6"/>
+    <mergeCell ref="AW5:AX6"/>
+    <mergeCell ref="AT3:AV8"/>
+    <mergeCell ref="T17:AG20"/>
+    <mergeCell ref="T26:AG29"/>
+    <mergeCell ref="T35:AG39"/>
+    <mergeCell ref="BE52:BQ55"/>
+    <mergeCell ref="AX42:AZ42"/>
+    <mergeCell ref="AW43:AW44"/>
+    <mergeCell ref="AY5:BB6"/>
+    <mergeCell ref="BF20:BK20"/>
+    <mergeCell ref="AW20:AX20"/>
+    <mergeCell ref="AW52:BD52"/>
+    <mergeCell ref="BO42:BQ42"/>
+    <mergeCell ref="BP5:BP6"/>
+    <mergeCell ref="BO40:BQ40"/>
+    <mergeCell ref="BQ5:BQ6"/>
+    <mergeCell ref="AW14:AX14"/>
+    <mergeCell ref="AY7:BB7"/>
+    <mergeCell ref="BC10:BE10"/>
+    <mergeCell ref="BM17:BO17"/>
+    <mergeCell ref="BC23:BE23"/>
+    <mergeCell ref="BF18:BK18"/>
+    <mergeCell ref="AW12:AX12"/>
+    <mergeCell ref="BM14:BO14"/>
+    <mergeCell ref="BC12:BE12"/>
+    <mergeCell ref="BF19:BK19"/>
+    <mergeCell ref="BM21:BO21"/>
+    <mergeCell ref="BF13:BK13"/>
+    <mergeCell ref="AW13:AX13"/>
+    <mergeCell ref="AW8:AX8"/>
+    <mergeCell ref="BF8:BK8"/>
+    <mergeCell ref="BI46:BQ46"/>
+    <mergeCell ref="BM23:BO23"/>
+    <mergeCell ref="BF15:BK15"/>
+    <mergeCell ref="BL5:BL6"/>
+    <mergeCell ref="AY14:BB14"/>
+    <mergeCell ref="AY25:BB25"/>
+    <mergeCell ref="AY31:BQ36"/>
+    <mergeCell ref="AY12:BB12"/>
+    <mergeCell ref="BC14:BE14"/>
+    <mergeCell ref="BM22:BO22"/>
+    <mergeCell ref="BL43:BN44"/>
+    <mergeCell ref="BC24:BE24"/>
+    <mergeCell ref="BA45:BH45"/>
+    <mergeCell ref="BL45:BN45"/>
+    <mergeCell ref="BI40:BK40"/>
+    <mergeCell ref="AW46:AZ46"/>
+    <mergeCell ref="BC26:BE26"/>
+    <mergeCell ref="BF26:BK26"/>
+    <mergeCell ref="BM26:BO26"/>
     <mergeCell ref="M2:X2"/>
     <mergeCell ref="AU2:BF2"/>
     <mergeCell ref="AW18:AX18"/>
@@ -4030,171 +4190,6 @@
     <mergeCell ref="AW19:AX19"/>
     <mergeCell ref="AW53:BD55"/>
     <mergeCell ref="AW3:BQ4"/>
-    <mergeCell ref="BI46:BQ46"/>
-    <mergeCell ref="BM23:BO23"/>
-    <mergeCell ref="BF15:BK15"/>
-    <mergeCell ref="BL5:BL6"/>
-    <mergeCell ref="AY14:BB14"/>
-    <mergeCell ref="AY25:BB25"/>
-    <mergeCell ref="AY31:BQ36"/>
-    <mergeCell ref="AY12:BB12"/>
-    <mergeCell ref="BC14:BE14"/>
-    <mergeCell ref="BM22:BO22"/>
-    <mergeCell ref="AW14:AX14"/>
-    <mergeCell ref="AY7:BB7"/>
-    <mergeCell ref="BC10:BE10"/>
-    <mergeCell ref="BM17:BO17"/>
-    <mergeCell ref="BC23:BE23"/>
-    <mergeCell ref="BF18:BK18"/>
-    <mergeCell ref="AW12:AX12"/>
-    <mergeCell ref="BM14:BO14"/>
-    <mergeCell ref="BC12:BE12"/>
-    <mergeCell ref="BL43:BN44"/>
-    <mergeCell ref="BF19:BK19"/>
-    <mergeCell ref="BC24:BE24"/>
-    <mergeCell ref="T7:AG11"/>
-    <mergeCell ref="B17:B29"/>
-    <mergeCell ref="AW7:AX7"/>
-    <mergeCell ref="B44:B56"/>
-    <mergeCell ref="BL41:BN41"/>
-    <mergeCell ref="T47:AG51"/>
-    <mergeCell ref="C3:D5"/>
-    <mergeCell ref="BM5:BO6"/>
-    <mergeCell ref="AW5:AX6"/>
-    <mergeCell ref="AT3:AV8"/>
-    <mergeCell ref="T17:AG20"/>
-    <mergeCell ref="T26:AG29"/>
-    <mergeCell ref="T35:AG39"/>
-    <mergeCell ref="BE52:BQ55"/>
-    <mergeCell ref="AX42:AZ42"/>
-    <mergeCell ref="AW43:AW44"/>
-    <mergeCell ref="AY5:BB6"/>
-    <mergeCell ref="BF20:BK20"/>
-    <mergeCell ref="AW20:AX20"/>
-    <mergeCell ref="AW52:BD52"/>
-    <mergeCell ref="BO42:BQ42"/>
-    <mergeCell ref="BP5:BP6"/>
-    <mergeCell ref="BO40:BQ40"/>
-    <mergeCell ref="BQ5:BQ6"/>
-    <mergeCell ref="BM21:BO21"/>
-    <mergeCell ref="BF13:BK13"/>
-    <mergeCell ref="AW13:AX13"/>
-    <mergeCell ref="BA45:BH45"/>
-    <mergeCell ref="AW8:AX8"/>
-    <mergeCell ref="BL45:BN45"/>
-    <mergeCell ref="BR30:BR43"/>
-    <mergeCell ref="BM8:BO8"/>
-    <mergeCell ref="AX39:AZ39"/>
-    <mergeCell ref="BM16:BO16"/>
-    <mergeCell ref="BA46:BH46"/>
-    <mergeCell ref="BA39:BH39"/>
-    <mergeCell ref="BM10:BO10"/>
-    <mergeCell ref="AW31:AX36"/>
-    <mergeCell ref="BE48:BQ49"/>
-    <mergeCell ref="BL42:BN42"/>
-    <mergeCell ref="AY23:BB23"/>
-    <mergeCell ref="AX45:AZ45"/>
-    <mergeCell ref="BI42:BK42"/>
-    <mergeCell ref="BF21:BK21"/>
-    <mergeCell ref="BO45:BQ45"/>
-    <mergeCell ref="BR44:BR56"/>
-    <mergeCell ref="AY9:BB9"/>
-    <mergeCell ref="AW25:AX25"/>
-    <mergeCell ref="AW15:AX15"/>
-    <mergeCell ref="BC9:BE9"/>
-    <mergeCell ref="AY18:BB18"/>
-    <mergeCell ref="AW49:BD51"/>
-    <mergeCell ref="BI45:BK45"/>
-    <mergeCell ref="BC16:BE16"/>
-    <mergeCell ref="B30:B43"/>
-    <mergeCell ref="AW47:AZ47"/>
-    <mergeCell ref="BF10:BK10"/>
-    <mergeCell ref="AW10:AX10"/>
-    <mergeCell ref="BF17:BK17"/>
-    <mergeCell ref="AW23:AX23"/>
-    <mergeCell ref="BC18:BE18"/>
-    <mergeCell ref="AW48:BD48"/>
-    <mergeCell ref="BI41:BK41"/>
-    <mergeCell ref="B3:B16"/>
-    <mergeCell ref="BI47:BQ47"/>
-    <mergeCell ref="AW21:AX21"/>
-    <mergeCell ref="BC19:BE19"/>
-    <mergeCell ref="AX41:AZ41"/>
-    <mergeCell ref="BM24:BO24"/>
-    <mergeCell ref="BI39:BK39"/>
-    <mergeCell ref="BC21:BE21"/>
-    <mergeCell ref="AX43:AZ44"/>
-    <mergeCell ref="AY20:BB20"/>
-    <mergeCell ref="AW16:AX16"/>
-    <mergeCell ref="BF5:BK6"/>
-    <mergeCell ref="BC17:BE17"/>
-    <mergeCell ref="AY24:BB24"/>
-    <mergeCell ref="BC5:BE6"/>
-    <mergeCell ref="BF8:BK8"/>
-    <mergeCell ref="BI40:BK40"/>
-    <mergeCell ref="AW46:AZ46"/>
-    <mergeCell ref="BC26:BE26"/>
-    <mergeCell ref="BF26:BK26"/>
-    <mergeCell ref="BM26:BO26"/>
-    <mergeCell ref="BE50:BQ51"/>
-    <mergeCell ref="AY26:BB26"/>
-    <mergeCell ref="BR17:BR29"/>
-    <mergeCell ref="BM9:BO9"/>
-    <mergeCell ref="AY16:BB16"/>
-    <mergeCell ref="BO39:BQ39"/>
-    <mergeCell ref="BM19:BO19"/>
-    <mergeCell ref="BF14:BK14"/>
-    <mergeCell ref="BF23:BK23"/>
-    <mergeCell ref="BM12:BO12"/>
-    <mergeCell ref="BR3:BR16"/>
-    <mergeCell ref="BF25:BK25"/>
-    <mergeCell ref="BF22:BK22"/>
-    <mergeCell ref="BF12:BK12"/>
-    <mergeCell ref="BM20:BO20"/>
-    <mergeCell ref="BF7:BK7"/>
-    <mergeCell ref="AY21:BB21"/>
-    <mergeCell ref="BM18:BO18"/>
-    <mergeCell ref="BC13:BE13"/>
-    <mergeCell ref="BM13:BO13"/>
-    <mergeCell ref="C57:L57"/>
-    <mergeCell ref="M57:X57"/>
-    <mergeCell ref="Y57:AI57"/>
-    <mergeCell ref="AJ57:AT57"/>
-    <mergeCell ref="AW56:AX56"/>
-    <mergeCell ref="BM25:BO25"/>
-    <mergeCell ref="BL39:BN39"/>
-    <mergeCell ref="E47:R51"/>
-    <mergeCell ref="BA42:BH42"/>
-    <mergeCell ref="AY19:BB19"/>
-    <mergeCell ref="AY13:BB13"/>
-    <mergeCell ref="AX40:AZ40"/>
-    <mergeCell ref="AY22:BB22"/>
-    <mergeCell ref="BA43:BH44"/>
-    <mergeCell ref="BL40:BN40"/>
-    <mergeCell ref="C2:L2"/>
-    <mergeCell ref="BO41:BQ41"/>
-    <mergeCell ref="BF16:BK16"/>
-    <mergeCell ref="AY10:BB10"/>
-    <mergeCell ref="AW11:AX11"/>
-    <mergeCell ref="AY11:BB11"/>
-    <mergeCell ref="BC11:BE11"/>
-    <mergeCell ref="BF11:BK11"/>
-    <mergeCell ref="BM11:BO11"/>
-    <mergeCell ref="AY17:BB17"/>
-    <mergeCell ref="AW24:AX24"/>
-    <mergeCell ref="BF24:BK24"/>
-    <mergeCell ref="BC20:BE20"/>
-    <mergeCell ref="AY15:BB15"/>
-    <mergeCell ref="AW22:AX22"/>
-    <mergeCell ref="BA41:BH41"/>
-    <mergeCell ref="AW26:AX26"/>
-    <mergeCell ref="E7:R11"/>
-    <mergeCell ref="E17:R20"/>
-    <mergeCell ref="E26:R29"/>
-    <mergeCell ref="E35:R39"/>
-    <mergeCell ref="BM7:BO7"/>
-    <mergeCell ref="BM15:BO15"/>
-    <mergeCell ref="BC25:BE25"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>